<commit_message>
Added visualizer.js and corresponding scripts in package.json
</commit_message>
<xml_diff>
--- a/data/stocks.xlsx
+++ b/data/stocks.xlsx
@@ -12,13 +12,14 @@
     <sheet sheetId="6" name="Dow_Jones" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="Nasdaq" state="visible" r:id="rId10"/>
     <sheet sheetId="8" name="SP_100" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="Composite_Formula" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="141">
   <si>
     <t>Ticker</t>
   </si>
@@ -194,157 +195,253 @@
     <t>Daily_Composite_Score_delta</t>
   </si>
   <si>
+    <t>WSR</t>
+  </si>
+  <si>
+    <t>MD</t>
+  </si>
+  <si>
+    <t>CSCO</t>
+  </si>
+  <si>
+    <t>DELL</t>
+  </si>
+  <si>
+    <t>ETN</t>
+  </si>
+  <si>
     <t>_date_</t>
   </si>
   <si>
+    <t>2026-04-21</t>
+  </si>
+  <si>
+    <t>Criteria</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Last Run</t>
+  </si>
+  <si>
+    <t>Index</t>
+  </si>
+  <si>
+    <t>Russell 2000</t>
+  </si>
+  <si>
+    <t>Cap</t>
+  </si>
+  <si>
+    <t>Small ($300M–$2B)</t>
+  </si>
+  <si>
+    <t>Price min</t>
+  </si>
+  <si>
+    <t>&gt; $7</t>
+  </si>
+  <si>
+    <t>YTD perf min</t>
+  </si>
+  <si>
+    <t>&gt; +10%</t>
+  </si>
+  <si>
+    <t>P/E max</t>
+  </si>
+  <si>
+    <t>&lt; 28</t>
+  </si>
+  <si>
+    <t>EPS Q/Q</t>
+  </si>
+  <si>
+    <t>Positive</t>
+  </si>
+  <si>
+    <t>Sectors</t>
+  </si>
+  <si>
+    <t>Technology, Consumer Staples, Materials, Real Estate, Financials, Industrials, Consumer Discretionary</t>
+  </si>
+  <si>
+    <t>Beta range</t>
+  </si>
+  <si>
+    <t>0.7 – 1.2</t>
+  </si>
+  <si>
+    <t>RSI min</t>
+  </si>
+  <si>
+    <t>68</t>
+  </si>
+  <si>
+    <t>Alpha</t>
+  </si>
+  <si>
+    <t>&gt; 0</t>
+  </si>
+  <si>
+    <t>Ranked by</t>
+  </si>
+  <si>
+    <t>Alpha (highest first)</t>
+  </si>
+  <si>
+    <t>Top N</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>Results</t>
+  </si>
+  <si>
+    <t>2 of 2 qualified</t>
+  </si>
+  <si>
+    <t>Dow Jones 30</t>
+  </si>
+  <si>
+    <t>&gt; $10</t>
+  </si>
+  <si>
+    <t>&gt; +5%</t>
+  </si>
+  <si>
+    <t>&lt; 35</t>
+  </si>
+  <si>
+    <t>All sectors</t>
+  </si>
+  <si>
+    <t>64</t>
+  </si>
+  <si>
+    <t>1 of 1 qualified</t>
+  </si>
+  <si>
+    <t>Nasdaq 100</t>
+  </si>
+  <si>
+    <t>&lt; 50</t>
+  </si>
+  <si>
+    <t>0.7 – 1.3</t>
+  </si>
+  <si>
+    <t>S&amp;P 500 (large-cap subset)</t>
+  </si>
+  <si>
+    <t>Large (approx. S&amp;P 100)</t>
+  </si>
+  <si>
+    <t>&gt; +8%</t>
+  </si>
+  <si>
+    <t>&lt; 40</t>
+  </si>
+  <si>
+    <t>Component</t>
+  </si>
+  <si>
+    <t>Weight</t>
+  </si>
+  <si>
+    <t>Signal Type</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>30%</t>
+  </si>
+  <si>
+    <t>Earnings quality vs peers</t>
+  </si>
+  <si>
+    <t>Finviz</t>
+  </si>
+  <si>
+    <t>P(EPS_Fwd_Growth)</t>
+  </si>
+  <si>
+    <t>Earnings acceleration</t>
+  </si>
+  <si>
+    <t>P(MA_Slope_50)</t>
+  </si>
+  <si>
+    <t>20%</t>
+  </si>
+  <si>
+    <t>Medium-term price trend</t>
+  </si>
+  <si>
+    <t>Yahoo Finance prices</t>
+  </si>
+  <si>
+    <t>P(RSI_14)</t>
+  </si>
+  <si>
+    <t>10%</t>
+  </si>
+  <si>
+    <t>Short-term momentum strength</t>
+  </si>
+  <si>
+    <t>P(SMA200_Dist)</t>
+  </si>
+  <si>
+    <t>Long-term trend confirmation</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>Criteria</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>WSR</t>
-  </si>
-  <si>
-    <t>Last Run</t>
-  </si>
-  <si>
-    <t>2026-04-21</t>
-  </si>
-  <si>
-    <t>MD</t>
-  </si>
-  <si>
-    <t>Index</t>
-  </si>
-  <si>
-    <t>Russell 2000</t>
-  </si>
-  <si>
-    <t>Cap</t>
-  </si>
-  <si>
-    <t>Small ($300M–$2B)</t>
-  </si>
-  <si>
-    <t>Price min</t>
-  </si>
-  <si>
-    <t>&gt; $7</t>
-  </si>
-  <si>
-    <t>YTD perf min</t>
-  </si>
-  <si>
-    <t>&gt; +10%</t>
-  </si>
-  <si>
-    <t>P/E max</t>
-  </si>
-  <si>
-    <t>&lt; 28</t>
-  </si>
-  <si>
-    <t>EPS Q/Q</t>
-  </si>
-  <si>
-    <t>Positive</t>
-  </si>
-  <si>
-    <t>Sectors</t>
-  </si>
-  <si>
-    <t>Technology, Consumer Staples, Materials, Real Estate, Financials, Industrials, Consumer Discretionary</t>
-  </si>
-  <si>
-    <t>Beta range</t>
-  </si>
-  <si>
-    <t>0.7 – 1.2</t>
-  </si>
-  <si>
-    <t>RSI min</t>
-  </si>
-  <si>
-    <t>68</t>
-  </si>
-  <si>
-    <t>Alpha</t>
-  </si>
-  <si>
-    <t>&gt; 0</t>
-  </si>
-  <si>
-    <t>Ranked by</t>
-  </si>
-  <si>
-    <t>Alpha (highest first)</t>
-  </si>
-  <si>
-    <t>Top N</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>Results</t>
-  </si>
-  <si>
-    <t>2 of 2 qualified</t>
-  </si>
-  <si>
-    <t>CSCO</t>
-  </si>
-  <si>
-    <t>Dow Jones 30</t>
-  </si>
-  <si>
-    <t>&gt; $10</t>
-  </si>
-  <si>
-    <t>&gt; +5%</t>
-  </si>
-  <si>
-    <t>&lt; 35</t>
-  </si>
-  <si>
-    <t>All sectors</t>
-  </si>
-  <si>
-    <t>64</t>
-  </si>
-  <si>
-    <t>1 of 1 qualified</t>
-  </si>
-  <si>
-    <t>Nasdaq 100</t>
-  </si>
-  <si>
-    <t>&lt; 50</t>
-  </si>
-  <si>
-    <t>0.7 – 1.3</t>
-  </si>
-  <si>
-    <t>DELL</t>
-  </si>
-  <si>
-    <t>ETN</t>
-  </si>
-  <si>
-    <t>S&amp;P 500 (large-cap subset)</t>
-  </si>
-  <si>
-    <t>Large (approx. S&amp;P 100)</t>
-  </si>
-  <si>
-    <t>&gt; +8%</t>
-  </si>
-  <si>
-    <t>&lt; 40</t>
+    <t>Formula</t>
+  </si>
+  <si>
+    <t>Composite = 0.30 × P(EPS_Univ) + 0.30 × P(Fwd_Growth) + 0.20 × P(MA_Slope_50) + 0.10 × P(RSI_14) + 0.10 × P(SMA200_Dist)</t>
+  </si>
+  <si>
+    <t>Score Range</t>
+  </si>
+  <si>
+    <t>Signal</t>
+  </si>
+  <si>
+    <t>≥ 70</t>
+  </si>
+  <si>
+    <t>Strong Buy candidate</t>
+  </si>
+  <si>
+    <t>50 – 70</t>
+  </si>
+  <si>
+    <t>Hold / Monitor</t>
+  </si>
+  <si>
+    <t>30 – 50</t>
+  </si>
+  <si>
+    <t>Weak / Neutral</t>
+  </si>
+  <si>
+    <t>&lt; 30</t>
+  </si>
+  <si>
+    <t>Consider reducing position</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>All P(x) values are percentile ranks within the current universe (0-100). Score is relative, not absolute.</t>
   </si>
 </sst>
 </file>
@@ -360,12 +457,32 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -380,8 +497,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -968,7 +1089,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:O49"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
@@ -1017,6 +1138,2166 @@
       <c r="O1" t="s">
         <v>57</v>
       </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1">
+        <v>6.69</v>
+      </c>
+      <c r="C2" s="1">
+        <v>85.41666666666666</v>
+      </c>
+      <c r="D2" s="1">
+        <v>-0.8191330343796712</v>
+      </c>
+      <c r="E2" s="1">
+        <v>-0.01</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0.11940253782009777</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0.18</v>
+      </c>
+      <c r="H2" s="1">
+        <v>39.81</v>
+      </c>
+      <c r="I2" s="1">
+        <v>17.35</v>
+      </c>
+      <c r="J2" s="1">
+        <v>0.0023737785663199627</v>
+      </c>
+      <c r="K2" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L2" s="1">
+        <v>364</v>
+      </c>
+      <c r="M2" s="1">
+        <v>0.09774252789480942</v>
+      </c>
+      <c r="N2" s="1">
+        <v>44.375</v>
+      </c>
+      <c r="O2" s="1"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2">
+        <v>2.64</v>
+      </c>
+      <c r="C3" s="2">
+        <v>66.66666666666666</v>
+      </c>
+      <c r="D3" s="2">
+        <v>23.181818181818183</v>
+      </c>
+      <c r="E3" s="2">
+        <v>2.75</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0.15463133361194895</v>
+      </c>
+      <c r="G3" s="2">
+        <v>2.1</v>
+      </c>
+      <c r="H3" s="2">
+        <v>79.25</v>
+      </c>
+      <c r="I3" s="2">
+        <v>39.15</v>
+      </c>
+      <c r="J3" s="2">
+        <v>0.027035824145518757</v>
+      </c>
+      <c r="K3" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L3" s="2">
+        <v>375</v>
+      </c>
+      <c r="M3" s="2">
+        <v>0.18368744448733576</v>
+      </c>
+      <c r="N3" s="2">
+        <v>77.29166666666666</v>
+      </c>
+      <c r="O3" s="2"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3">
+        <v>-3.95</v>
+      </c>
+      <c r="C4" s="3">
+        <v>8.333333333333332</v>
+      </c>
+      <c r="D4" s="3">
+        <v>9.721518987341772</v>
+      </c>
+      <c r="E4" s="3">
+        <v>4.7</v>
+      </c>
+      <c r="F4" s="3">
+        <v>-0.2997874815980858</v>
+      </c>
+      <c r="G4" s="3">
+        <v>1.18</v>
+      </c>
+      <c r="H4" s="3">
+        <v>50.03</v>
+      </c>
+      <c r="I4" s="3">
+        <v>-27.2</v>
+      </c>
+      <c r="J4" s="3">
+        <v>-0.01432968093560943</v>
+      </c>
+      <c r="K4" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L4" s="3">
+        <v>50</v>
+      </c>
+      <c r="M4" s="3">
+        <v>-0.29503284527302254</v>
+      </c>
+      <c r="N4" s="3">
+        <v>24.583333333333332</v>
+      </c>
+      <c r="O4" s="3"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4">
+        <v>1.08</v>
+      </c>
+      <c r="C5" s="4">
+        <v>56.25</v>
+      </c>
+      <c r="D5" s="4">
+        <v>27.981481481481477</v>
+      </c>
+      <c r="E5" s="4">
+        <v>0.58</v>
+      </c>
+      <c r="F5" s="4">
+        <v>-0.1324852835010605</v>
+      </c>
+      <c r="G5" s="4">
+        <v>1.85</v>
+      </c>
+      <c r="H5" s="4">
+        <v>55.13</v>
+      </c>
+      <c r="I5" s="4">
+        <v>-2.42</v>
+      </c>
+      <c r="J5" s="4">
+        <v>-0.004872619589082648</v>
+      </c>
+      <c r="K5" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L5" s="4">
+        <v>312</v>
+      </c>
+      <c r="M5" s="4">
+        <v>-0.1100328341882616</v>
+      </c>
+      <c r="N5" s="4">
+        <v>51.66666666666667</v>
+      </c>
+      <c r="O5" s="4"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1">
+        <v>3.09</v>
+      </c>
+      <c r="C6" s="1">
+        <v>70.83333333333334</v>
+      </c>
+      <c r="D6" s="1">
+        <v>1.5663430420711975</v>
+      </c>
+      <c r="E6" s="1">
+        <v>-2.3</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0.015574698750199387</v>
+      </c>
+      <c r="G6" s="1">
+        <v>1.6</v>
+      </c>
+      <c r="H6" s="1">
+        <v>41.72</v>
+      </c>
+      <c r="I6" s="1">
+        <v>-11.59</v>
+      </c>
+      <c r="J6" s="1">
+        <v>0.020971830186022736</v>
+      </c>
+      <c r="K6" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L6" s="1">
+        <v>139</v>
+      </c>
+      <c r="M6" s="1">
+        <v>0.03142348650041038</v>
+      </c>
+      <c r="N6" s="1">
+        <v>49.375</v>
+      </c>
+      <c r="O6" s="1"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4">
+        <v>4.9</v>
+      </c>
+      <c r="C7" s="4">
+        <v>79.16666666666666</v>
+      </c>
+      <c r="D7" s="4">
+        <v>5.9</v>
+      </c>
+      <c r="E7" s="4">
+        <v>0.37</v>
+      </c>
+      <c r="F7" s="4">
+        <v>0.05216692912061721</v>
+      </c>
+      <c r="G7" s="4">
+        <v>2.29</v>
+      </c>
+      <c r="H7" s="4">
+        <v>68.67</v>
+      </c>
+      <c r="I7" s="4">
+        <v>10.03</v>
+      </c>
+      <c r="J7" s="4">
+        <v>0.011374279129554401</v>
+      </c>
+      <c r="K7" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L7" s="4">
+        <v>434</v>
+      </c>
+      <c r="M7" s="4">
+        <v>0.08624182278357084</v>
+      </c>
+      <c r="N7" s="4">
+        <v>61.875</v>
+      </c>
+      <c r="O7" s="4"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4">
+        <v>13.19</v>
+      </c>
+      <c r="C8" s="4">
+        <v>97.91666666666666</v>
+      </c>
+      <c r="D8" s="4">
+        <v>-0.044730856709628494</v>
+      </c>
+      <c r="E8" s="4">
+        <v>0.43</v>
+      </c>
+      <c r="F8" s="4">
+        <v>0.013480296772397392</v>
+      </c>
+      <c r="G8" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="H8" s="4">
+        <v>80.84</v>
+      </c>
+      <c r="I8" s="4">
+        <v>12.36</v>
+      </c>
+      <c r="J8" s="4">
+        <v>0.016806327810061392</v>
+      </c>
+      <c r="K8" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L8" s="4">
+        <v>69</v>
+      </c>
+      <c r="M8" s="4">
+        <v>0.0002729736472215638</v>
+      </c>
+      <c r="N8" s="4">
+        <v>62.708333333333336</v>
+      </c>
+      <c r="O8" s="4"/>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4">
+        <v>0.63</v>
+      </c>
+      <c r="C9" s="4">
+        <v>50</v>
+      </c>
+      <c r="D9" s="4">
+        <v>67.1111111111111</v>
+      </c>
+      <c r="E9" s="4">
+        <v>1.75</v>
+      </c>
+      <c r="F9" s="4">
+        <v>-0.18257434339651085</v>
+      </c>
+      <c r="G9" s="4">
+        <v>1.6</v>
+      </c>
+      <c r="H9" s="4">
+        <v>52.98</v>
+      </c>
+      <c r="I9" s="4">
+        <v>-10.4</v>
+      </c>
+      <c r="J9" s="4">
+        <v>0.0017804758732523362</v>
+      </c>
+      <c r="K9" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L9" s="4">
+        <v>189</v>
+      </c>
+      <c r="M9" s="4">
+        <v>-0.16672555564629987</v>
+      </c>
+      <c r="N9" s="4">
+        <v>52.29166666666667</v>
+      </c>
+      <c r="O9" s="4"/>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1">
+        <v>6.79</v>
+      </c>
+      <c r="C10" s="1">
+        <v>87.5</v>
+      </c>
+      <c r="D10" s="1">
+        <v>0.6435935198821797</v>
+      </c>
+      <c r="E10" s="1">
+        <v>0.88</v>
+      </c>
+      <c r="F10" s="1">
+        <v>-0.09935027283030967</v>
+      </c>
+      <c r="G10" s="1">
+        <v>1.45</v>
+      </c>
+      <c r="H10" s="1">
+        <v>62.08</v>
+      </c>
+      <c r="I10" s="1">
+        <v>-5.15</v>
+      </c>
+      <c r="J10" s="1">
+        <v>-0.0009973918374701378</v>
+      </c>
+      <c r="K10" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L10" s="1">
+        <v>56</v>
+      </c>
+      <c r="M10" s="1">
+        <v>-0.08746368201765142</v>
+      </c>
+      <c r="N10" s="1">
+        <v>46.875</v>
+      </c>
+      <c r="O10" s="1"/>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="C11" s="3">
+        <v>43.75</v>
+      </c>
+      <c r="D11" s="3">
+        <v>-1653.5</v>
+      </c>
+      <c r="E11" s="3">
+        <v>10.01</v>
+      </c>
+      <c r="F11" s="3">
+        <v>-0.2373041633607682</v>
+      </c>
+      <c r="G11" s="3">
+        <v>1.41</v>
+      </c>
+      <c r="H11" s="3">
+        <v>49.11</v>
+      </c>
+      <c r="I11" s="3">
+        <v>-0.49</v>
+      </c>
+      <c r="J11" s="3">
+        <v>-0.012954170042827666</v>
+      </c>
+      <c r="K11" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L11" s="3">
+        <v>28</v>
+      </c>
+      <c r="M11" s="3">
+        <v>-0.22647415839812401</v>
+      </c>
+      <c r="N11" s="3">
+        <v>22.916666666666668</v>
+      </c>
+      <c r="O11" s="3"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1">
+        <v>1.31</v>
+      </c>
+      <c r="C12" s="1">
+        <v>60.416666666666664</v>
+      </c>
+      <c r="D12" s="1">
+        <v>7.5114503816793885</v>
+      </c>
+      <c r="E12" s="1">
+        <v>0.13</v>
+      </c>
+      <c r="F12" s="1">
+        <v>-0.1266387692870606</v>
+      </c>
+      <c r="G12" s="1">
+        <v>0.63</v>
+      </c>
+      <c r="H12" s="1">
+        <v>55.45</v>
+      </c>
+      <c r="I12" s="1">
+        <v>-9.56</v>
+      </c>
+      <c r="J12" s="1">
+        <v>-0.01441421206345179</v>
+      </c>
+      <c r="K12" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L12" s="1">
+        <v>10</v>
+      </c>
+      <c r="M12" s="1">
+        <v>-0.13641218839969071</v>
+      </c>
+      <c r="N12" s="1">
+        <v>40.208333333333336</v>
+      </c>
+      <c r="O12" s="1"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2">
+        <v>-0.08</v>
+      </c>
+      <c r="C13" s="2">
+        <v>37.5</v>
+      </c>
+      <c r="D13" s="2">
+        <v>1166</v>
+      </c>
+      <c r="E13" s="2">
+        <v>6.17</v>
+      </c>
+      <c r="F13" s="2">
+        <v>0.31134277324890075</v>
+      </c>
+      <c r="G13" s="2">
+        <v>1.66</v>
+      </c>
+      <c r="H13" s="2">
+        <v>71.41</v>
+      </c>
+      <c r="I13" s="2">
+        <v>76.95</v>
+      </c>
+      <c r="J13" s="2">
+        <v>0.036955400678864</v>
+      </c>
+      <c r="K13" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L13" s="2">
+        <v>249</v>
+      </c>
+      <c r="M13" s="2">
+        <v>0.32877643977413284</v>
+      </c>
+      <c r="N13" s="2">
+        <v>75.625</v>
+      </c>
+      <c r="O13" s="2"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1">
+        <v>-3.83</v>
+      </c>
+      <c r="C14" s="1">
+        <v>10.416666666666668</v>
+      </c>
+      <c r="D14" s="1">
+        <v>12.668407310704959</v>
+      </c>
+      <c r="E14" s="1">
+        <v>2.52</v>
+      </c>
+      <c r="F14" s="1">
+        <v>0.1367064575621085</v>
+      </c>
+      <c r="G14" s="1">
+        <v>2.06</v>
+      </c>
+      <c r="H14" s="1">
+        <v>64.5</v>
+      </c>
+      <c r="I14" s="1">
+        <v>18.73</v>
+      </c>
+      <c r="J14" s="1">
+        <v>0.019616079754584414</v>
+      </c>
+      <c r="K14" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L14" s="1">
+        <v>27</v>
+      </c>
+      <c r="M14" s="1">
+        <v>0.16470598258748126</v>
+      </c>
+      <c r="N14" s="1">
+        <v>49.791666666666664</v>
+      </c>
+      <c r="O14" s="1"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1">
+        <v>-6.51</v>
+      </c>
+      <c r="C15" s="1">
+        <v>4.166666666666666</v>
+      </c>
+      <c r="D15" s="1">
+        <v>4.411674347158218</v>
+      </c>
+      <c r="E15" s="1">
+        <v>4.53</v>
+      </c>
+      <c r="F15" s="1">
+        <v>0.02551684943171327</v>
+      </c>
+      <c r="G15" s="1">
+        <v>1.84</v>
+      </c>
+      <c r="H15" s="1">
+        <v>63.5</v>
+      </c>
+      <c r="I15" s="1">
+        <v>1.17</v>
+      </c>
+      <c r="J15" s="1">
+        <v>0.014393856469644214</v>
+      </c>
+      <c r="K15" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L15" s="1">
+        <v>43</v>
+      </c>
+      <c r="M15" s="1">
+        <v>0.04770515228200867</v>
+      </c>
+      <c r="N15" s="1">
+        <v>36.25</v>
+      </c>
+      <c r="O15" s="1"/>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="4">
+        <v>-0.01</v>
+      </c>
+      <c r="C16" s="4">
+        <v>41.66666666666667</v>
+      </c>
+      <c r="D16" s="4">
+        <v>18685</v>
+      </c>
+      <c r="E16" s="4">
+        <v>11.11</v>
+      </c>
+      <c r="F16" s="4">
+        <v>-0.07710107317789963</v>
+      </c>
+      <c r="G16" s="4">
+        <v>1.23</v>
+      </c>
+      <c r="H16" s="4">
+        <v>66.28</v>
+      </c>
+      <c r="I16" s="4">
+        <v>22.53</v>
+      </c>
+      <c r="J16" s="4">
+        <v>-0.003388255450886434</v>
+      </c>
+      <c r="K16" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L16" s="4">
+        <v>32</v>
+      </c>
+      <c r="M16" s="4">
+        <v>-0.07102570454031876</v>
+      </c>
+      <c r="N16" s="4">
+        <v>63.125</v>
+      </c>
+      <c r="O16" s="4"/>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="1">
+        <v>8.81</v>
+      </c>
+      <c r="C17" s="1">
+        <v>93.75</v>
+      </c>
+      <c r="D17" s="1">
+        <v>-0.27922814982973904</v>
+      </c>
+      <c r="E17" s="1">
+        <v>4.52</v>
+      </c>
+      <c r="F17" s="1">
+        <v>0.11848178357699889</v>
+      </c>
+      <c r="G17" s="1">
+        <v>0.17</v>
+      </c>
+      <c r="H17" s="1">
+        <v>56.37</v>
+      </c>
+      <c r="I17" s="1">
+        <v>15.34</v>
+      </c>
+      <c r="J17" s="1">
+        <v>-0.002480406015349057</v>
+      </c>
+      <c r="K17" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L17" s="1">
+        <v>94</v>
+      </c>
+      <c r="M17" s="1">
+        <v>0.09655762718920702</v>
+      </c>
+      <c r="N17" s="1">
+        <v>49.166666666666664</v>
+      </c>
+      <c r="O17" s="1"/>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="4">
+        <v>27.92</v>
+      </c>
+      <c r="C18" s="4">
+        <v>100</v>
+      </c>
+      <c r="D18" s="4">
+        <v>-0.5508595988538683</v>
+      </c>
+      <c r="E18" s="4">
+        <v>-1.85</v>
+      </c>
+      <c r="F18" s="4">
+        <v>-0.06458700033216558</v>
+      </c>
+      <c r="G18" s="4">
+        <v>1.14</v>
+      </c>
+      <c r="H18" s="4">
+        <v>69.94</v>
+      </c>
+      <c r="I18" s="4">
+        <v>4.92</v>
+      </c>
+      <c r="J18" s="4">
+        <v>-0.0006200222082913154</v>
+      </c>
+      <c r="K18" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L18" s="4">
+        <v>4</v>
+      </c>
+      <c r="M18" s="4">
+        <v>-0.06088894985711635</v>
+      </c>
+      <c r="N18" s="4">
+        <v>53.54166666666667</v>
+      </c>
+      <c r="O18" s="4"/>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="1">
+        <v>1.29</v>
+      </c>
+      <c r="C19" s="1">
+        <v>58.333333333333336</v>
+      </c>
+      <c r="D19" s="1">
+        <v>15.426356589147288</v>
+      </c>
+      <c r="E19" s="1">
+        <v>3.37</v>
+      </c>
+      <c r="F19" s="1">
+        <v>-0.04129758439236603</v>
+      </c>
+      <c r="G19" s="1">
+        <v>1.31</v>
+      </c>
+      <c r="H19" s="1">
+        <v>46.23</v>
+      </c>
+      <c r="I19" s="1">
+        <v>-4.53</v>
+      </c>
+      <c r="J19" s="1">
+        <v>-0.027338011861329586</v>
+      </c>
+      <c r="K19" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L19" s="1">
+        <v>-7</v>
+      </c>
+      <c r="M19" s="1">
+        <v>-0.03310904405475701</v>
+      </c>
+      <c r="N19" s="1">
+        <v>43.958333333333336</v>
+      </c>
+      <c r="O19" s="1"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3">
+        <v>-18.39</v>
+      </c>
+      <c r="C20" s="3">
+        <v>2.083333333333333</v>
+      </c>
+      <c r="D20" s="3">
+        <v>-4.206090266449157</v>
+      </c>
+      <c r="E20" s="3">
+        <v>8.76</v>
+      </c>
+      <c r="F20" s="3">
+        <v>-0.061258483063819674</v>
+      </c>
+      <c r="G20" s="3">
+        <v>3.67</v>
+      </c>
+      <c r="H20" s="3">
+        <v>71</v>
+      </c>
+      <c r="I20" s="3">
+        <v>-29.81</v>
+      </c>
+      <c r="J20" s="3">
+        <v>0.023188818679715038</v>
+      </c>
+      <c r="K20" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L20" s="3">
+        <v>-44</v>
+      </c>
+      <c r="M20" s="3">
+        <v>0.009268622424619233</v>
+      </c>
+      <c r="N20" s="3">
+        <v>27.916666666666664</v>
+      </c>
+      <c r="O20" s="3"/>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3">
+        <v>-2.25</v>
+      </c>
+      <c r="C21" s="3">
+        <v>18.75</v>
+      </c>
+      <c r="D21" s="3">
+        <v>10.44</v>
+      </c>
+      <c r="E21" s="3">
+        <v>12.21</v>
+      </c>
+      <c r="F21" s="3">
+        <v>-0.43969939957864956</v>
+      </c>
+      <c r="G21" s="3">
+        <v>2.31</v>
+      </c>
+      <c r="H21" s="3">
+        <v>54.4</v>
+      </c>
+      <c r="I21" s="3">
+        <v>-55.05</v>
+      </c>
+      <c r="J21" s="3">
+        <v>-0.03547797069677966</v>
+      </c>
+      <c r="K21" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L21" s="3">
+        <v>17</v>
+      </c>
+      <c r="M21" s="3">
+        <v>-0.4050962129906889</v>
+      </c>
+      <c r="N21" s="3">
+        <v>25.625</v>
+      </c>
+      <c r="O21" s="3"/>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1">
+        <v>-2.38</v>
+      </c>
+      <c r="C22" s="1">
+        <v>16.666666666666664</v>
+      </c>
+      <c r="D22" s="1">
+        <v>1.4705882352941178</v>
+      </c>
+      <c r="E22" s="1">
+        <v>5.89</v>
+      </c>
+      <c r="F22" s="1">
+        <v>-0.17120120712554815</v>
+      </c>
+      <c r="G22" s="1">
+        <v>3.13</v>
+      </c>
+      <c r="H22" s="1">
+        <v>73.51</v>
+      </c>
+      <c r="I22" s="1">
+        <v>0.82</v>
+      </c>
+      <c r="J22" s="1">
+        <v>0.03109288839166161</v>
+      </c>
+      <c r="K22" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L22" s="1">
+        <v>43</v>
+      </c>
+      <c r="M22" s="1">
+        <v>-0.11493801061229914</v>
+      </c>
+      <c r="N22" s="1">
+        <v>46.04166666666667</v>
+      </c>
+      <c r="O22" s="1"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3">
+        <v>-1.13</v>
+      </c>
+      <c r="C23" s="3">
+        <v>20.833333333333336</v>
+      </c>
+      <c r="D23" s="3">
+        <v>5.7522123893805315</v>
+      </c>
+      <c r="E23" s="3">
+        <v>1.42</v>
+      </c>
+      <c r="F23" s="3">
+        <v>-0.4662787098315891</v>
+      </c>
+      <c r="G23" s="3">
+        <v>2.65</v>
+      </c>
+      <c r="H23" s="3">
+        <v>49.67</v>
+      </c>
+      <c r="I23" s="3">
+        <v>-33.89</v>
+      </c>
+      <c r="J23" s="3">
+        <v>-0.012401909198076783</v>
+      </c>
+      <c r="K23" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L23" s="3">
+        <v>37</v>
+      </c>
+      <c r="M23" s="3">
+        <v>-0.4226945435185089</v>
+      </c>
+      <c r="N23" s="3">
+        <v>24.16666666666667</v>
+      </c>
+      <c r="O23" s="3"/>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3">
+        <v>-0.99</v>
+      </c>
+      <c r="C24" s="3">
+        <v>22.916666666666664</v>
+      </c>
+      <c r="D24" s="3">
+        <v>3.04040404040404</v>
+      </c>
+      <c r="E24" s="3">
+        <v>3.54</v>
+      </c>
+      <c r="F24" s="3">
+        <v>-0.40154728528252626</v>
+      </c>
+      <c r="G24" s="3">
+        <v>3.24</v>
+      </c>
+      <c r="H24" s="3">
+        <v>53.77</v>
+      </c>
+      <c r="I24" s="3">
+        <v>-29.95</v>
+      </c>
+      <c r="J24" s="3">
+        <v>-0.01464141824677345</v>
+      </c>
+      <c r="K24" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L24" s="3">
+        <v>60</v>
+      </c>
+      <c r="M24" s="3">
+        <v>-0.34237847768173857</v>
+      </c>
+      <c r="N24" s="3">
+        <v>23.125000000000004</v>
+      </c>
+      <c r="O24" s="3"/>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25" s="4">
+        <v>0.38</v>
+      </c>
+      <c r="C25" s="4">
+        <v>45.83333333333333</v>
+      </c>
+      <c r="D25" s="4">
+        <v>89.71052631578947</v>
+      </c>
+      <c r="E25" s="4">
+        <v>2.21</v>
+      </c>
+      <c r="F25" s="4">
+        <v>-0.3170927581740075</v>
+      </c>
+      <c r="G25" s="4">
+        <v>2.32</v>
+      </c>
+      <c r="H25" s="4">
+        <v>63.79</v>
+      </c>
+      <c r="I25" s="4">
+        <v>-19.66</v>
+      </c>
+      <c r="J25" s="4">
+        <v>-0.009812260461178298</v>
+      </c>
+      <c r="K25" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L25" s="4">
+        <v>70</v>
+      </c>
+      <c r="M25" s="4">
+        <v>-0.2822254251235433</v>
+      </c>
+      <c r="N25" s="4">
+        <v>51.87499999999999</v>
+      </c>
+      <c r="O25" s="4"/>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" s="4">
+        <v>1.9</v>
+      </c>
+      <c r="C26" s="4">
+        <v>62.5</v>
+      </c>
+      <c r="D26" s="4">
+        <v>2990.236842105264</v>
+      </c>
+      <c r="E26" s="4">
+        <v>2.07</v>
+      </c>
+      <c r="F26" s="4">
+        <v>-0.1547367590902501</v>
+      </c>
+      <c r="G26" s="4">
+        <v>1.2</v>
+      </c>
+      <c r="H26" s="4">
+        <v>55.52</v>
+      </c>
+      <c r="I26" s="4">
+        <v>0.85</v>
+      </c>
+      <c r="J26" s="4">
+        <v>-0.006328987029654367</v>
+      </c>
+      <c r="K26" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L26" s="4">
+        <v>116</v>
+      </c>
+      <c r="M26" s="4">
+        <v>-0.14945382984017974</v>
+      </c>
+      <c r="N26" s="4">
+        <v>61.875</v>
+      </c>
+      <c r="O26" s="4"/>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2">
+        <v>5.13</v>
+      </c>
+      <c r="C27" s="2">
+        <v>81.25</v>
+      </c>
+      <c r="D27" s="2">
+        <v>10.491228070175438</v>
+      </c>
+      <c r="E27" s="2">
+        <v>0.39</v>
+      </c>
+      <c r="F27" s="2">
+        <v>0.16421433169186833</v>
+      </c>
+      <c r="G27" s="2">
+        <v>1.39</v>
+      </c>
+      <c r="H27" s="2">
+        <v>74.94</v>
+      </c>
+      <c r="I27" s="2">
+        <v>20.62</v>
+      </c>
+      <c r="J27" s="2">
+        <v>0.024434924341505217</v>
+      </c>
+      <c r="K27" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L27" s="2">
+        <v>412</v>
+      </c>
+      <c r="M27" s="2">
+        <v>0.17451604372950547</v>
+      </c>
+      <c r="N27" s="2">
+        <v>75.62500000000001</v>
+      </c>
+      <c r="O27" s="2"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28" s="1">
+        <v>-3.07</v>
+      </c>
+      <c r="C28" s="1">
+        <v>12.5</v>
+      </c>
+      <c r="D28" s="1">
+        <v>8.671009771986972</v>
+      </c>
+      <c r="E28" s="1">
+        <v>2.29</v>
+      </c>
+      <c r="F28" s="1">
+        <v>0.00989392080333086</v>
+      </c>
+      <c r="G28" s="1">
+        <v>1.69</v>
+      </c>
+      <c r="H28" s="1">
+        <v>63.26</v>
+      </c>
+      <c r="I28" s="1">
+        <v>13.66</v>
+      </c>
+      <c r="J28" s="1">
+        <v>0.0168781609811</v>
+      </c>
+      <c r="K28" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L28" s="1">
+        <v>44</v>
+      </c>
+      <c r="M28" s="1">
+        <v>0.0281200267160735</v>
+      </c>
+      <c r="N28" s="1">
+        <v>43.74999999999999</v>
+      </c>
+      <c r="O28" s="1"/>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29" s="1">
+        <v>7.4</v>
+      </c>
+      <c r="C29" s="1">
+        <v>89.58333333333334</v>
+      </c>
+      <c r="D29" s="1">
+        <v>1.2283783783783782</v>
+      </c>
+      <c r="E29" s="1">
+        <v>-0.84</v>
+      </c>
+      <c r="F29" s="1">
+        <v>-0.09024617250147376</v>
+      </c>
+      <c r="G29" s="1">
+        <v>1.1</v>
+      </c>
+      <c r="H29" s="1">
+        <v>42.46</v>
+      </c>
+      <c r="I29" s="1">
+        <v>-14.49</v>
+      </c>
+      <c r="J29" s="1">
+        <v>0.010836343223542119</v>
+      </c>
+      <c r="K29" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L29" s="1">
+        <v>149</v>
+      </c>
+      <c r="M29" s="1">
+        <v>-0.08760470787643859</v>
+      </c>
+      <c r="N29" s="1">
+        <v>49.583333333333336</v>
+      </c>
+      <c r="O29" s="1"/>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30" s="4">
+        <v>5.41</v>
+      </c>
+      <c r="C30" s="4">
+        <v>83.33333333333334</v>
+      </c>
+      <c r="D30" s="4">
+        <v>0.6598890942698706</v>
+      </c>
+      <c r="E30" s="4">
+        <v>-0.09</v>
+      </c>
+      <c r="F30" s="4">
+        <v>-0.11560724672853408</v>
+      </c>
+      <c r="G30" s="4">
+        <v>1.43</v>
+      </c>
+      <c r="H30" s="4">
+        <v>70.08</v>
+      </c>
+      <c r="I30" s="4">
+        <v>-14.71</v>
+      </c>
+      <c r="J30" s="4">
+        <v>0.016935392611379864</v>
+      </c>
+      <c r="K30" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L30" s="4">
+        <v>-63</v>
+      </c>
+      <c r="M30" s="4">
+        <v>-0.10424894884088287</v>
+      </c>
+      <c r="N30" s="4">
+        <v>54.375</v>
+      </c>
+      <c r="O30" s="4"/>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A31" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31" s="4">
+        <v>-0.74</v>
+      </c>
+      <c r="C31" s="4">
+        <v>27.083333333333332</v>
+      </c>
+      <c r="D31" s="4">
+        <v>36.608108108108105</v>
+      </c>
+      <c r="E31" s="4">
+        <v>1.22</v>
+      </c>
+      <c r="F31" s="4">
+        <v>-0.012600547693719072</v>
+      </c>
+      <c r="G31" s="4">
+        <v>1.05</v>
+      </c>
+      <c r="H31" s="4">
+        <v>63.53</v>
+      </c>
+      <c r="I31" s="4">
+        <v>-1.24</v>
+      </c>
+      <c r="J31" s="4">
+        <v>0.004536771046019471</v>
+      </c>
+      <c r="K31" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L31" s="4">
+        <v>93</v>
+      </c>
+      <c r="M31" s="4">
+        <v>-0.011279815381201486</v>
+      </c>
+      <c r="N31" s="4">
+        <v>50.833333333333336</v>
+      </c>
+      <c r="O31" s="4"/>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A32" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32" s="4">
+        <v>-0.18</v>
+      </c>
+      <c r="C32" s="4">
+        <v>35.41666666666667</v>
+      </c>
+      <c r="D32" s="4">
+        <v>105.33333333333334</v>
+      </c>
+      <c r="E32" s="4">
+        <v>-4.72</v>
+      </c>
+      <c r="F32" s="4">
+        <v>0.1381086728940456</v>
+      </c>
+      <c r="G32" s="4">
+        <v>1.36</v>
+      </c>
+      <c r="H32" s="4">
+        <v>75</v>
+      </c>
+      <c r="I32" s="4">
+        <v>13.25</v>
+      </c>
+      <c r="J32" s="4">
+        <v>0.02243554574533957</v>
+      </c>
+      <c r="K32" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L32" s="4">
+        <v>-11</v>
+      </c>
+      <c r="M32" s="4">
+        <v>0.14761794554417218</v>
+      </c>
+      <c r="N32" s="4">
+        <v>68.54166666666666</v>
+      </c>
+      <c r="O32" s="4"/>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33" s="1">
+        <v>-4.08</v>
+      </c>
+      <c r="C33" s="1">
+        <v>6.25</v>
+      </c>
+      <c r="D33" s="1">
+        <v>14.372549019607844</v>
+      </c>
+      <c r="E33" s="1">
+        <v>13.14</v>
+      </c>
+      <c r="F33" s="1">
+        <v>0.0749569552980534</v>
+      </c>
+      <c r="G33" s="1">
+        <v>0</v>
+      </c>
+      <c r="H33" s="1">
+        <v>62.34</v>
+      </c>
+      <c r="I33" s="1">
+        <v>-7.11</v>
+      </c>
+      <c r="J33" s="1">
+        <v>0.04408771991281714</v>
+      </c>
+      <c r="K33" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L33" s="1">
+        <v>20</v>
+      </c>
+      <c r="M33" s="1">
+        <v>0.04854230904770174</v>
+      </c>
+      <c r="N33" s="1">
+        <v>48.333333333333336</v>
+      </c>
+      <c r="O33" s="1"/>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34" s="1">
+        <v>-0.48</v>
+      </c>
+      <c r="C34" s="1">
+        <v>29.166666666666668</v>
+      </c>
+      <c r="D34" s="1">
+        <v>86.47916666666667</v>
+      </c>
+      <c r="E34" s="1">
+        <v>-1.38</v>
+      </c>
+      <c r="F34" s="1">
+        <v>-0.27528167947146365</v>
+      </c>
+      <c r="G34" s="1">
+        <v>0.91</v>
+      </c>
+      <c r="H34" s="1">
+        <v>56.83</v>
+      </c>
+      <c r="I34" s="1">
+        <v>-32.31</v>
+      </c>
+      <c r="J34" s="1">
+        <v>-0.010654340748782016</v>
+      </c>
+      <c r="K34" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L34" s="1">
+        <v>3</v>
+      </c>
+      <c r="M34" s="1">
+        <v>-0.27765899763399526</v>
+      </c>
+      <c r="N34" s="1">
+        <v>42.708333333333336</v>
+      </c>
+      <c r="O34" s="1"/>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35" s="1">
+        <v>3.52</v>
+      </c>
+      <c r="C35" s="1">
+        <v>75</v>
+      </c>
+      <c r="D35" s="1">
+        <v>1.1988636363636365</v>
+      </c>
+      <c r="E35" s="1">
+        <v>0.4</v>
+      </c>
+      <c r="F35" s="1">
+        <v>0.04837859130682097</v>
+      </c>
+      <c r="G35" s="1">
+        <v>0.38</v>
+      </c>
+      <c r="H35" s="1">
+        <v>43.38</v>
+      </c>
+      <c r="I35" s="1">
+        <v>4.13</v>
+      </c>
+      <c r="J35" s="1">
+        <v>0.007072343136519611</v>
+      </c>
+      <c r="K35" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L35" s="1">
+        <v>28</v>
+      </c>
+      <c r="M35" s="1">
+        <v>0.03200151063160295</v>
+      </c>
+      <c r="N35" s="1">
+        <v>47.083333333333336</v>
+      </c>
+      <c r="O35" s="1"/>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36" s="4">
+        <v>-0.02</v>
+      </c>
+      <c r="C36" s="4">
+        <v>39.58333333333333</v>
+      </c>
+      <c r="D36" s="4">
+        <v>1215</v>
+      </c>
+      <c r="E36" s="4">
+        <v>5.89</v>
+      </c>
+      <c r="F36" s="4">
+        <v>-0.048296298967170956</v>
+      </c>
+      <c r="G36" s="4">
+        <v>1.38</v>
+      </c>
+      <c r="H36" s="4">
+        <v>57.58</v>
+      </c>
+      <c r="I36" s="4">
+        <v>-8.94</v>
+      </c>
+      <c r="J36" s="4">
+        <v>0.017724750523772582</v>
+      </c>
+      <c r="K36" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L36" s="4">
+        <v>31</v>
+      </c>
+      <c r="M36" s="4">
+        <v>-0.038258733392037336</v>
+      </c>
+      <c r="N36" s="4">
+        <v>62.08333333333333</v>
+      </c>
+      <c r="O36" s="4"/>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A37" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37" s="4">
+        <v>0.94</v>
+      </c>
+      <c r="C37" s="4">
+        <v>52.083333333333336</v>
+      </c>
+      <c r="D37" s="4">
+        <v>31.03191489361702</v>
+      </c>
+      <c r="E37" s="4">
+        <v>-0.72</v>
+      </c>
+      <c r="F37" s="4">
+        <v>-0.15913082613344948</v>
+      </c>
+      <c r="G37" s="4">
+        <v>2.78</v>
+      </c>
+      <c r="H37" s="4">
+        <v>62.2</v>
+      </c>
+      <c r="I37" s="4">
+        <v>-5.66</v>
+      </c>
+      <c r="J37" s="4">
+        <v>0.010883126809017934</v>
+      </c>
+      <c r="K37" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L37" s="4">
+        <v>134</v>
+      </c>
+      <c r="M37" s="4">
+        <v>-0.11211275580782354</v>
+      </c>
+      <c r="N37" s="4">
+        <v>57.70833333333334</v>
+      </c>
+      <c r="O37" s="4"/>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2">
+        <v>3.41</v>
+      </c>
+      <c r="C38" s="2">
+        <v>72.91666666666666</v>
+      </c>
+      <c r="D38" s="2">
+        <v>8.926686217008797</v>
+      </c>
+      <c r="E38" s="2">
+        <v>-1.19</v>
+      </c>
+      <c r="F38" s="2">
+        <v>0.7532144984691509</v>
+      </c>
+      <c r="G38" s="2">
+        <v>2.08</v>
+      </c>
+      <c r="H38" s="2">
+        <v>68.52</v>
+      </c>
+      <c r="I38" s="2">
+        <v>72.37</v>
+      </c>
+      <c r="J38" s="2">
+        <v>0.04794036718733313</v>
+      </c>
+      <c r="K38" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L38" s="2">
+        <v>234</v>
+      </c>
+      <c r="M38" s="2">
+        <v>0.7817423164195307</v>
+      </c>
+      <c r="N38" s="2">
+        <v>73.33333333333333</v>
+      </c>
+      <c r="O38" s="2"/>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2">
+        <v>-0.38</v>
+      </c>
+      <c r="C39" s="2">
+        <v>31.25</v>
+      </c>
+      <c r="D39" s="2">
+        <v>325.07894736842104</v>
+      </c>
+      <c r="E39" s="2">
+        <v>3.31</v>
+      </c>
+      <c r="F39" s="2">
+        <v>0.4244393059541854</v>
+      </c>
+      <c r="G39" s="2">
+        <v>3.47</v>
+      </c>
+      <c r="H39" s="2">
+        <v>73.96</v>
+      </c>
+      <c r="I39" s="2">
+        <v>120.27</v>
+      </c>
+      <c r="J39" s="2">
+        <v>0.04318873970246332</v>
+      </c>
+      <c r="K39" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L39" s="2">
+        <v>211</v>
+      </c>
+      <c r="M39" s="2">
+        <v>0.489683482192554</v>
+      </c>
+      <c r="N39" s="2">
+        <v>74.58333333333333</v>
+      </c>
+      <c r="O39" s="2"/>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40" s="1">
+        <v>-0.32</v>
+      </c>
+      <c r="C40" s="1">
+        <v>33.33333333333333</v>
+      </c>
+      <c r="D40" s="1">
+        <v>228.28125</v>
+      </c>
+      <c r="E40" s="1">
+        <v>3.34</v>
+      </c>
+      <c r="F40" s="1">
+        <v>-0.20047544049218177</v>
+      </c>
+      <c r="G40" s="1">
+        <v>1.68</v>
+      </c>
+      <c r="H40" s="1">
+        <v>45.97</v>
+      </c>
+      <c r="I40" s="1">
+        <v>-3.8</v>
+      </c>
+      <c r="J40" s="1">
+        <v>-0.01178367415794677</v>
+      </c>
+      <c r="K40" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L40" s="1">
+        <v>11</v>
+      </c>
+      <c r="M40" s="1">
+        <v>-0.18251348104194265</v>
+      </c>
+      <c r="N40" s="1">
+        <v>46.041666666666664</v>
+      </c>
+      <c r="O40" s="1"/>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B41" s="3">
+        <v>-2.92</v>
+      </c>
+      <c r="C41" s="3">
+        <v>14.583333333333334</v>
+      </c>
+      <c r="D41" s="3">
+        <v>-23.77054794520548</v>
+      </c>
+      <c r="E41" s="3">
+        <v>16.88</v>
+      </c>
+      <c r="F41" s="3">
+        <v>0.1549289351552015</v>
+      </c>
+      <c r="G41" s="3">
+        <v>1.95</v>
+      </c>
+      <c r="H41" s="3">
+        <v>70.81</v>
+      </c>
+      <c r="I41" s="3">
+        <v>31.67</v>
+      </c>
+      <c r="J41" s="3">
+        <v>-0.012185710379580567</v>
+      </c>
+      <c r="K41" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L41" s="3">
+        <v>83</v>
+      </c>
+      <c r="M41" s="3">
+        <v>0.18002284909303556</v>
+      </c>
+      <c r="N41" s="3">
+        <v>25.625</v>
+      </c>
+      <c r="O41" s="3"/>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A42" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B42" s="4">
+        <v>4.88</v>
+      </c>
+      <c r="C42" s="4">
+        <v>77.08333333333334</v>
+      </c>
+      <c r="D42" s="4">
+        <v>6.178278688524591</v>
+      </c>
+      <c r="E42" s="4">
+        <v>-0.19</v>
+      </c>
+      <c r="F42" s="4">
+        <v>0.11548747115132582</v>
+      </c>
+      <c r="G42" s="4">
+        <v>1.85</v>
+      </c>
+      <c r="H42" s="4">
+        <v>61.04</v>
+      </c>
+      <c r="I42" s="4">
+        <v>56.14</v>
+      </c>
+      <c r="J42" s="4">
+        <v>0.017137808683028773</v>
+      </c>
+      <c r="K42" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L42" s="4">
+        <v>300</v>
+      </c>
+      <c r="M42" s="4">
+        <v>0.13793992046412473</v>
+      </c>
+      <c r="N42" s="4">
+        <v>64.58333333333334</v>
+      </c>
+      <c r="O42" s="4"/>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B43" s="1">
+        <v>-0.76</v>
+      </c>
+      <c r="C43" s="1">
+        <v>25</v>
+      </c>
+      <c r="D43" s="1">
+        <v>13.236842105263158</v>
+      </c>
+      <c r="E43" s="1">
+        <v>7.72</v>
+      </c>
+      <c r="F43" s="1">
+        <v>-0.38174499445726107</v>
+      </c>
+      <c r="G43" s="1">
+        <v>2.61</v>
+      </c>
+      <c r="H43" s="1">
+        <v>56.14</v>
+      </c>
+      <c r="I43" s="1">
+        <v>-31.84</v>
+      </c>
+      <c r="J43" s="1">
+        <v>-0.01874205106563216</v>
+      </c>
+      <c r="K43" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L43" s="1">
+        <v>64</v>
+      </c>
+      <c r="M43" s="1">
+        <v>-0.3392174139941949</v>
+      </c>
+      <c r="N43" s="1">
+        <v>31.666666666666664</v>
+      </c>
+      <c r="O43" s="1"/>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A44" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B44" s="4">
+        <v>0.54</v>
+      </c>
+      <c r="C44" s="4">
+        <v>47.91666666666667</v>
+      </c>
+      <c r="D44" s="4">
+        <v>41.629629629629626</v>
+      </c>
+      <c r="E44" s="4">
+        <v>0</v>
+      </c>
+      <c r="F44" s="4">
+        <v>0</v>
+      </c>
+      <c r="G44" s="4">
+        <v>1.41</v>
+      </c>
+      <c r="H44" s="4">
+        <v>63.64</v>
+      </c>
+      <c r="I44" s="4">
+        <v>-3.37</v>
+      </c>
+      <c r="J44" s="4">
+        <v>0</v>
+      </c>
+      <c r="K44" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L44" s="4">
+        <v>45</v>
+      </c>
+      <c r="M44" s="4">
+        <v>0</v>
+      </c>
+      <c r="N44" s="4">
+        <v>55.83333333333333</v>
+      </c>
+      <c r="O44" s="4"/>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B45" s="2">
+        <v>0.95</v>
+      </c>
+      <c r="C45" s="2">
+        <v>54.166666666666664</v>
+      </c>
+      <c r="D45" s="2">
+        <v>14.789473684210527</v>
+      </c>
+      <c r="E45" s="2">
+        <v>2.01</v>
+      </c>
+      <c r="F45" s="2">
+        <v>0.31067145981052635</v>
+      </c>
+      <c r="G45" s="2">
+        <v>0.8</v>
+      </c>
+      <c r="H45" s="2">
+        <v>83.89</v>
+      </c>
+      <c r="I45" s="2">
+        <v>36.93</v>
+      </c>
+      <c r="J45" s="2">
+        <v>0.026608906205351935</v>
+      </c>
+      <c r="K45" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L45" s="2">
+        <v>11</v>
+      </c>
+      <c r="M45" s="2">
+        <v>0.305388530560456</v>
+      </c>
+      <c r="N45" s="2">
+        <v>72.08333333333333</v>
+      </c>
+      <c r="O45" s="2"/>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A46" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B46" s="4">
+        <v>1.94</v>
+      </c>
+      <c r="C46" s="4">
+        <v>64.58333333333334</v>
+      </c>
+      <c r="D46" s="4">
+        <v>1.1030927835051547</v>
+      </c>
+      <c r="E46" s="4">
+        <v>0.54</v>
+      </c>
+      <c r="F46" s="4">
+        <v>0.04356416389380155</v>
+      </c>
+      <c r="G46" s="4">
+        <v>0.74</v>
+      </c>
+      <c r="H46" s="4">
+        <v>70.05</v>
+      </c>
+      <c r="I46" s="4">
+        <v>22.64</v>
+      </c>
+      <c r="J46" s="4">
+        <v>0.008830482815401951</v>
+      </c>
+      <c r="K46" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L46" s="4">
+        <v>23</v>
+      </c>
+      <c r="M46" s="4">
+        <v>0.03669635586871012</v>
+      </c>
+      <c r="N46" s="4">
+        <v>52.91666666666667</v>
+      </c>
+      <c r="O46" s="4"/>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A47" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B47" s="4">
+        <v>2.84</v>
+      </c>
+      <c r="C47" s="4">
+        <v>68.75</v>
+      </c>
+      <c r="D47" s="4">
+        <v>2.0880281690140845</v>
+      </c>
+      <c r="E47" s="4">
+        <v>0.95</v>
+      </c>
+      <c r="F47" s="4">
+        <v>0.18093353280757316</v>
+      </c>
+      <c r="G47" s="4">
+        <v>0.88</v>
+      </c>
+      <c r="H47" s="4">
+        <v>72.82</v>
+      </c>
+      <c r="I47" s="4">
+        <v>19.81</v>
+      </c>
+      <c r="J47" s="4">
+        <v>0.004465546501666247</v>
+      </c>
+      <c r="K47" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L47" s="4">
+        <v>248</v>
+      </c>
+      <c r="M47" s="4">
+        <v>0.17776377525753095</v>
+      </c>
+      <c r="N47" s="4">
+        <v>56.666666666666664</v>
+      </c>
+      <c r="O47" s="4"/>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B48" s="2">
+        <v>8.72</v>
+      </c>
+      <c r="C48" s="2">
+        <v>91.66666666666666</v>
+      </c>
+      <c r="D48" s="2">
+        <v>0.8061926605504586</v>
+      </c>
+      <c r="E48" s="2">
+        <v>6.35</v>
+      </c>
+      <c r="F48" s="2">
+        <v>0.873048360184754</v>
+      </c>
+      <c r="G48" s="2">
+        <v>0.96</v>
+      </c>
+      <c r="H48" s="2">
+        <v>72.13</v>
+      </c>
+      <c r="I48" s="2">
+        <v>52.56</v>
+      </c>
+      <c r="J48" s="2">
+        <v>0.05270914285945323</v>
+      </c>
+      <c r="K48" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L48" s="2">
+        <v>115</v>
+      </c>
+      <c r="M48" s="2">
+        <v>0.8719917743347398</v>
+      </c>
+      <c r="N48" s="2">
+        <v>71.875</v>
+      </c>
+      <c r="O48" s="2"/>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A49" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B49" s="4">
+        <v>10.45</v>
+      </c>
+      <c r="C49" s="4">
+        <v>95.83333333333334</v>
+      </c>
+      <c r="D49" s="4">
+        <v>0.4545454545454546</v>
+      </c>
+      <c r="E49" s="4">
+        <v>-0.36</v>
+      </c>
+      <c r="F49" s="4">
+        <v>0.177434564940825</v>
+      </c>
+      <c r="G49" s="4">
+        <v>1.2</v>
+      </c>
+      <c r="H49" s="4">
+        <v>68.18</v>
+      </c>
+      <c r="I49" s="4">
+        <v>14.22</v>
+      </c>
+      <c r="J49" s="4">
+        <v>0.010713778808231215</v>
+      </c>
+      <c r="K49" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L49" s="4">
+        <v>133</v>
+      </c>
+      <c r="M49" s="4">
+        <v>0.18271749419089534</v>
+      </c>
+      <c r="N49" s="4">
+        <v>57.91666666666667</v>
+      </c>
+      <c r="O49" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1026,15 +3307,399 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B49"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>44.375</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>77.29166666666666</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>24.583333333333332</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>51.66666666666667</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>49.375</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>61.875</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>62.708333333333336</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>52.29166666666667</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>46.875</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>22.916666666666668</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>40.208333333333336</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>75.625</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>49.791666666666664</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>36.25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>63.125</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>49.166666666666664</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18">
+        <v>53.54166666666667</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19">
+        <v>43.958333333333336</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <v>27.916666666666664</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <v>25.625</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22">
+        <v>46.04166666666667</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23">
+        <v>24.16666666666667</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24">
+        <v>23.125000000000004</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25">
+        <v>51.87499999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26">
+        <v>61.875</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27">
+        <v>75.62500000000001</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28">
+        <v>43.74999999999999</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29">
+        <v>49.583333333333336</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <v>54.375</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31">
+        <v>50.833333333333336</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32">
+        <v>68.54166666666666</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <v>48.333333333333336</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <v>42.708333333333336</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>47.083333333333336</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <v>62.08333333333333</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37">
+        <v>57.70833333333334</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <v>73.33333333333333</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>38</v>
+      </c>
+      <c r="B39">
+        <v>74.58333333333333</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <v>46.041666666666664</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <v>25.625</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>41</v>
+      </c>
+      <c r="B42">
+        <v>64.58333333333334</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>42</v>
+      </c>
+      <c r="B43">
+        <v>31.666666666666664</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>43</v>
+      </c>
+      <c r="B44">
+        <v>55.83333333333333</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>58</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B45">
+        <v>72.08333333333333</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>59</v>
+      </c>
+      <c r="B46">
+        <v>52.91666666666667</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>60</v>
+      </c>
+      <c r="B47">
+        <v>56.666666666666664</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>61</v>
+      </c>
+      <c r="B48">
+        <v>71.875</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>62</v>
+      </c>
+      <c r="B49">
+        <v>57.91666666666667</v>
       </c>
     </row>
   </sheetData>
@@ -1053,18 +3718,18 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D1" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D2" t="s">
         <v>64</v>
@@ -1072,109 +3737,109 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="C3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D7" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D8" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D9" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D10" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="11" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D11" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="13" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D13" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D14" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D15" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -1193,18 +3858,18 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D1" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>92</v>
+        <v>60</v>
       </c>
       <c r="C2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D2" t="s">
         <v>64</v>
@@ -1212,98 +3877,98 @@
     </row>
     <row r="3" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D8" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D11" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D12" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="14" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1322,18 +3987,18 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D1" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>92</v>
+        <v>60</v>
       </c>
       <c r="C2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D2" t="s">
         <v>64</v>
@@ -1341,98 +4006,98 @@
     </row>
     <row r="3" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D8" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="10" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D11" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D12" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="14" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1451,18 +4116,18 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D1" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="C2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D2" t="s">
         <v>64</v>
@@ -1470,113 +4135,348 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D3" t="s">
         <v>104</v>
-      </c>
-      <c r="C3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D3" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="4" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="5" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="7" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D8" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D9" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D10" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="11" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D11" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="13" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D13" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D14" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D15" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C1" t="s">
+        <v>110</v>
+      </c>
+      <c r="D1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C3" t="s">
+        <v>116</v>
+      </c>
+      <c r="D3" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B5" t="s">
+        <v>122</v>
+      </c>
+      <c r="C5" t="s">
+        <v>123</v>
+      </c>
+      <c r="D5" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>124</v>
+      </c>
+      <c r="B6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C6" t="s">
+        <v>125</v>
+      </c>
+      <c r="D6" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>126</v>
+      </c>
+      <c r="B7" t="s">
+        <v>126</v>
+      </c>
+      <c r="C7" t="s">
+        <v>126</v>
+      </c>
+      <c r="D7" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>127</v>
+      </c>
+      <c r="B8" t="s">
+        <v>128</v>
+      </c>
+      <c r="C8" t="s">
+        <v>126</v>
+      </c>
+      <c r="D8" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>126</v>
+      </c>
+      <c r="B9" t="s">
+        <v>126</v>
+      </c>
+      <c r="C9" t="s">
+        <v>126</v>
+      </c>
+      <c r="D9" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>129</v>
+      </c>
+      <c r="B10" t="s">
+        <v>130</v>
+      </c>
+      <c r="C10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D10" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>126</v>
+      </c>
+      <c r="B15" t="s">
+        <v>126</v>
+      </c>
+      <c r="C15" t="s">
+        <v>126</v>
+      </c>
+      <c r="D15" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>139</v>
+      </c>
+      <c r="B16" t="s">
+        <v>140</v>
+      </c>
+      <c r="C16" t="s">
+        <v>126</v>
+      </c>
+      <c r="D16" t="s">
+        <v>126</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Feature for Earnings Calendar card in next week by changes in index visualizer factors-fundamentals sheet-wrtieSheet
</commit_message>
<xml_diff>
--- a/data/stocks.xlsx
+++ b/data/stocks.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="144">
   <si>
     <t>Ticker</t>
   </si>
@@ -198,12 +198,18 @@
     <t>WSR</t>
   </si>
   <si>
+    <t>BLX</t>
+  </si>
+  <si>
     <t>MD</t>
   </si>
   <si>
     <t>CSCO</t>
   </si>
   <si>
+    <t>JPM</t>
+  </si>
+  <si>
     <t>DELL</t>
   </si>
   <si>
@@ -300,37 +306,40 @@
     <t>Results</t>
   </si>
   <si>
+    <t>3 of 3 qualified</t>
+  </si>
+  <si>
+    <t>Dow Jones 30</t>
+  </si>
+  <si>
+    <t>&gt; $10</t>
+  </si>
+  <si>
+    <t>&gt; +5%</t>
+  </si>
+  <si>
+    <t>&lt; 35</t>
+  </si>
+  <si>
+    <t>All sectors</t>
+  </si>
+  <si>
+    <t>64</t>
+  </si>
+  <si>
     <t>2 of 2 qualified</t>
   </si>
   <si>
-    <t>Dow Jones 30</t>
-  </si>
-  <si>
-    <t>&gt; $10</t>
-  </si>
-  <si>
-    <t>&gt; +5%</t>
-  </si>
-  <si>
-    <t>&lt; 35</t>
-  </si>
-  <si>
-    <t>All sectors</t>
-  </si>
-  <si>
-    <t>64</t>
+    <t>Nasdaq 100</t>
+  </si>
+  <si>
+    <t>&lt; 50</t>
+  </si>
+  <si>
+    <t>0.7 – 1.3</t>
   </si>
   <si>
     <t>1 of 1 qualified</t>
-  </si>
-  <si>
-    <t>Nasdaq 100</t>
-  </si>
-  <si>
-    <t>&lt; 50</t>
-  </si>
-  <si>
-    <t>0.7 – 1.3</t>
   </si>
   <si>
     <t>S&amp;P 500 (large-cap subset)</t>
@@ -1089,7 +1098,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O49"/>
+  <dimension ref="A1:O51"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
@@ -1147,7 +1156,7 @@
         <v>6.69</v>
       </c>
       <c r="C2" s="1">
-        <v>85.41666666666666</v>
+        <v>84</v>
       </c>
       <c r="D2" s="1">
         <v>-0.8191330343796712</v>
@@ -1156,16 +1165,16 @@
         <v>-0.01</v>
       </c>
       <c r="F2" s="1">
-        <v>0.11940253782009777</v>
+        <v>0.11967941242595193</v>
       </c>
       <c r="G2" s="1">
         <v>0.18</v>
       </c>
       <c r="H2" s="1">
-        <v>39.81</v>
+        <v>39.49</v>
       </c>
       <c r="I2" s="1">
-        <v>17.35</v>
+        <v>17.22</v>
       </c>
       <c r="J2" s="1">
         <v>0.0023737785663199627</v>
@@ -1177,12 +1186,14 @@
         <v>364</v>
       </c>
       <c r="M2" s="1">
-        <v>0.09774252789480942</v>
+        <v>0.09928072014955469</v>
       </c>
       <c r="N2" s="1">
-        <v>44.375</v>
-      </c>
-      <c r="O2" s="1"/>
+        <v>43.800000000000004</v>
+      </c>
+      <c r="O2" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -1192,7 +1203,7 @@
         <v>2.64</v>
       </c>
       <c r="C3" s="2">
-        <v>66.66666666666666</v>
+        <v>64</v>
       </c>
       <c r="D3" s="2">
         <v>23.181818181818183</v>
@@ -1201,19 +1212,19 @@
         <v>2.75</v>
       </c>
       <c r="F3" s="2">
-        <v>0.15463133361194895</v>
+        <v>0.15876698515967727</v>
       </c>
       <c r="G3" s="2">
         <v>2.1</v>
       </c>
       <c r="H3" s="2">
-        <v>79.25</v>
+        <v>78.96</v>
       </c>
       <c r="I3" s="2">
-        <v>39.15</v>
+        <v>38.57</v>
       </c>
       <c r="J3" s="2">
-        <v>0.027035824145518757</v>
+        <v>0.02705586046568028</v>
       </c>
       <c r="K3" s="2" t="b">
         <v>0</v>
@@ -1222,12 +1233,14 @@
         <v>375</v>
       </c>
       <c r="M3" s="2">
-        <v>0.18368744448733576</v>
+        <v>0.18613108455484428</v>
       </c>
       <c r="N3" s="2">
-        <v>77.29166666666666</v>
-      </c>
-      <c r="O3" s="2"/>
+        <v>77</v>
+      </c>
+      <c r="O3" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
@@ -1237,7 +1250,7 @@
         <v>-3.95</v>
       </c>
       <c r="C4" s="3">
-        <v>8.333333333333332</v>
+        <v>8</v>
       </c>
       <c r="D4" s="3">
         <v>9.721518987341772</v>
@@ -1246,19 +1259,19 @@
         <v>4.7</v>
       </c>
       <c r="F4" s="3">
-        <v>-0.2997874815980858</v>
+        <v>-0.3033310828445169</v>
       </c>
       <c r="G4" s="3">
         <v>1.18</v>
       </c>
       <c r="H4" s="3">
-        <v>50.03</v>
+        <v>48.95</v>
       </c>
       <c r="I4" s="3">
-        <v>-27.2</v>
+        <v>-27.88</v>
       </c>
       <c r="J4" s="3">
-        <v>-0.01432968093560943</v>
+        <v>-0.01446289471733941</v>
       </c>
       <c r="K4" s="3" t="b">
         <v>0</v>
@@ -1267,12 +1280,14 @@
         <v>50</v>
       </c>
       <c r="M4" s="3">
-        <v>-0.29503284527302254</v>
+        <v>-0.2988533211253077</v>
       </c>
       <c r="N4" s="3">
-        <v>24.583333333333332</v>
-      </c>
-      <c r="O4" s="3"/>
+        <v>24.6</v>
+      </c>
+      <c r="O4" s="3">
+        <v>-0.2</v>
+      </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
@@ -1282,28 +1297,28 @@
         <v>1.08</v>
       </c>
       <c r="C5" s="4">
-        <v>56.25</v>
+        <v>54</v>
       </c>
       <c r="D5" s="4">
-        <v>27.981481481481477</v>
+        <v>27.944444444444443</v>
       </c>
       <c r="E5" s="4">
         <v>0.58</v>
       </c>
       <c r="F5" s="4">
-        <v>-0.1324852835010605</v>
+        <v>-0.12866175509386943</v>
       </c>
       <c r="G5" s="4">
         <v>1.85</v>
       </c>
       <c r="H5" s="4">
-        <v>55.13</v>
+        <v>54.34</v>
       </c>
       <c r="I5" s="4">
-        <v>-2.42</v>
+        <v>-2.85</v>
       </c>
       <c r="J5" s="4">
-        <v>-0.004872619589082648</v>
+        <v>-0.004851686507586286</v>
       </c>
       <c r="K5" s="4" t="b">
         <v>0</v>
@@ -1312,12 +1327,14 @@
         <v>312</v>
       </c>
       <c r="M5" s="4">
-        <v>-0.1100328341882616</v>
+        <v>-0.107516769197604</v>
       </c>
       <c r="N5" s="4">
-        <v>51.66666666666667</v>
-      </c>
-      <c r="O5" s="4"/>
+        <v>50.800000000000004</v>
+      </c>
+      <c r="O5" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
@@ -1327,7 +1344,7 @@
         <v>3.09</v>
       </c>
       <c r="C6" s="1">
-        <v>70.83333333333334</v>
+        <v>68</v>
       </c>
       <c r="D6" s="1">
         <v>1.5663430420711975</v>
@@ -1336,19 +1353,19 @@
         <v>-2.3</v>
       </c>
       <c r="F6" s="1">
-        <v>0.015574698750199387</v>
+        <v>0.016374056771371423</v>
       </c>
       <c r="G6" s="1">
         <v>1.6</v>
       </c>
       <c r="H6" s="1">
-        <v>41.72</v>
+        <v>41.41</v>
       </c>
       <c r="I6" s="1">
-        <v>-11.59</v>
+        <v>-11.78</v>
       </c>
       <c r="J6" s="1">
-        <v>0.020971830186022736</v>
+        <v>0.02093980443525671</v>
       </c>
       <c r="K6" s="1" t="b">
         <v>1</v>
@@ -1357,12 +1374,14 @@
         <v>139</v>
       </c>
       <c r="M6" s="1">
-        <v>0.03142348650041038</v>
+        <v>0.03129992916873525</v>
       </c>
       <c r="N6" s="1">
-        <v>49.375</v>
-      </c>
-      <c r="O6" s="1"/>
+        <v>49.6</v>
+      </c>
+      <c r="O6" s="1">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
@@ -1372,7 +1391,7 @@
         <v>4.9</v>
       </c>
       <c r="C7" s="4">
-        <v>79.16666666666666</v>
+        <v>76</v>
       </c>
       <c r="D7" s="4">
         <v>5.9</v>
@@ -1381,19 +1400,19 @@
         <v>0.37</v>
       </c>
       <c r="F7" s="4">
-        <v>0.05216692912061721</v>
+        <v>0.05439778654196077</v>
       </c>
       <c r="G7" s="4">
         <v>2.29</v>
       </c>
       <c r="H7" s="4">
-        <v>68.67</v>
+        <v>67.39</v>
       </c>
       <c r="I7" s="4">
-        <v>10.03</v>
+        <v>9.64</v>
       </c>
       <c r="J7" s="4">
-        <v>0.011374279129554401</v>
+        <v>0.011349021721240592</v>
       </c>
       <c r="K7" s="4" t="b">
         <v>0</v>
@@ -1402,12 +1421,14 @@
         <v>434</v>
       </c>
       <c r="M7" s="4">
-        <v>0.08624182278357084</v>
+        <v>0.086488412196293</v>
       </c>
       <c r="N7" s="4">
-        <v>61.875</v>
-      </c>
-      <c r="O7" s="4"/>
+        <v>61</v>
+      </c>
+      <c r="O7" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
@@ -1417,7 +1438,7 @@
         <v>13.19</v>
       </c>
       <c r="C8" s="4">
-        <v>97.91666666666666</v>
+        <v>96</v>
       </c>
       <c r="D8" s="4">
         <v>-0.044730856709628494</v>
@@ -1426,19 +1447,19 @@
         <v>0.43</v>
       </c>
       <c r="F8" s="4">
-        <v>0.013480296772397392</v>
+        <v>0.018164476427022368</v>
       </c>
       <c r="G8" s="4">
         <v>0.5</v>
       </c>
       <c r="H8" s="4">
-        <v>80.84</v>
+        <v>80.91</v>
       </c>
       <c r="I8" s="4">
-        <v>12.36</v>
+        <v>12.46</v>
       </c>
       <c r="J8" s="4">
-        <v>0.016806327810061392</v>
+        <v>0.016899589420790572</v>
       </c>
       <c r="K8" s="4" t="b">
         <v>0</v>
@@ -1447,12 +1468,14 @@
         <v>69</v>
       </c>
       <c r="M8" s="4">
-        <v>0.0002729736472215638</v>
+        <v>0.005726249429219177</v>
       </c>
       <c r="N8" s="4">
-        <v>62.708333333333336</v>
-      </c>
-      <c r="O8" s="4"/>
+        <v>63.599999999999994</v>
+      </c>
+      <c r="O8" s="4">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
@@ -1462,7 +1485,7 @@
         <v>0.63</v>
       </c>
       <c r="C9" s="4">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D9" s="4">
         <v>67.1111111111111</v>
@@ -1471,19 +1494,19 @@
         <v>1.75</v>
       </c>
       <c r="F9" s="4">
-        <v>-0.18257434339651085</v>
+        <v>-0.17753265067641916</v>
       </c>
       <c r="G9" s="4">
         <v>1.6</v>
       </c>
       <c r="H9" s="4">
-        <v>52.98</v>
+        <v>52.36</v>
       </c>
       <c r="I9" s="4">
-        <v>-10.4</v>
+        <v>-10.8</v>
       </c>
       <c r="J9" s="4">
-        <v>0.0017804758732523362</v>
+        <v>0.001840994302116228</v>
       </c>
       <c r="K9" s="4" t="b">
         <v>0</v>
@@ -1492,12 +1515,14 @@
         <v>189</v>
       </c>
       <c r="M9" s="4">
-        <v>-0.16672555564629987</v>
+        <v>-0.16260677827905534</v>
       </c>
       <c r="N9" s="4">
-        <v>52.29166666666667</v>
-      </c>
-      <c r="O9" s="4"/>
+        <v>52</v>
+      </c>
+      <c r="O9" s="4">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
@@ -1507,7 +1532,7 @@
         <v>6.79</v>
       </c>
       <c r="C10" s="1">
-        <v>87.5</v>
+        <v>86</v>
       </c>
       <c r="D10" s="1">
         <v>0.6435935198821797</v>
@@ -1516,19 +1541,19 @@
         <v>0.88</v>
       </c>
       <c r="F10" s="1">
-        <v>-0.09935027283030967</v>
+        <v>-0.0974824182303593</v>
       </c>
       <c r="G10" s="1">
         <v>1.45</v>
       </c>
       <c r="H10" s="1">
-        <v>62.08</v>
+        <v>62.54</v>
       </c>
       <c r="I10" s="1">
-        <v>-5.15</v>
+        <v>-5.04</v>
       </c>
       <c r="J10" s="1">
-        <v>-0.0009973918374701378</v>
+        <v>-0.0010052609990238268</v>
       </c>
       <c r="K10" s="1" t="b">
         <v>0</v>
@@ -1537,12 +1562,14 @@
         <v>56</v>
       </c>
       <c r="M10" s="1">
-        <v>-0.08746368201765142</v>
+        <v>-0.08628801393233643</v>
       </c>
       <c r="N10" s="1">
-        <v>46.875</v>
-      </c>
-      <c r="O10" s="1"/>
+        <v>48.4</v>
+      </c>
+      <c r="O10" s="1">
+        <v>1</v>
+      </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
@@ -1552,7 +1579,7 @@
         <v>0.02</v>
       </c>
       <c r="C11" s="3">
-        <v>43.75</v>
+        <v>42</v>
       </c>
       <c r="D11" s="3">
         <v>-1653.5</v>
@@ -1561,16 +1588,16 @@
         <v>10.01</v>
       </c>
       <c r="F11" s="3">
-        <v>-0.2373041633607682</v>
+        <v>-0.23513531228157736</v>
       </c>
       <c r="G11" s="3">
         <v>1.41</v>
       </c>
       <c r="H11" s="3">
-        <v>49.11</v>
+        <v>47.58</v>
       </c>
       <c r="I11" s="3">
-        <v>-0.49</v>
+        <v>-1.59</v>
       </c>
       <c r="J11" s="3">
         <v>-0.012954170042827666</v>
@@ -1582,12 +1609,14 @@
         <v>28</v>
       </c>
       <c r="M11" s="3">
-        <v>-0.22647415839812401</v>
+        <v>-0.22493596614337874</v>
       </c>
       <c r="N11" s="3">
-        <v>22.916666666666668</v>
-      </c>
-      <c r="O11" s="3"/>
+        <v>22</v>
+      </c>
+      <c r="O11" s="3">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
@@ -1597,7 +1626,7 @@
         <v>1.31</v>
       </c>
       <c r="C12" s="1">
-        <v>60.416666666666664</v>
+        <v>57.99999999999999</v>
       </c>
       <c r="D12" s="1">
         <v>7.5114503816793885</v>
@@ -1606,19 +1635,19 @@
         <v>0.13</v>
       </c>
       <c r="F12" s="1">
-        <v>-0.1266387692870606</v>
+        <v>-0.13422061465190438</v>
       </c>
       <c r="G12" s="1">
         <v>0.63</v>
       </c>
       <c r="H12" s="1">
-        <v>55.45</v>
+        <v>54.75</v>
       </c>
       <c r="I12" s="1">
-        <v>-9.56</v>
+        <v>-10.23</v>
       </c>
       <c r="J12" s="1">
-        <v>-0.01441421206345179</v>
+        <v>-0.014605975442797736</v>
       </c>
       <c r="K12" s="1" t="b">
         <v>0</v>
@@ -1627,12 +1656,14 @@
         <v>10</v>
       </c>
       <c r="M12" s="1">
-        <v>-0.13641218839969071</v>
+        <v>-0.14342490263027874</v>
       </c>
       <c r="N12" s="1">
-        <v>40.208333333333336</v>
-      </c>
-      <c r="O12" s="1"/>
+        <v>40.2</v>
+      </c>
+      <c r="O12" s="1">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
@@ -1642,7 +1673,7 @@
         <v>-0.08</v>
       </c>
       <c r="C13" s="2">
-        <v>37.5</v>
+        <v>36</v>
       </c>
       <c r="D13" s="2">
         <v>1166</v>
@@ -1651,19 +1682,19 @@
         <v>6.17</v>
       </c>
       <c r="F13" s="2">
-        <v>0.31134277324890075</v>
+        <v>0.31368202773667075</v>
       </c>
       <c r="G13" s="2">
         <v>1.66</v>
       </c>
       <c r="H13" s="2">
-        <v>71.41</v>
+        <v>70.84</v>
       </c>
       <c r="I13" s="2">
-        <v>76.95</v>
+        <v>75.58</v>
       </c>
       <c r="J13" s="2">
-        <v>0.036955400678864</v>
+        <v>0.03695105739468107</v>
       </c>
       <c r="K13" s="2" t="b">
         <v>0</v>
@@ -1672,57 +1703,61 @@
         <v>249</v>
       </c>
       <c r="M13" s="2">
-        <v>0.32877643977413284</v>
+        <v>0.33010048737377096</v>
       </c>
       <c r="N13" s="2">
-        <v>75.625</v>
-      </c>
-      <c r="O13" s="2"/>
+        <v>75.2</v>
+      </c>
+      <c r="O13" s="2">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="1">
+      <c r="B14" s="4">
         <v>-3.83</v>
       </c>
-      <c r="C14" s="1">
-        <v>10.416666666666668</v>
-      </c>
-      <c r="D14" s="1">
+      <c r="C14" s="4">
+        <v>10</v>
+      </c>
+      <c r="D14" s="4">
         <v>12.668407310704959</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="4">
         <v>2.52</v>
       </c>
-      <c r="F14" s="1">
-        <v>0.1367064575621085</v>
-      </c>
-      <c r="G14" s="1">
+      <c r="F14" s="4">
+        <v>0.15078708560651521</v>
+      </c>
+      <c r="G14" s="4">
         <v>2.06</v>
       </c>
-      <c r="H14" s="1">
-        <v>64.5</v>
-      </c>
-      <c r="I14" s="1">
-        <v>18.73</v>
-      </c>
-      <c r="J14" s="1">
-        <v>0.019616079754584414</v>
-      </c>
-      <c r="K14" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="L14" s="1">
+      <c r="H14" s="4">
+        <v>64.43</v>
+      </c>
+      <c r="I14" s="4">
+        <v>18.63</v>
+      </c>
+      <c r="J14" s="4">
+        <v>0.019829962781969673</v>
+      </c>
+      <c r="K14" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L14" s="4">
         <v>27</v>
       </c>
-      <c r="M14" s="1">
-        <v>0.16470598258748126</v>
-      </c>
-      <c r="N14" s="1">
-        <v>49.791666666666664</v>
-      </c>
-      <c r="O14" s="1"/>
+      <c r="M14" s="4">
+        <v>0.177156126841858</v>
+      </c>
+      <c r="N14" s="4">
+        <v>50.199999999999996</v>
+      </c>
+      <c r="O14" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
@@ -1732,7 +1767,7 @@
         <v>-6.51</v>
       </c>
       <c r="C15" s="1">
-        <v>4.166666666666666</v>
+        <v>4</v>
       </c>
       <c r="D15" s="1">
         <v>4.411674347158218</v>
@@ -1741,19 +1776,19 @@
         <v>4.53</v>
       </c>
       <c r="F15" s="1">
-        <v>0.02551684943171327</v>
+        <v>0.022359621987671996</v>
       </c>
       <c r="G15" s="1">
         <v>1.84</v>
       </c>
       <c r="H15" s="1">
-        <v>63.5</v>
+        <v>62</v>
       </c>
       <c r="I15" s="1">
-        <v>1.17</v>
+        <v>0.41</v>
       </c>
       <c r="J15" s="1">
-        <v>0.014393856469644214</v>
+        <v>0.014271758714584973</v>
       </c>
       <c r="K15" s="1" t="b">
         <v>0</v>
@@ -1762,12 +1797,14 @@
         <v>43</v>
       </c>
       <c r="M15" s="1">
-        <v>0.04770515228200867</v>
+        <v>0.04325584334398136</v>
       </c>
       <c r="N15" s="1">
-        <v>36.25</v>
-      </c>
-      <c r="O15" s="1"/>
+        <v>36.400000000000006</v>
+      </c>
+      <c r="O15" s="1">
+        <v>-0.4</v>
+      </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
@@ -1777,7 +1814,7 @@
         <v>-0.01</v>
       </c>
       <c r="C16" s="4">
-        <v>41.66666666666667</v>
+        <v>40</v>
       </c>
       <c r="D16" s="4">
         <v>18685</v>
@@ -1786,19 +1823,19 @@
         <v>11.11</v>
       </c>
       <c r="F16" s="4">
-        <v>-0.07710107317789963</v>
+        <v>-0.08136562225678619</v>
       </c>
       <c r="G16" s="4">
         <v>1.23</v>
       </c>
       <c r="H16" s="4">
-        <v>66.28</v>
+        <v>66.22</v>
       </c>
       <c r="I16" s="4">
-        <v>22.53</v>
+        <v>22.47</v>
       </c>
       <c r="J16" s="4">
-        <v>-0.003388255450886434</v>
+        <v>-0.003532875449604242</v>
       </c>
       <c r="K16" s="4" t="b">
         <v>0</v>
@@ -1807,12 +1844,14 @@
         <v>32</v>
       </c>
       <c r="M16" s="4">
-        <v>-0.07102570454031876</v>
+        <v>-0.07564403783779672</v>
       </c>
       <c r="N16" s="4">
-        <v>63.125</v>
-      </c>
-      <c r="O16" s="4"/>
+        <v>62.6</v>
+      </c>
+      <c r="O16" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
@@ -1822,7 +1861,7 @@
         <v>8.81</v>
       </c>
       <c r="C17" s="1">
-        <v>93.75</v>
+        <v>92</v>
       </c>
       <c r="D17" s="1">
         <v>-0.27922814982973904</v>
@@ -1831,19 +1870,19 @@
         <v>4.52</v>
       </c>
       <c r="F17" s="1">
-        <v>0.11848178357699889</v>
+        <v>0.11748865655087395</v>
       </c>
       <c r="G17" s="1">
         <v>0.17</v>
       </c>
       <c r="H17" s="1">
-        <v>56.37</v>
+        <v>56.43</v>
       </c>
       <c r="I17" s="1">
-        <v>15.34</v>
+        <v>15.38</v>
       </c>
       <c r="J17" s="1">
-        <v>-0.002480406015349057</v>
+        <v>-0.0025026903760530404</v>
       </c>
       <c r="K17" s="1" t="b">
         <v>0</v>
@@ -1852,12 +1891,14 @@
         <v>94</v>
       </c>
       <c r="M17" s="1">
-        <v>0.09655762718920702</v>
+        <v>0.09684119973452066</v>
       </c>
       <c r="N17" s="1">
-        <v>49.166666666666664</v>
-      </c>
-      <c r="O17" s="1"/>
+        <v>48.99999999999999</v>
+      </c>
+      <c r="O17" s="1">
+        <v>0.4</v>
+      </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
@@ -1876,19 +1917,19 @@
         <v>-1.85</v>
       </c>
       <c r="F18" s="4">
-        <v>-0.06458700033216558</v>
+        <v>-0.0675655590646727</v>
       </c>
       <c r="G18" s="4">
         <v>1.14</v>
       </c>
       <c r="H18" s="4">
-        <v>69.94</v>
+        <v>69.08</v>
       </c>
       <c r="I18" s="4">
-        <v>4.92</v>
+        <v>4.38</v>
       </c>
       <c r="J18" s="4">
-        <v>-0.0006200222082913154</v>
+        <v>-0.0007267240423029835</v>
       </c>
       <c r="K18" s="4" t="b">
         <v>0</v>
@@ -1897,12 +1938,14 @@
         <v>4</v>
       </c>
       <c r="M18" s="4">
-        <v>-0.06088894985711635</v>
+        <v>-0.0640828555052878</v>
       </c>
       <c r="N18" s="4">
-        <v>53.54166666666667</v>
-      </c>
-      <c r="O18" s="4"/>
+        <v>54.2</v>
+      </c>
+      <c r="O18" s="4">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
@@ -1912,7 +1955,7 @@
         <v>1.29</v>
       </c>
       <c r="C19" s="1">
-        <v>58.333333333333336</v>
+        <v>56.00000000000001</v>
       </c>
       <c r="D19" s="1">
         <v>15.426356589147288</v>
@@ -1921,19 +1964,19 @@
         <v>3.37</v>
       </c>
       <c r="F19" s="1">
-        <v>-0.04129758439236603</v>
+        <v>-0.055505071827900376</v>
       </c>
       <c r="G19" s="1">
         <v>1.31</v>
       </c>
       <c r="H19" s="1">
-        <v>46.23</v>
+        <v>43.15</v>
       </c>
       <c r="I19" s="1">
-        <v>-4.53</v>
+        <v>-6.89</v>
       </c>
       <c r="J19" s="1">
-        <v>-0.027338011861329586</v>
+        <v>-0.027605050492327275</v>
       </c>
       <c r="K19" s="1" t="b">
         <v>1</v>
@@ -1942,12 +1985,14 @@
         <v>-7</v>
       </c>
       <c r="M19" s="1">
-        <v>-0.03310904405475701</v>
+        <v>-0.047793371089262404</v>
       </c>
       <c r="N19" s="1">
-        <v>43.958333333333336</v>
-      </c>
-      <c r="O19" s="1"/>
+        <v>42.8</v>
+      </c>
+      <c r="O19" s="1">
+        <v>-0.2</v>
+      </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
@@ -1957,7 +2002,7 @@
         <v>-18.39</v>
       </c>
       <c r="C20" s="3">
-        <v>2.083333333333333</v>
+        <v>2</v>
       </c>
       <c r="D20" s="3">
         <v>-4.206090266449157</v>
@@ -1966,19 +2011,19 @@
         <v>8.76</v>
       </c>
       <c r="F20" s="3">
-        <v>-0.061258483063819674</v>
+        <v>-0.05948272480163863</v>
       </c>
       <c r="G20" s="3">
         <v>3.67</v>
       </c>
       <c r="H20" s="3">
-        <v>71</v>
+        <v>69.53</v>
       </c>
       <c r="I20" s="3">
-        <v>-29.81</v>
+        <v>-30.43</v>
       </c>
       <c r="J20" s="3">
-        <v>0.023188818679715038</v>
+        <v>0.023095206533151898</v>
       </c>
       <c r="K20" s="3" t="b">
         <v>1</v>
@@ -1987,12 +2032,14 @@
         <v>-44</v>
       </c>
       <c r="M20" s="3">
-        <v>0.009268622424619233</v>
+        <v>0.006937407366630399</v>
       </c>
       <c r="N20" s="3">
-        <v>27.916666666666664</v>
-      </c>
-      <c r="O20" s="3"/>
+        <v>27.400000000000002</v>
+      </c>
+      <c r="O20" s="3">
+        <v>0</v>
+      </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
@@ -2002,7 +2049,7 @@
         <v>-2.25</v>
       </c>
       <c r="C21" s="3">
-        <v>18.75</v>
+        <v>18</v>
       </c>
       <c r="D21" s="3">
         <v>10.44</v>
@@ -2011,19 +2058,19 @@
         <v>12.21</v>
       </c>
       <c r="F21" s="3">
-        <v>-0.43969939957864956</v>
+        <v>-0.4405830197438053</v>
       </c>
       <c r="G21" s="3">
         <v>2.31</v>
       </c>
       <c r="H21" s="3">
-        <v>54.4</v>
+        <v>53.95</v>
       </c>
       <c r="I21" s="3">
-        <v>-55.05</v>
+        <v>-55.29</v>
       </c>
       <c r="J21" s="3">
-        <v>-0.03547797069677966</v>
+        <v>-0.03561172296348668</v>
       </c>
       <c r="K21" s="3" t="b">
         <v>1</v>
@@ -2032,12 +2079,14 @@
         <v>17</v>
       </c>
       <c r="M21" s="3">
-        <v>-0.4050962129906889</v>
+        <v>-0.40799486500956095</v>
       </c>
       <c r="N21" s="3">
-        <v>25.625</v>
-      </c>
-      <c r="O21" s="3"/>
+        <v>25.799999999999994</v>
+      </c>
+      <c r="O21" s="3">
+        <v>0</v>
+      </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
@@ -2047,7 +2096,7 @@
         <v>-2.38</v>
       </c>
       <c r="C22" s="1">
-        <v>16.666666666666664</v>
+        <v>16</v>
       </c>
       <c r="D22" s="1">
         <v>1.4705882352941178</v>
@@ -2056,19 +2105,19 @@
         <v>5.89</v>
       </c>
       <c r="F22" s="1">
-        <v>-0.17120120712554815</v>
+        <v>-0.1655971450178095</v>
       </c>
       <c r="G22" s="1">
         <v>3.13</v>
       </c>
       <c r="H22" s="1">
-        <v>73.51</v>
+        <v>72.8</v>
       </c>
       <c r="I22" s="1">
-        <v>0.82</v>
+        <v>0.29</v>
       </c>
       <c r="J22" s="1">
-        <v>0.03109288839166161</v>
+        <v>0.031117144788648583</v>
       </c>
       <c r="K22" s="1" t="b">
         <v>1</v>
@@ -2077,12 +2126,14 @@
         <v>43</v>
       </c>
       <c r="M22" s="1">
-        <v>-0.11493801061229914</v>
+        <v>-0.11261029800716793</v>
       </c>
       <c r="N22" s="1">
-        <v>46.04166666666667</v>
-      </c>
-      <c r="O22" s="1"/>
+        <v>46.400000000000006</v>
+      </c>
+      <c r="O22" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
@@ -2092,7 +2143,7 @@
         <v>-1.13</v>
       </c>
       <c r="C23" s="3">
-        <v>20.833333333333336</v>
+        <v>20</v>
       </c>
       <c r="D23" s="3">
         <v>5.7522123893805315</v>
@@ -2101,7 +2152,7 @@
         <v>1.42</v>
       </c>
       <c r="F23" s="3">
-        <v>-0.4662787098315891</v>
+        <v>-0.46051095944106835</v>
       </c>
       <c r="G23" s="3">
         <v>2.65</v>
@@ -2113,7 +2164,7 @@
         <v>-33.89</v>
       </c>
       <c r="J23" s="3">
-        <v>-0.012401909198076783</v>
+        <v>-0.012349525627281642</v>
       </c>
       <c r="K23" s="3" t="b">
         <v>0</v>
@@ -2122,12 +2173,14 @@
         <v>37</v>
       </c>
       <c r="M23" s="3">
-        <v>-0.4226945435185089</v>
+        <v>-0.41946481034831784</v>
       </c>
       <c r="N23" s="3">
-        <v>24.16666666666667</v>
-      </c>
-      <c r="O23" s="3"/>
+        <v>24.599999999999998</v>
+      </c>
+      <c r="O23" s="3">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
@@ -2137,7 +2190,7 @@
         <v>-0.99</v>
       </c>
       <c r="C24" s="3">
-        <v>22.916666666666664</v>
+        <v>22</v>
       </c>
       <c r="D24" s="3">
         <v>3.04040404040404</v>
@@ -2146,19 +2199,19 @@
         <v>3.54</v>
       </c>
       <c r="F24" s="3">
-        <v>-0.40154728528252626</v>
+        <v>-0.400598246421679</v>
       </c>
       <c r="G24" s="3">
         <v>3.24</v>
       </c>
       <c r="H24" s="3">
-        <v>53.77</v>
+        <v>52.34</v>
       </c>
       <c r="I24" s="3">
-        <v>-29.95</v>
+        <v>-30.64</v>
       </c>
       <c r="J24" s="3">
-        <v>-0.01464141824677345</v>
+        <v>-0.014752019382312919</v>
       </c>
       <c r="K24" s="3" t="b">
         <v>0</v>
@@ -2167,12 +2220,14 @@
         <v>60</v>
       </c>
       <c r="M24" s="3">
-        <v>-0.34237847768173857</v>
+        <v>-0.34487498947152073</v>
       </c>
       <c r="N24" s="3">
-        <v>23.125000000000004</v>
-      </c>
-      <c r="O24" s="3"/>
+        <v>23.200000000000003</v>
+      </c>
+      <c r="O24" s="3">
+        <v>-0.4</v>
+      </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
@@ -2182,7 +2237,7 @@
         <v>0.38</v>
       </c>
       <c r="C25" s="4">
-        <v>45.83333333333333</v>
+        <v>44</v>
       </c>
       <c r="D25" s="4">
         <v>89.71052631578947</v>
@@ -2191,19 +2246,19 @@
         <v>2.21</v>
       </c>
       <c r="F25" s="4">
-        <v>-0.3170927581740075</v>
+        <v>-0.31542297047728074</v>
       </c>
       <c r="G25" s="4">
         <v>2.32</v>
       </c>
       <c r="H25" s="4">
-        <v>63.79</v>
+        <v>63.1</v>
       </c>
       <c r="I25" s="4">
-        <v>-19.66</v>
+        <v>-19.91</v>
       </c>
       <c r="J25" s="4">
-        <v>-0.009812260461178298</v>
+        <v>-0.009865523158916659</v>
       </c>
       <c r="K25" s="4" t="b">
         <v>0</v>
@@ -2212,12 +2267,14 @@
         <v>70</v>
       </c>
       <c r="M25" s="4">
-        <v>-0.2822254251235433</v>
+        <v>-0.28258605120308034</v>
       </c>
       <c r="N25" s="4">
-        <v>51.87499999999999</v>
-      </c>
-      <c r="O25" s="4"/>
+        <v>51</v>
+      </c>
+      <c r="O25" s="4">
+        <v>-0.2</v>
+      </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
@@ -2227,7 +2284,7 @@
         <v>1.9</v>
       </c>
       <c r="C26" s="4">
-        <v>62.5</v>
+        <v>60</v>
       </c>
       <c r="D26" s="4">
         <v>2990.236842105264</v>
@@ -2236,19 +2293,19 @@
         <v>2.07</v>
       </c>
       <c r="F26" s="4">
-        <v>-0.1547367590902501</v>
+        <v>-0.15608369211525974</v>
       </c>
       <c r="G26" s="4">
         <v>1.2</v>
       </c>
       <c r="H26" s="4">
-        <v>55.52</v>
+        <v>54.45</v>
       </c>
       <c r="I26" s="4">
-        <v>0.85</v>
+        <v>0.38</v>
       </c>
       <c r="J26" s="4">
-        <v>-0.006328987029654367</v>
+        <v>-0.006401082366864428</v>
       </c>
       <c r="K26" s="4" t="b">
         <v>0</v>
@@ -2257,12 +2314,14 @@
         <v>116</v>
       </c>
       <c r="M26" s="4">
-        <v>-0.14945382984017974</v>
+        <v>-0.15110840131613845</v>
       </c>
       <c r="N26" s="4">
-        <v>61.875</v>
-      </c>
-      <c r="O26" s="4"/>
+        <v>60.400000000000006</v>
+      </c>
+      <c r="O26" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
@@ -2272,7 +2331,7 @@
         <v>5.13</v>
       </c>
       <c r="C27" s="2">
-        <v>81.25</v>
+        <v>78</v>
       </c>
       <c r="D27" s="2">
         <v>10.491228070175438</v>
@@ -2281,19 +2340,19 @@
         <v>0.39</v>
       </c>
       <c r="F27" s="2">
-        <v>0.16421433169186833</v>
+        <v>0.1639470722757364</v>
       </c>
       <c r="G27" s="2">
         <v>1.39</v>
       </c>
       <c r="H27" s="2">
-        <v>74.94</v>
+        <v>74.36</v>
       </c>
       <c r="I27" s="2">
-        <v>20.62</v>
+        <v>19.93</v>
       </c>
       <c r="J27" s="2">
-        <v>0.024434924341505217</v>
+        <v>0.024386229289761436</v>
       </c>
       <c r="K27" s="2" t="b">
         <v>0</v>
@@ -2302,12 +2361,14 @@
         <v>412</v>
       </c>
       <c r="M27" s="2">
-        <v>0.17451604372950547</v>
+        <v>0.1736488893340229</v>
       </c>
       <c r="N27" s="2">
-        <v>75.62500000000001</v>
-      </c>
-      <c r="O27" s="2"/>
+        <v>75.2</v>
+      </c>
+      <c r="O27" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
@@ -2317,7 +2378,7 @@
         <v>-3.07</v>
       </c>
       <c r="C28" s="1">
-        <v>12.5</v>
+        <v>12</v>
       </c>
       <c r="D28" s="1">
         <v>8.671009771986972</v>
@@ -2326,19 +2387,19 @@
         <v>2.29</v>
       </c>
       <c r="F28" s="1">
-        <v>0.00989392080333086</v>
+        <v>0.0041394910754501135</v>
       </c>
       <c r="G28" s="1">
         <v>1.69</v>
       </c>
       <c r="H28" s="1">
-        <v>63.26</v>
+        <v>62.1</v>
       </c>
       <c r="I28" s="1">
-        <v>13.66</v>
+        <v>12.57</v>
       </c>
       <c r="J28" s="1">
-        <v>0.0168781609811</v>
+        <v>0.016701733911623943</v>
       </c>
       <c r="K28" s="1" t="b">
         <v>0</v>
@@ -2347,57 +2408,61 @@
         <v>44</v>
       </c>
       <c r="M28" s="1">
-        <v>0.0281200267160735</v>
+        <v>0.02130424433241851</v>
       </c>
       <c r="N28" s="1">
-        <v>43.74999999999999</v>
-      </c>
-      <c r="O28" s="1"/>
+        <v>43.800000000000004</v>
+      </c>
+      <c r="O28" s="1">
+        <v>-0.8</v>
+      </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
+      <c r="A29" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B29" s="1">
+      <c r="B29" s="4">
         <v>7.4</v>
       </c>
-      <c r="C29" s="1">
-        <v>89.58333333333334</v>
-      </c>
-      <c r="D29" s="1">
+      <c r="C29" s="4">
+        <v>88</v>
+      </c>
+      <c r="D29" s="4">
         <v>1.2283783783783782</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="4">
         <v>-0.84</v>
       </c>
-      <c r="F29" s="1">
-        <v>-0.09024617250147376</v>
-      </c>
-      <c r="G29" s="1">
+      <c r="F29" s="4">
+        <v>-0.09146541819570014</v>
+      </c>
+      <c r="G29" s="4">
         <v>1.1</v>
       </c>
-      <c r="H29" s="1">
-        <v>42.46</v>
-      </c>
-      <c r="I29" s="1">
+      <c r="H29" s="4">
+        <v>42.45</v>
+      </c>
+      <c r="I29" s="4">
         <v>-14.49</v>
       </c>
-      <c r="J29" s="1">
-        <v>0.010836343223542119</v>
-      </c>
-      <c r="K29" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="L29" s="1">
+      <c r="J29" s="4">
+        <v>0.010778051501450026</v>
+      </c>
+      <c r="K29" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L29" s="4">
         <v>149</v>
       </c>
-      <c r="M29" s="1">
-        <v>-0.08760470787643859</v>
-      </c>
-      <c r="N29" s="1">
-        <v>49.583333333333336</v>
-      </c>
-      <c r="O29" s="1"/>
+      <c r="M29" s="4">
+        <v>-0.0889777727961395</v>
+      </c>
+      <c r="N29" s="4">
+        <v>50.4</v>
+      </c>
+      <c r="O29" s="4">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
@@ -2407,7 +2472,7 @@
         <v>5.41</v>
       </c>
       <c r="C30" s="4">
-        <v>83.33333333333334</v>
+        <v>80</v>
       </c>
       <c r="D30" s="4">
         <v>0.6598890942698706</v>
@@ -2416,19 +2481,19 @@
         <v>-0.09</v>
       </c>
       <c r="F30" s="4">
-        <v>-0.11560724672853408</v>
+        <v>-0.11776489135020235</v>
       </c>
       <c r="G30" s="4">
         <v>1.43</v>
       </c>
       <c r="H30" s="4">
-        <v>70.08</v>
+        <v>68.13</v>
       </c>
       <c r="I30" s="4">
-        <v>-14.71</v>
+        <v>-15.24</v>
       </c>
       <c r="J30" s="4">
-        <v>0.016935392611379864</v>
+        <v>0.01682745320942556</v>
       </c>
       <c r="K30" s="4" t="b">
         <v>0</v>
@@ -2437,12 +2502,14 @@
         <v>-63</v>
       </c>
       <c r="M30" s="4">
-        <v>-0.10424894884088287</v>
+        <v>-0.1070680161320916</v>
       </c>
       <c r="N30" s="4">
-        <v>54.375</v>
-      </c>
-      <c r="O30" s="4"/>
+        <v>53.39999999999999</v>
+      </c>
+      <c r="O30" s="4">
+        <v>-0.6</v>
+      </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
@@ -2452,7 +2519,7 @@
         <v>-0.74</v>
       </c>
       <c r="C31" s="4">
-        <v>27.083333333333332</v>
+        <v>26</v>
       </c>
       <c r="D31" s="4">
         <v>36.608108108108105</v>
@@ -2461,19 +2528,19 @@
         <v>1.22</v>
       </c>
       <c r="F31" s="4">
-        <v>-0.012600547693719072</v>
+        <v>-0.020539826332099193</v>
       </c>
       <c r="G31" s="4">
         <v>1.05</v>
       </c>
       <c r="H31" s="4">
-        <v>63.53</v>
+        <v>62.82</v>
       </c>
       <c r="I31" s="4">
-        <v>-1.24</v>
+        <v>-1.92</v>
       </c>
       <c r="J31" s="4">
-        <v>0.004536771046019471</v>
+        <v>0.004328291007456379</v>
       </c>
       <c r="K31" s="4" t="b">
         <v>0</v>
@@ -2482,12 +2549,14 @@
         <v>93</v>
       </c>
       <c r="M31" s="4">
-        <v>-0.011279815381201486</v>
+        <v>-0.01929600363231887</v>
       </c>
       <c r="N31" s="4">
-        <v>50.833333333333336</v>
-      </c>
-      <c r="O31" s="4"/>
+        <v>50</v>
+      </c>
+      <c r="O31" s="4">
+        <v>-0.8</v>
+      </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
@@ -2497,7 +2566,7 @@
         <v>-0.18</v>
       </c>
       <c r="C32" s="4">
-        <v>35.41666666666667</v>
+        <v>34</v>
       </c>
       <c r="D32" s="4">
         <v>105.33333333333334</v>
@@ -2506,19 +2575,19 @@
         <v>-4.72</v>
       </c>
       <c r="F32" s="4">
-        <v>0.1381086728940456</v>
+        <v>0.13313544243322997</v>
       </c>
       <c r="G32" s="4">
         <v>1.36</v>
       </c>
       <c r="H32" s="4">
-        <v>75</v>
+        <v>74.22</v>
       </c>
       <c r="I32" s="4">
-        <v>13.25</v>
+        <v>12.57</v>
       </c>
       <c r="J32" s="4">
-        <v>0.02243554574533957</v>
+        <v>0.022292434755870626</v>
       </c>
       <c r="K32" s="4" t="b">
         <v>0</v>
@@ -2527,12 +2596,14 @@
         <v>-11</v>
       </c>
       <c r="M32" s="4">
-        <v>0.14761794554417218</v>
+        <v>0.14209096587164827</v>
       </c>
       <c r="N32" s="4">
-        <v>68.54166666666666</v>
-      </c>
-      <c r="O32" s="4"/>
+        <v>68.39999999999999</v>
+      </c>
+      <c r="O32" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
@@ -2542,7 +2613,7 @@
         <v>-4.08</v>
       </c>
       <c r="C33" s="1">
-        <v>6.25</v>
+        <v>6</v>
       </c>
       <c r="D33" s="1">
         <v>14.372549019607844</v>
@@ -2551,19 +2622,19 @@
         <v>13.14</v>
       </c>
       <c r="F33" s="1">
-        <v>0.0749569552980534</v>
+        <v>0.0794475694006667</v>
       </c>
       <c r="G33" s="1">
         <v>0</v>
       </c>
       <c r="H33" s="1">
-        <v>62.34</v>
+        <v>61.98</v>
       </c>
       <c r="I33" s="1">
-        <v>-7.11</v>
+        <v>-7.32</v>
       </c>
       <c r="J33" s="1">
-        <v>0.04408771991281714</v>
+        <v>0.044189170511191735</v>
       </c>
       <c r="K33" s="1" t="b">
         <v>0</v>
@@ -2572,12 +2643,14 @@
         <v>20</v>
       </c>
       <c r="M33" s="1">
-        <v>0.04854230904770174</v>
+        <v>0.05457111540506032</v>
       </c>
       <c r="N33" s="1">
-        <v>48.333333333333336</v>
-      </c>
-      <c r="O33" s="1"/>
+        <v>48.2</v>
+      </c>
+      <c r="O33" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
@@ -2587,7 +2660,7 @@
         <v>-0.48</v>
       </c>
       <c r="C34" s="1">
-        <v>29.166666666666668</v>
+        <v>28.000000000000004</v>
       </c>
       <c r="D34" s="1">
         <v>86.47916666666667</v>
@@ -2596,19 +2669,19 @@
         <v>-1.38</v>
       </c>
       <c r="F34" s="1">
-        <v>-0.27528167947146365</v>
+        <v>-0.28006059158760466</v>
       </c>
       <c r="G34" s="1">
         <v>0.91</v>
       </c>
       <c r="H34" s="1">
-        <v>56.83</v>
+        <v>55.97</v>
       </c>
       <c r="I34" s="1">
-        <v>-32.31</v>
+        <v>-32.6</v>
       </c>
       <c r="J34" s="1">
-        <v>-0.010654340748782016</v>
+        <v>-0.010815020008760702</v>
       </c>
       <c r="K34" s="1" t="b">
         <v>0</v>
@@ -2617,12 +2690,14 @@
         <v>3</v>
       </c>
       <c r="M34" s="1">
-        <v>-0.27765899763399526</v>
+        <v>-0.2822994724472092</v>
       </c>
       <c r="N34" s="1">
-        <v>42.708333333333336</v>
-      </c>
-      <c r="O34" s="1"/>
+        <v>42.2</v>
+      </c>
+      <c r="O34" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
@@ -2632,7 +2707,7 @@
         <v>3.52</v>
       </c>
       <c r="C35" s="1">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D35" s="1">
         <v>1.1988636363636365</v>
@@ -2641,19 +2716,19 @@
         <v>0.4</v>
       </c>
       <c r="F35" s="1">
-        <v>0.04837859130682097</v>
+        <v>0.04342695466623904</v>
       </c>
       <c r="G35" s="1">
         <v>0.38</v>
       </c>
       <c r="H35" s="1">
-        <v>43.38</v>
+        <v>41.35</v>
       </c>
       <c r="I35" s="1">
-        <v>4.13</v>
+        <v>3.54</v>
       </c>
       <c r="J35" s="1">
-        <v>0.007072343136519611</v>
+        <v>0.006968933733247495</v>
       </c>
       <c r="K35" s="1" t="b">
         <v>0</v>
@@ -2662,12 +2737,14 @@
         <v>28</v>
       </c>
       <c r="M35" s="1">
-        <v>0.03200151063160295</v>
+        <v>0.028003553188963082</v>
       </c>
       <c r="N35" s="1">
-        <v>47.083333333333336</v>
-      </c>
-      <c r="O35" s="1"/>
+        <v>46.599999999999994</v>
+      </c>
+      <c r="O35" s="1">
+        <v>-0.4</v>
+      </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
@@ -2677,7 +2754,7 @@
         <v>-0.02</v>
       </c>
       <c r="C36" s="4">
-        <v>39.58333333333333</v>
+        <v>38</v>
       </c>
       <c r="D36" s="4">
         <v>1215</v>
@@ -2686,19 +2763,19 @@
         <v>5.89</v>
       </c>
       <c r="F36" s="4">
-        <v>-0.048296298967170956</v>
+        <v>-0.06133460065223531</v>
       </c>
       <c r="G36" s="4">
         <v>1.38</v>
       </c>
       <c r="H36" s="4">
-        <v>57.58</v>
+        <v>55.75</v>
       </c>
       <c r="I36" s="4">
-        <v>-8.94</v>
+        <v>-10.45</v>
       </c>
       <c r="J36" s="4">
-        <v>0.017724750523772582</v>
+        <v>0.01739455982384013</v>
       </c>
       <c r="K36" s="4" t="b">
         <v>1</v>
@@ -2707,12 +2784,14 @@
         <v>31</v>
       </c>
       <c r="M36" s="4">
-        <v>-0.038258733392037336</v>
+        <v>-0.05188154813390489</v>
       </c>
       <c r="N36" s="4">
-        <v>62.08333333333333</v>
-      </c>
-      <c r="O36" s="4"/>
+        <v>61</v>
+      </c>
+      <c r="O36" s="4">
+        <v>-0.6</v>
+      </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
@@ -2722,7 +2801,7 @@
         <v>0.94</v>
       </c>
       <c r="C37" s="4">
-        <v>52.083333333333336</v>
+        <v>50</v>
       </c>
       <c r="D37" s="4">
         <v>31.03191489361702</v>
@@ -2731,19 +2810,19 @@
         <v>-0.72</v>
       </c>
       <c r="F37" s="4">
-        <v>-0.15913082613344948</v>
+        <v>-0.16146366087670874</v>
       </c>
       <c r="G37" s="4">
         <v>2.78</v>
       </c>
       <c r="H37" s="4">
-        <v>62.2</v>
+        <v>60.56</v>
       </c>
       <c r="I37" s="4">
-        <v>-5.66</v>
+        <v>-6.56</v>
       </c>
       <c r="J37" s="4">
-        <v>0.010883126809017934</v>
+        <v>0.010724473081475675</v>
       </c>
       <c r="K37" s="4" t="b">
         <v>0</v>
@@ -2752,12 +2831,14 @@
         <v>134</v>
       </c>
       <c r="M37" s="4">
-        <v>-0.11211275580782354</v>
+        <v>-0.1171835727645294</v>
       </c>
       <c r="N37" s="4">
-        <v>57.70833333333334</v>
-      </c>
-      <c r="O37" s="4"/>
+        <v>56.6</v>
+      </c>
+      <c r="O37" s="4">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
@@ -2767,7 +2848,7 @@
         <v>3.41</v>
       </c>
       <c r="C38" s="2">
-        <v>72.91666666666666</v>
+        <v>70</v>
       </c>
       <c r="D38" s="2">
         <v>8.926686217008797</v>
@@ -2776,19 +2857,19 @@
         <v>-1.19</v>
       </c>
       <c r="F38" s="2">
-        <v>0.7532144984691509</v>
+        <v>0.7522690315963407</v>
       </c>
       <c r="G38" s="2">
         <v>2.08</v>
       </c>
       <c r="H38" s="2">
-        <v>68.52</v>
+        <v>68.69</v>
       </c>
       <c r="I38" s="2">
-        <v>72.37</v>
+        <v>72.68</v>
       </c>
       <c r="J38" s="2">
-        <v>0.04794036718733313</v>
+        <v>0.04788231480104818</v>
       </c>
       <c r="K38" s="2" t="b">
         <v>0</v>
@@ -2797,12 +2878,14 @@
         <v>234</v>
       </c>
       <c r="M38" s="2">
-        <v>0.7817423164195307</v>
+        <v>0.7791356019115956</v>
       </c>
       <c r="N38" s="2">
-        <v>73.33333333333333</v>
-      </c>
-      <c r="O38" s="2"/>
+        <v>73.4</v>
+      </c>
+      <c r="O38" s="2">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
@@ -2812,7 +2895,7 @@
         <v>-0.38</v>
       </c>
       <c r="C39" s="2">
-        <v>31.25</v>
+        <v>30</v>
       </c>
       <c r="D39" s="2">
         <v>325.07894736842104</v>
@@ -2821,19 +2904,19 @@
         <v>3.31</v>
       </c>
       <c r="F39" s="2">
-        <v>0.4244393059541854</v>
+        <v>0.4187112698573938</v>
       </c>
       <c r="G39" s="2">
         <v>3.47</v>
       </c>
       <c r="H39" s="2">
-        <v>73.96</v>
+        <v>73.66</v>
       </c>
       <c r="I39" s="2">
-        <v>120.27</v>
+        <v>118.84</v>
       </c>
       <c r="J39" s="2">
-        <v>0.04318873970246332</v>
+        <v>0.04296879405972401</v>
       </c>
       <c r="K39" s="2" t="b">
         <v>0</v>
@@ -2842,12 +2925,14 @@
         <v>211</v>
       </c>
       <c r="M39" s="2">
-        <v>0.489683482192554</v>
+        <v>0.48015611122654156</v>
       </c>
       <c r="N39" s="2">
-        <v>74.58333333333333</v>
-      </c>
-      <c r="O39" s="2"/>
+        <v>74.39999999999999</v>
+      </c>
+      <c r="O39" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
@@ -2857,7 +2942,7 @@
         <v>-0.32</v>
       </c>
       <c r="C40" s="1">
-        <v>33.33333333333333</v>
+        <v>32</v>
       </c>
       <c r="D40" s="1">
         <v>228.28125</v>
@@ -2866,19 +2951,19 @@
         <v>3.34</v>
       </c>
       <c r="F40" s="1">
-        <v>-0.20047544049218177</v>
+        <v>-0.2007982514277325</v>
       </c>
       <c r="G40" s="1">
         <v>1.68</v>
       </c>
       <c r="H40" s="1">
-        <v>45.97</v>
+        <v>43.52</v>
       </c>
       <c r="I40" s="1">
-        <v>-3.8</v>
+        <v>-5.97</v>
       </c>
       <c r="J40" s="1">
-        <v>-0.01178367415794677</v>
+        <v>-0.011845693448925713</v>
       </c>
       <c r="K40" s="1" t="b">
         <v>0</v>
@@ -2887,12 +2972,14 @@
         <v>11</v>
       </c>
       <c r="M40" s="1">
-        <v>-0.18251348104194265</v>
+        <v>-0.18388226271072017</v>
       </c>
       <c r="N40" s="1">
-        <v>46.041666666666664</v>
-      </c>
-      <c r="O40" s="1"/>
+        <v>45.400000000000006</v>
+      </c>
+      <c r="O40" s="1">
+        <v>-0.2</v>
+      </c>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
@@ -2902,7 +2989,7 @@
         <v>-2.92</v>
       </c>
       <c r="C41" s="3">
-        <v>14.583333333333334</v>
+        <v>14.000000000000002</v>
       </c>
       <c r="D41" s="3">
         <v>-23.77054794520548</v>
@@ -2911,19 +2998,19 @@
         <v>16.88</v>
       </c>
       <c r="F41" s="3">
-        <v>0.1549289351552015</v>
+        <v>0.16678258034043136</v>
       </c>
       <c r="G41" s="3">
         <v>1.95</v>
       </c>
       <c r="H41" s="3">
-        <v>70.81</v>
+        <v>71.02</v>
       </c>
       <c r="I41" s="3">
-        <v>31.67</v>
+        <v>32.21</v>
       </c>
       <c r="J41" s="3">
-        <v>-0.012185710379580567</v>
+        <v>-0.012003514083289334</v>
       </c>
       <c r="K41" s="3" t="b">
         <v>1</v>
@@ -2932,12 +3019,14 @@
         <v>83</v>
       </c>
       <c r="M41" s="3">
-        <v>0.18002284909303556</v>
+        <v>0.1904152116362574</v>
       </c>
       <c r="N41" s="3">
-        <v>25.625</v>
-      </c>
-      <c r="O41" s="3"/>
+        <v>25.800000000000004</v>
+      </c>
+      <c r="O41" s="3">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
@@ -2947,7 +3036,7 @@
         <v>4.88</v>
       </c>
       <c r="C42" s="4">
-        <v>77.08333333333334</v>
+        <v>74</v>
       </c>
       <c r="D42" s="4">
         <v>6.178278688524591</v>
@@ -2956,19 +3045,19 @@
         <v>-0.19</v>
       </c>
       <c r="F42" s="4">
-        <v>0.11548747115132582</v>
+        <v>0.11162120817244162</v>
       </c>
       <c r="G42" s="4">
         <v>1.85</v>
       </c>
       <c r="H42" s="4">
-        <v>61.04</v>
+        <v>59.95</v>
       </c>
       <c r="I42" s="4">
-        <v>56.14</v>
+        <v>55.15</v>
       </c>
       <c r="J42" s="4">
-        <v>0.017137808683028773</v>
+        <v>0.01700763705192206</v>
       </c>
       <c r="K42" s="4" t="b">
         <v>0</v>
@@ -2977,12 +3066,14 @@
         <v>300</v>
       </c>
       <c r="M42" s="4">
-        <v>0.13793992046412473</v>
+        <v>0.13276619406870704</v>
       </c>
       <c r="N42" s="4">
-        <v>64.58333333333334</v>
-      </c>
-      <c r="O42" s="4"/>
+        <v>64.39999999999999</v>
+      </c>
+      <c r="O42" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
@@ -2992,7 +3083,7 @@
         <v>-0.76</v>
       </c>
       <c r="C43" s="1">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D43" s="1">
         <v>13.236842105263158</v>
@@ -3001,19 +3092,19 @@
         <v>7.72</v>
       </c>
       <c r="F43" s="1">
-        <v>-0.38174499445726107</v>
+        <v>-0.3845729028929534</v>
       </c>
       <c r="G43" s="1">
         <v>2.61</v>
       </c>
       <c r="H43" s="1">
-        <v>56.14</v>
+        <v>54.93</v>
       </c>
       <c r="I43" s="1">
-        <v>-31.84</v>
+        <v>-32.36</v>
       </c>
       <c r="J43" s="1">
-        <v>-0.01874205106563216</v>
+        <v>-0.01893993006080149</v>
       </c>
       <c r="K43" s="1" t="b">
         <v>1</v>
@@ -3022,12 +3113,14 @@
         <v>64</v>
       </c>
       <c r="M43" s="1">
-        <v>-0.3392174139941949</v>
+        <v>-0.3445218119600272</v>
       </c>
       <c r="N43" s="1">
-        <v>31.666666666666664</v>
-      </c>
-      <c r="O43" s="1"/>
+        <v>31.599999999999998</v>
+      </c>
+      <c r="O43" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
@@ -3037,7 +3130,7 @@
         <v>0.54</v>
       </c>
       <c r="C44" s="4">
-        <v>47.91666666666667</v>
+        <v>46</v>
       </c>
       <c r="D44" s="4">
         <v>41.629629629629626</v>
@@ -3052,10 +3145,10 @@
         <v>1.41</v>
       </c>
       <c r="H44" s="4">
-        <v>63.64</v>
+        <v>62.96</v>
       </c>
       <c r="I44" s="4">
-        <v>-3.37</v>
+        <v>-3.92</v>
       </c>
       <c r="J44" s="4">
         <v>0</v>
@@ -3070,9 +3163,11 @@
         <v>0</v>
       </c>
       <c r="N44" s="4">
-        <v>55.83333333333333</v>
-      </c>
-      <c r="O44" s="4"/>
+        <v>55.199999999999996</v>
+      </c>
+      <c r="O44" s="4">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
@@ -3082,7 +3177,7 @@
         <v>0.95</v>
       </c>
       <c r="C45" s="2">
-        <v>54.166666666666664</v>
+        <v>52</v>
       </c>
       <c r="D45" s="2">
         <v>14.789473684210527</v>
@@ -3091,7 +3186,7 @@
         <v>2.01</v>
       </c>
       <c r="F45" s="2">
-        <v>0.31067145981052635</v>
+        <v>0.31197289663961014</v>
       </c>
       <c r="G45" s="2">
         <v>0.8</v>
@@ -3103,7 +3198,7 @@
         <v>36.93</v>
       </c>
       <c r="J45" s="2">
-        <v>0.026608906205351935</v>
+        <v>0.026610161244824973</v>
       </c>
       <c r="K45" s="2" t="b">
         <v>0</v>
@@ -3112,192 +3207,296 @@
         <v>11</v>
       </c>
       <c r="M45" s="2">
-        <v>0.305388530560456</v>
+        <v>0.30699760584048885</v>
       </c>
       <c r="N45" s="2">
-        <v>72.08333333333333</v>
-      </c>
-      <c r="O45" s="2"/>
+        <v>72</v>
+      </c>
+      <c r="O45" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
         <v>59</v>
       </c>
       <c r="B46" s="4">
-        <v>1.94</v>
+        <v>6.11</v>
       </c>
       <c r="C46" s="4">
-        <v>64.58333333333334</v>
+        <v>82</v>
       </c>
       <c r="D46" s="4">
-        <v>1.1030927835051547</v>
+        <v>0.6121112929623567</v>
       </c>
       <c r="E46" s="4">
-        <v>0.54</v>
+        <v>-2.35</v>
       </c>
       <c r="F46" s="4">
-        <v>0.04356416389380155</v>
+        <v>0.2268171383624703</v>
       </c>
       <c r="G46" s="4">
-        <v>0.74</v>
+        <v>0.87</v>
       </c>
       <c r="H46" s="4">
-        <v>70.05</v>
+        <v>70.66</v>
       </c>
       <c r="I46" s="4">
-        <v>22.64</v>
+        <v>21.83</v>
       </c>
       <c r="J46" s="4">
-        <v>0.008830482815401951</v>
+        <v>0.014065204785143063</v>
       </c>
       <c r="K46" s="4" t="b">
         <v>0</v>
       </c>
       <c r="L46" s="4">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="M46" s="4">
-        <v>0.03669635586871012</v>
+        <v>0.2235831993430415</v>
       </c>
       <c r="N46" s="4">
-        <v>52.91666666666667</v>
-      </c>
-      <c r="O46" s="4"/>
+        <v>58.8</v>
+      </c>
+      <c r="O46" s="4">
+        <v>-0.4</v>
+      </c>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
         <v>60</v>
       </c>
       <c r="B47" s="4">
+        <v>1.94</v>
+      </c>
+      <c r="C47" s="4">
+        <v>62</v>
+      </c>
+      <c r="D47" s="4">
+        <v>1.1030927835051547</v>
+      </c>
+      <c r="E47" s="4">
+        <v>0.54</v>
+      </c>
+      <c r="F47" s="4">
+        <v>0.04217143679343387</v>
+      </c>
+      <c r="G47" s="4">
+        <v>0.74</v>
+      </c>
+      <c r="H47" s="4">
+        <v>69.66</v>
+      </c>
+      <c r="I47" s="4">
+        <v>22.32</v>
+      </c>
+      <c r="J47" s="4">
+        <v>0.008776966289988017</v>
+      </c>
+      <c r="K47" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L47" s="4">
+        <v>23</v>
+      </c>
+      <c r="M47" s="4">
+        <v>0.0357035587545762</v>
+      </c>
+      <c r="N47" s="4">
+        <v>53.2</v>
+      </c>
+      <c r="O47" s="4">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A48" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B48" s="4">
         <v>2.84</v>
       </c>
-      <c r="C47" s="4">
-        <v>68.75</v>
-      </c>
-      <c r="D47" s="4">
+      <c r="C48" s="4">
+        <v>66</v>
+      </c>
+      <c r="D48" s="4">
         <v>2.0880281690140845</v>
       </c>
-      <c r="E47" s="4">
+      <c r="E48" s="4">
         <v>0.95</v>
       </c>
-      <c r="F47" s="4">
-        <v>0.18093353280757316</v>
-      </c>
-      <c r="G47" s="4">
+      <c r="F48" s="4">
+        <v>0.1842640237296823</v>
+      </c>
+      <c r="G48" s="4">
         <v>0.88</v>
       </c>
-      <c r="H47" s="4">
-        <v>72.82</v>
-      </c>
-      <c r="I47" s="4">
-        <v>19.81</v>
-      </c>
-      <c r="J47" s="4">
-        <v>0.004465546501666247</v>
-      </c>
-      <c r="K47" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="L47" s="4">
+      <c r="H48" s="4">
+        <v>73.46</v>
+      </c>
+      <c r="I48" s="4">
+        <v>20.33</v>
+      </c>
+      <c r="J48" s="4">
+        <v>0.004501832495174733</v>
+      </c>
+      <c r="K48" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L48" s="4">
         <v>248</v>
       </c>
-      <c r="M47" s="4">
-        <v>0.17776377525753095</v>
-      </c>
-      <c r="N47" s="4">
-        <v>56.666666666666664</v>
-      </c>
-      <c r="O47" s="4"/>
-    </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A48" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B48" s="2">
-        <v>8.72</v>
-      </c>
-      <c r="C48" s="2">
-        <v>91.66666666666666</v>
-      </c>
-      <c r="D48" s="2">
-        <v>0.8061926605504586</v>
-      </c>
-      <c r="E48" s="2">
-        <v>6.35</v>
-      </c>
-      <c r="F48" s="2">
-        <v>0.873048360184754</v>
-      </c>
-      <c r="G48" s="2">
-        <v>0.96</v>
-      </c>
-      <c r="H48" s="2">
-        <v>72.13</v>
-      </c>
-      <c r="I48" s="2">
-        <v>52.56</v>
-      </c>
-      <c r="J48" s="2">
-        <v>0.05270914285945323</v>
-      </c>
-      <c r="K48" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="L48" s="2">
-        <v>115</v>
-      </c>
-      <c r="M48" s="2">
-        <v>0.8719917743347398</v>
-      </c>
-      <c r="N48" s="2">
-        <v>71.875</v>
-      </c>
-      <c r="O48" s="2"/>
+      <c r="M48" s="4">
+        <v>0.18127884925020954</v>
+      </c>
+      <c r="N48" s="4">
+        <v>57.400000000000006</v>
+      </c>
+      <c r="O48" s="4">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
         <v>62</v>
       </c>
       <c r="B49" s="4">
+        <v>20.88</v>
+      </c>
+      <c r="C49" s="4">
+        <v>98</v>
+      </c>
+      <c r="D49" s="4">
+        <v>-0.7054597701149425</v>
+      </c>
+      <c r="E49" s="4">
+        <v>-0.3</v>
+      </c>
+      <c r="F49" s="4">
+        <v>0.002233231868567248</v>
+      </c>
+      <c r="G49" s="4">
+        <v>1.05</v>
+      </c>
+      <c r="H49" s="4">
+        <v>63.33</v>
+      </c>
+      <c r="I49" s="4">
+        <v>3.52</v>
+      </c>
+      <c r="J49" s="4">
+        <v>-0.0010066168117376939</v>
+      </c>
+      <c r="K49" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L49" s="4">
+        <v>318</v>
+      </c>
+      <c r="M49" s="4">
+        <v>0.0034770545683475707</v>
+      </c>
+      <c r="N49" s="4">
+        <v>50.4</v>
+      </c>
+      <c r="O49" s="4">
+        <v>-0.2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B50" s="2">
+        <v>8.72</v>
+      </c>
+      <c r="C50" s="2">
+        <v>90</v>
+      </c>
+      <c r="D50" s="2">
+        <v>0.8061926605504586</v>
+      </c>
+      <c r="E50" s="2">
+        <v>6.35</v>
+      </c>
+      <c r="F50" s="2">
+        <v>0.8831681458235491</v>
+      </c>
+      <c r="G50" s="2">
+        <v>0.96</v>
+      </c>
+      <c r="H50" s="2">
+        <v>72.55</v>
+      </c>
+      <c r="I50" s="2">
+        <v>53.49</v>
+      </c>
+      <c r="J50" s="2">
+        <v>0.05283941505704367</v>
+      </c>
+      <c r="K50" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L50" s="2">
+        <v>115</v>
+      </c>
+      <c r="M50" s="2">
+        <v>0.8821730876637248</v>
+      </c>
+      <c r="N50" s="2">
+        <v>72.39999999999999</v>
+      </c>
+      <c r="O50" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A51" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B51" s="4">
         <v>10.45</v>
       </c>
-      <c r="C49" s="4">
-        <v>95.83333333333334</v>
-      </c>
-      <c r="D49" s="4">
+      <c r="C51" s="4">
+        <v>94</v>
+      </c>
+      <c r="D51" s="4">
         <v>0.4545454545454546</v>
       </c>
-      <c r="E49" s="4">
+      <c r="E51" s="4">
         <v>-0.36</v>
       </c>
-      <c r="F49" s="4">
-        <v>0.177434564940825</v>
-      </c>
-      <c r="G49" s="4">
+      <c r="F51" s="4">
+        <v>0.1777696584470837</v>
+      </c>
+      <c r="G51" s="4">
         <v>1.2</v>
       </c>
-      <c r="H49" s="4">
-        <v>68.18</v>
-      </c>
-      <c r="I49" s="4">
-        <v>14.22</v>
-      </c>
-      <c r="J49" s="4">
-        <v>0.010713778808231215</v>
-      </c>
-      <c r="K49" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="L49" s="4">
+      <c r="H51" s="4">
+        <v>68.11</v>
+      </c>
+      <c r="I51" s="4">
+        <v>14.17</v>
+      </c>
+      <c r="J51" s="4">
+        <v>0.0106861724220283</v>
+      </c>
+      <c r="K51" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L51" s="4">
         <v>133</v>
       </c>
-      <c r="M49" s="4">
-        <v>0.18271749419089534</v>
-      </c>
-      <c r="N49" s="4">
-        <v>57.91666666666667</v>
-      </c>
-      <c r="O49" s="4"/>
+      <c r="M51" s="4">
+        <v>0.182744949246205</v>
+      </c>
+      <c r="N51" s="4">
+        <v>57.80000000000001</v>
+      </c>
+      <c r="O51" s="4">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3307,15 +3506,15 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:B51"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -3323,7 +3522,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>44.375</v>
+        <v>43.800000000000004</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -3331,7 +3530,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>77.29166666666666</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3339,7 +3538,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>24.583333333333332</v>
+        <v>24.6</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -3347,7 +3546,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>51.66666666666667</v>
+        <v>50.800000000000004</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -3355,7 +3554,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>49.375</v>
+        <v>49.6</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -3363,7 +3562,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>61.875</v>
+        <v>61</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -3371,7 +3570,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>62.708333333333336</v>
+        <v>63.599999999999994</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -3379,7 +3578,7 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>52.29166666666667</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -3387,7 +3586,7 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>46.875</v>
+        <v>48.4</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -3395,7 +3594,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>22.916666666666668</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -3403,7 +3602,7 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>40.208333333333336</v>
+        <v>40.2</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -3411,7 +3610,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>75.625</v>
+        <v>75.2</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -3419,7 +3618,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>49.791666666666664</v>
+        <v>50.199999999999996</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -3427,7 +3626,7 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>36.25</v>
+        <v>36.400000000000006</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -3435,7 +3634,7 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>63.125</v>
+        <v>62.6</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -3443,7 +3642,7 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>49.166666666666664</v>
+        <v>48.99999999999999</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -3451,7 +3650,7 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>53.54166666666667</v>
+        <v>54.2</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -3459,7 +3658,7 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>43.958333333333336</v>
+        <v>42.8</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -3467,7 +3666,7 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>27.916666666666664</v>
+        <v>27.400000000000002</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -3475,7 +3674,7 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>25.625</v>
+        <v>25.799999999999994</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -3483,7 +3682,7 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>46.04166666666667</v>
+        <v>46.400000000000006</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -3491,7 +3690,7 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>24.16666666666667</v>
+        <v>24.599999999999998</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -3499,7 +3698,7 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>23.125000000000004</v>
+        <v>23.200000000000003</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -3507,7 +3706,7 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>51.87499999999999</v>
+        <v>51</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -3515,7 +3714,7 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>61.875</v>
+        <v>60.400000000000006</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -3523,7 +3722,7 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>75.62500000000001</v>
+        <v>75.2</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -3531,7 +3730,7 @@
         <v>27</v>
       </c>
       <c r="B28">
-        <v>43.74999999999999</v>
+        <v>43.800000000000004</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -3539,7 +3738,7 @@
         <v>28</v>
       </c>
       <c r="B29">
-        <v>49.583333333333336</v>
+        <v>50.4</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -3547,7 +3746,7 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>54.375</v>
+        <v>53.39999999999999</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
@@ -3555,7 +3754,7 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>50.833333333333336</v>
+        <v>50</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
@@ -3563,7 +3762,7 @@
         <v>31</v>
       </c>
       <c r="B32">
-        <v>68.54166666666666</v>
+        <v>68.39999999999999</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
@@ -3571,7 +3770,7 @@
         <v>32</v>
       </c>
       <c r="B33">
-        <v>48.333333333333336</v>
+        <v>48.2</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
@@ -3579,7 +3778,7 @@
         <v>33</v>
       </c>
       <c r="B34">
-        <v>42.708333333333336</v>
+        <v>42.2</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
@@ -3587,7 +3786,7 @@
         <v>34</v>
       </c>
       <c r="B35">
-        <v>47.083333333333336</v>
+        <v>46.599999999999994</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
@@ -3595,7 +3794,7 @@
         <v>35</v>
       </c>
       <c r="B36">
-        <v>62.08333333333333</v>
+        <v>61</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
@@ -3603,7 +3802,7 @@
         <v>36</v>
       </c>
       <c r="B37">
-        <v>57.70833333333334</v>
+        <v>56.6</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
@@ -3611,7 +3810,7 @@
         <v>37</v>
       </c>
       <c r="B38">
-        <v>73.33333333333333</v>
+        <v>73.4</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
@@ -3619,7 +3818,7 @@
         <v>38</v>
       </c>
       <c r="B39">
-        <v>74.58333333333333</v>
+        <v>74.39999999999999</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
@@ -3627,7 +3826,7 @@
         <v>39</v>
       </c>
       <c r="B40">
-        <v>46.041666666666664</v>
+        <v>45.400000000000006</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
@@ -3635,7 +3834,7 @@
         <v>40</v>
       </c>
       <c r="B41">
-        <v>25.625</v>
+        <v>25.800000000000004</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
@@ -3643,7 +3842,7 @@
         <v>41</v>
       </c>
       <c r="B42">
-        <v>64.58333333333334</v>
+        <v>64.39999999999999</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
@@ -3651,7 +3850,7 @@
         <v>42</v>
       </c>
       <c r="B43">
-        <v>31.666666666666664</v>
+        <v>31.599999999999998</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
@@ -3659,7 +3858,7 @@
         <v>43</v>
       </c>
       <c r="B44">
-        <v>55.83333333333333</v>
+        <v>55.199999999999996</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
@@ -3667,7 +3866,7 @@
         <v>58</v>
       </c>
       <c r="B45">
-        <v>72.08333333333333</v>
+        <v>72</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
@@ -3675,7 +3874,7 @@
         <v>59</v>
       </c>
       <c r="B46">
-        <v>52.91666666666667</v>
+        <v>58.8</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
@@ -3683,7 +3882,7 @@
         <v>60</v>
       </c>
       <c r="B47">
-        <v>56.666666666666664</v>
+        <v>53.2</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
@@ -3691,7 +3890,7 @@
         <v>61</v>
       </c>
       <c r="B48">
-        <v>71.875</v>
+        <v>57.400000000000006</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
@@ -3699,7 +3898,23 @@
         <v>62</v>
       </c>
       <c r="B49">
-        <v>57.91666666666667</v>
+        <v>50.4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>63</v>
+      </c>
+      <c r="B50">
+        <v>72.39999999999999</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>64</v>
+      </c>
+      <c r="B51">
+        <v>57.80000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -3718,10 +3933,10 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -3729,10 +3944,10 @@
         <v>58</v>
       </c>
       <c r="C2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -3740,106 +3955,109 @@
         <v>59</v>
       </c>
       <c r="C3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="4" spans="3:4" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>60</v>
+      </c>
       <c r="C4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D6" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D8" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D11" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D12" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="14" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D14" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="15" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D15" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -3858,117 +4076,120 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="3" spans="3:4" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>62</v>
+      </c>
       <c r="C3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D8" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D9" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D10" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D11" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="12" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D12" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="13" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D13" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D14" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -3987,117 +4208,117 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D6" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="7" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D8" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D9" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="10" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D10" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="11" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D11" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="12" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D12" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="13" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D13" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D14" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -4116,128 +4337,128 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D4" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
     <row r="5" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D6" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D7" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D8" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D11" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D12" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="14" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D14" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="15" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D15" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -4253,16 +4474,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B1" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C1" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="D1" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -4270,213 +4491,213 @@
         <v>45</v>
       </c>
       <c r="B2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D2" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B3" t="s">
         <v>115</v>
       </c>
-      <c r="B3" t="s">
-        <v>112</v>
-      </c>
       <c r="C3" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="D3" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B4" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="C4" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D4" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B5" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C5" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="D5" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B6" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C6" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D6" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B7" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C7" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D7" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B8" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C8" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D8" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B9" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C9" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D9" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>132</v>
+      </c>
+      <c r="B10" t="s">
+        <v>133</v>
+      </c>
+      <c r="C10" t="s">
         <v>129</v>
       </c>
-      <c r="B10" t="s">
-        <v>130</v>
-      </c>
-      <c r="C10" t="s">
-        <v>126</v>
-      </c>
       <c r="D10" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B15" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C15" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D15" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B16" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C16" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D16" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated README.me to include changes related to Visualization for next-week Earnings-Proximity signal
</commit_message>
<xml_diff>
--- a/data/stocks.xlsx
+++ b/data/stocks.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="172">
   <si>
     <t>Ticker</t>
   </si>
@@ -192,34 +192,118 @@
     <t>Composite_Score</t>
   </si>
   <si>
+    <t>Earnings_Date</t>
+  </si>
+  <si>
     <t>Daily_Composite_Score_delta</t>
   </si>
   <si>
+    <t>2026-05-01</t>
+  </si>
+  <si>
+    <t>2026-05-05</t>
+  </si>
+  <si>
+    <t>2027-02-25</t>
+  </si>
+  <si>
+    <t>2026-04-22</t>
+  </si>
+  <si>
+    <t>2026-04-16</t>
+  </si>
+  <si>
+    <t>2026-04-21</t>
+  </si>
+  <si>
+    <t>2026-05-04</t>
+  </si>
+  <si>
+    <t>2026-05-06</t>
+  </si>
+  <si>
+    <t>2027-03-10</t>
+  </si>
+  <si>
+    <t>2027-03-04</t>
+  </si>
+  <si>
+    <t>2026-04-23</t>
+  </si>
+  <si>
+    <t>2027-02-26</t>
+  </si>
+  <si>
+    <t>2027-02-12</t>
+  </si>
+  <si>
+    <t>2026-04-30</t>
+  </si>
+  <si>
+    <t>2026-04-29</t>
+  </si>
+  <si>
+    <t>2026-04-28</t>
+  </si>
+  <si>
+    <t>2026-05-07</t>
+  </si>
+  <si>
+    <t>2027-03-02</t>
+  </si>
+  <si>
+    <t>2027-02-24</t>
+  </si>
+  <si>
+    <t>2027-03-03</t>
+  </si>
+  <si>
+    <t>2027-02-18</t>
+  </si>
+  <si>
+    <t>2027-02-05</t>
+  </si>
+  <si>
+    <t>2027-03-05</t>
+  </si>
+  <si>
+    <t>2026-03-30</t>
+  </si>
+  <si>
     <t>WSR</t>
   </si>
   <si>
     <t>BLX</t>
   </si>
   <si>
+    <t>2026-04-27</t>
+  </si>
+  <si>
     <t>MD</t>
   </si>
   <si>
     <t>CSCO</t>
   </si>
   <si>
+    <t>2026-05-13</t>
+  </si>
+  <si>
     <t>JPM</t>
   </si>
   <si>
+    <t>2026-04-14</t>
+  </si>
+  <si>
     <t>DELL</t>
   </si>
   <si>
     <t>ETN</t>
   </si>
   <si>
+    <t>2027-02-03</t>
+  </si>
+  <si>
     <t>_date_</t>
-  </si>
-  <si>
-    <t>2026-04-21</t>
   </si>
   <si>
     <t>Criteria</t>
@@ -1098,10 +1182,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O51"/>
+  <dimension ref="A1:P51"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1147,8 +1231,11 @@
       <c r="O1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -1165,19 +1252,19 @@
         <v>-0.01</v>
       </c>
       <c r="F2" s="1">
-        <v>0.11967941242595193</v>
+        <v>0.12180671561557217</v>
       </c>
       <c r="G2" s="1">
         <v>0.18</v>
       </c>
       <c r="H2" s="1">
-        <v>39.49</v>
+        <v>40.62</v>
       </c>
       <c r="I2" s="1">
-        <v>17.22</v>
+        <v>17.71</v>
       </c>
       <c r="J2" s="1">
-        <v>0.0023737785663199627</v>
+        <v>0.002404876827358358</v>
       </c>
       <c r="K2" s="1" t="b">
         <v>0</v>
@@ -1186,16 +1273,19 @@
         <v>364</v>
       </c>
       <c r="M2" s="1">
-        <v>0.09928072014955469</v>
+        <v>0.10271827784503751</v>
       </c>
       <c r="N2" s="1">
         <v>43.800000000000004</v>
       </c>
-      <c r="O2" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O2" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="P2" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -1212,19 +1302,19 @@
         <v>2.75</v>
       </c>
       <c r="F3" s="2">
-        <v>0.15876698515967727</v>
+        <v>0.16600313720455306</v>
       </c>
       <c r="G3" s="2">
         <v>2.1</v>
       </c>
       <c r="H3" s="2">
-        <v>78.96</v>
+        <v>79.17</v>
       </c>
       <c r="I3" s="2">
-        <v>38.57</v>
+        <v>39</v>
       </c>
       <c r="J3" s="2">
-        <v>0.02705586046568028</v>
+        <v>0.02714173332106283</v>
       </c>
       <c r="K3" s="2" t="b">
         <v>0</v>
@@ -1233,16 +1323,19 @@
         <v>375</v>
       </c>
       <c r="M3" s="2">
-        <v>0.18613108455484428</v>
+        <v>0.1916095781162459</v>
       </c>
       <c r="N3" s="2">
         <v>77</v>
       </c>
-      <c r="O3" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="P3" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -1259,19 +1352,19 @@
         <v>4.7</v>
       </c>
       <c r="F4" s="3">
-        <v>-0.3033310828445169</v>
+        <v>-0.3021002404144685</v>
       </c>
       <c r="G4" s="3">
         <v>1.18</v>
       </c>
       <c r="H4" s="3">
-        <v>48.95</v>
+        <v>48.5</v>
       </c>
       <c r="I4" s="3">
-        <v>-27.88</v>
+        <v>-28.15</v>
       </c>
       <c r="J4" s="3">
-        <v>-0.01446289471733941</v>
+        <v>-0.014479168880212931</v>
       </c>
       <c r="K4" s="3" t="b">
         <v>0</v>
@@ -1280,16 +1373,19 @@
         <v>50</v>
       </c>
       <c r="M4" s="3">
-        <v>-0.2988533211253077</v>
+        <v>-0.2979100955380096</v>
       </c>
       <c r="N4" s="3">
         <v>24.6</v>
       </c>
-      <c r="O4" s="3">
-        <v>-0.2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O4" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="P4" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
@@ -1306,19 +1402,19 @@
         <v>0.58</v>
       </c>
       <c r="F5" s="4">
-        <v>-0.12866175509386943</v>
+        <v>-0.12558638884002832</v>
       </c>
       <c r="G5" s="4">
         <v>1.85</v>
       </c>
       <c r="H5" s="4">
-        <v>54.34</v>
+        <v>54.26</v>
       </c>
       <c r="I5" s="4">
-        <v>-2.85</v>
+        <v>-2.89</v>
       </c>
       <c r="J5" s="4">
-        <v>-0.004851686507586286</v>
+        <v>-0.004849132590616535</v>
       </c>
       <c r="K5" s="4" t="b">
         <v>0</v>
@@ -1327,16 +1423,19 @@
         <v>312</v>
       </c>
       <c r="M5" s="4">
-        <v>-0.107516769197604</v>
+        <v>-0.10579959359008384</v>
       </c>
       <c r="N5" s="4">
-        <v>50.800000000000004</v>
-      </c>
-      <c r="O5" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="P5" s="4">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
@@ -1353,19 +1452,19 @@
         <v>-2.3</v>
       </c>
       <c r="F6" s="1">
-        <v>0.016374056771371423</v>
+        <v>0.014610241897089274</v>
       </c>
       <c r="G6" s="1">
         <v>1.6</v>
       </c>
       <c r="H6" s="1">
-        <v>41.41</v>
+        <v>40.85</v>
       </c>
       <c r="I6" s="1">
-        <v>-11.78</v>
+        <v>-12.14</v>
       </c>
       <c r="J6" s="1">
-        <v>0.02093980443525671</v>
+        <v>0.020856540179318855</v>
       </c>
       <c r="K6" s="1" t="b">
         <v>1</v>
@@ -1374,16 +1473,19 @@
         <v>139</v>
       </c>
       <c r="M6" s="1">
-        <v>0.03129992916873525</v>
+        <v>0.028577391485285375</v>
       </c>
       <c r="N6" s="1">
         <v>49.6</v>
       </c>
-      <c r="O6" s="1">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O6" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="P6" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
@@ -1400,19 +1502,19 @@
         <v>0.37</v>
       </c>
       <c r="F7" s="4">
-        <v>0.05439778654196077</v>
+        <v>0.06350472870759938</v>
       </c>
       <c r="G7" s="4">
         <v>2.29</v>
       </c>
       <c r="H7" s="4">
-        <v>67.39</v>
+        <v>68.37</v>
       </c>
       <c r="I7" s="4">
-        <v>9.64</v>
+        <v>9.94</v>
       </c>
       <c r="J7" s="4">
-        <v>0.011349021721240592</v>
+        <v>0.011455554262271794</v>
       </c>
       <c r="K7" s="4" t="b">
         <v>0</v>
@@ -1421,16 +1523,19 @@
         <v>434</v>
       </c>
       <c r="M7" s="4">
-        <v>0.086488412196293</v>
+        <v>0.09353410032222098</v>
       </c>
       <c r="N7" s="4">
+        <v>61.6</v>
+      </c>
+      <c r="O7" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="O7" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P7" s="4">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
@@ -1447,19 +1552,19 @@
         <v>0.43</v>
       </c>
       <c r="F8" s="4">
-        <v>0.018164476427022368</v>
+        <v>0.008845260747195292</v>
       </c>
       <c r="G8" s="4">
         <v>0.5</v>
       </c>
       <c r="H8" s="4">
-        <v>80.91</v>
+        <v>80.5</v>
       </c>
       <c r="I8" s="4">
-        <v>12.46</v>
+        <v>11.86</v>
       </c>
       <c r="J8" s="4">
-        <v>0.016899589420790572</v>
+        <v>0.0166585638880483</v>
       </c>
       <c r="K8" s="4" t="b">
         <v>0</v>
@@ -1468,16 +1573,19 @@
         <v>69</v>
       </c>
       <c r="M8" s="4">
-        <v>0.005726249429219177</v>
+        <v>-0.002794030576301454</v>
       </c>
       <c r="N8" s="4">
-        <v>63.599999999999994</v>
-      </c>
-      <c r="O8" s="4">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+        <v>62.99999999999999</v>
+      </c>
+      <c r="O8" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="P8" s="4">
+        <v>-0.6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>8</v>
       </c>
@@ -1494,19 +1602,19 @@
         <v>1.75</v>
       </c>
       <c r="F9" s="4">
-        <v>-0.17753265067641916</v>
+        <v>-0.17610346672917965</v>
       </c>
       <c r="G9" s="4">
         <v>1.6</v>
       </c>
       <c r="H9" s="4">
-        <v>52.36</v>
+        <v>52.06</v>
       </c>
       <c r="I9" s="4">
-        <v>-10.8</v>
+        <v>-10.99</v>
       </c>
       <c r="J9" s="4">
-        <v>0.001840994302116228</v>
+        <v>0.0018145549127325065</v>
       </c>
       <c r="K9" s="4" t="b">
         <v>0</v>
@@ -1515,16 +1623,19 @@
         <v>189</v>
       </c>
       <c r="M9" s="4">
-        <v>-0.16260677827905534</v>
+        <v>-0.16213631714098353</v>
       </c>
       <c r="N9" s="4">
         <v>52</v>
       </c>
-      <c r="O9" s="4">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O9" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="P9" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
@@ -1541,19 +1652,19 @@
         <v>0.88</v>
       </c>
       <c r="F10" s="1">
-        <v>-0.0974824182303593</v>
+        <v>-0.09625307728316178</v>
       </c>
       <c r="G10" s="1">
         <v>1.45</v>
       </c>
       <c r="H10" s="1">
-        <v>62.54</v>
+        <v>60.93</v>
       </c>
       <c r="I10" s="1">
-        <v>-5.04</v>
+        <v>-5.42</v>
       </c>
       <c r="J10" s="1">
-        <v>-0.0010052609990238268</v>
+        <v>-0.0010288684836846146</v>
       </c>
       <c r="K10" s="1" t="b">
         <v>0</v>
@@ -1562,16 +1673,19 @@
         <v>56</v>
       </c>
       <c r="M10" s="1">
-        <v>-0.08628801393233643</v>
+        <v>-0.0857777150920147</v>
       </c>
       <c r="N10" s="1">
-        <v>48.4</v>
-      </c>
-      <c r="O10" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+        <v>48.00000000000001</v>
+      </c>
+      <c r="O10" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="P10" s="1">
+        <v>-0.4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>10</v>
       </c>
@@ -1588,19 +1702,19 @@
         <v>10.01</v>
       </c>
       <c r="F11" s="3">
-        <v>-0.23513531228157736</v>
+        <v>-0.23176875548911732</v>
       </c>
       <c r="G11" s="3">
         <v>1.41</v>
       </c>
       <c r="H11" s="3">
-        <v>47.58</v>
+        <v>47.54</v>
       </c>
       <c r="I11" s="3">
-        <v>-1.59</v>
+        <v>-1.62</v>
       </c>
       <c r="J11" s="3">
-        <v>-0.012954170042827666</v>
+        <v>-0.012928365562974076</v>
       </c>
       <c r="K11" s="3" t="b">
         <v>1</v>
@@ -1609,16 +1723,19 @@
         <v>28</v>
       </c>
       <c r="M11" s="3">
-        <v>-0.22493596614337874</v>
+        <v>-0.22222453660385</v>
       </c>
       <c r="N11" s="3">
         <v>22</v>
       </c>
-      <c r="O11" s="3">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O11" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="P11" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
@@ -1635,19 +1752,19 @@
         <v>0.13</v>
       </c>
       <c r="F12" s="1">
-        <v>-0.13422061465190438</v>
+        <v>-0.13213082696331171</v>
       </c>
       <c r="G12" s="1">
         <v>0.63</v>
       </c>
       <c r="H12" s="1">
-        <v>54.75</v>
+        <v>54.73</v>
       </c>
       <c r="I12" s="1">
-        <v>-10.23</v>
+        <v>-10.24</v>
       </c>
       <c r="J12" s="1">
-        <v>-0.014605975442797736</v>
+        <v>-0.014581685102632282</v>
       </c>
       <c r="K12" s="1" t="b">
         <v>0</v>
@@ -1656,16 +1773,19 @@
         <v>10</v>
       </c>
       <c r="M12" s="1">
-        <v>-0.14342490263027874</v>
+        <v>-0.1407439025426993</v>
       </c>
       <c r="N12" s="1">
-        <v>40.2</v>
-      </c>
-      <c r="O12" s="1">
+        <v>40.400000000000006</v>
+      </c>
+      <c r="O12" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="P12" s="1">
         <v>0.2</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
@@ -1682,19 +1802,19 @@
         <v>6.17</v>
       </c>
       <c r="F13" s="2">
-        <v>0.31368202773667075</v>
+        <v>0.3190176654298967</v>
       </c>
       <c r="G13" s="2">
         <v>1.66</v>
       </c>
       <c r="H13" s="2">
-        <v>70.84</v>
+        <v>70.69</v>
       </c>
       <c r="I13" s="2">
-        <v>75.58</v>
+        <v>75.24</v>
       </c>
       <c r="J13" s="2">
-        <v>0.03695105739468107</v>
+        <v>0.03700547750273439</v>
       </c>
       <c r="K13" s="2" t="b">
         <v>0</v>
@@ -1703,16 +1823,19 @@
         <v>249</v>
       </c>
       <c r="M13" s="2">
-        <v>0.33010048737377096</v>
+        <v>0.3343815299769124</v>
       </c>
       <c r="N13" s="2">
         <v>75.2</v>
       </c>
-      <c r="O13" s="2">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O13" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="P13" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>13</v>
       </c>
@@ -1729,19 +1852,19 @@
         <v>2.52</v>
       </c>
       <c r="F14" s="4">
-        <v>0.15078708560651521</v>
+        <v>0.1580303166649597</v>
       </c>
       <c r="G14" s="4">
         <v>2.06</v>
       </c>
       <c r="H14" s="4">
-        <v>64.43</v>
+        <v>64.17</v>
       </c>
       <c r="I14" s="4">
-        <v>18.63</v>
+        <v>18.3</v>
       </c>
       <c r="J14" s="4">
-        <v>0.019829962781969673</v>
+        <v>0.019907417632426136</v>
       </c>
       <c r="K14" s="4" t="b">
         <v>0</v>
@@ -1750,16 +1873,19 @@
         <v>27</v>
       </c>
       <c r="M14" s="4">
-        <v>0.177156126841858</v>
+        <v>0.1827056142707728</v>
       </c>
       <c r="N14" s="4">
         <v>50.199999999999996</v>
       </c>
-      <c r="O14" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O14" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="P14" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
@@ -1776,19 +1902,19 @@
         <v>4.53</v>
       </c>
       <c r="F15" s="1">
-        <v>0.022359621987671996</v>
+        <v>0.019977546439078106</v>
       </c>
       <c r="G15" s="1">
         <v>1.84</v>
       </c>
       <c r="H15" s="1">
-        <v>62</v>
+        <v>60.37</v>
       </c>
       <c r="I15" s="1">
-        <v>0.41</v>
+        <v>-0.44</v>
       </c>
       <c r="J15" s="1">
-        <v>0.014271758714584973</v>
+        <v>0.014163228691075109</v>
       </c>
       <c r="K15" s="1" t="b">
         <v>0</v>
@@ -1797,16 +1923,19 @@
         <v>43</v>
       </c>
       <c r="M15" s="1">
-        <v>0.04325584334398136</v>
+        <v>0.039531555862552636</v>
       </c>
       <c r="N15" s="1">
-        <v>36.400000000000006</v>
-      </c>
-      <c r="O15" s="1">
-        <v>-0.4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+        <v>35.8</v>
+      </c>
+      <c r="O15" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="P15" s="1">
+        <v>-0.6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>15</v>
       </c>
@@ -1823,19 +1952,19 @@
         <v>11.11</v>
       </c>
       <c r="F16" s="4">
-        <v>-0.08136562225678619</v>
+        <v>-0.07720150533687542</v>
       </c>
       <c r="G16" s="4">
         <v>1.23</v>
       </c>
       <c r="H16" s="4">
-        <v>66.22</v>
+        <v>65.26</v>
       </c>
       <c r="I16" s="4">
-        <v>22.47</v>
+        <v>21.48</v>
       </c>
       <c r="J16" s="4">
-        <v>-0.003532875449604242</v>
+        <v>-0.0034812260130050077</v>
       </c>
       <c r="K16" s="4" t="b">
         <v>0</v>
@@ -1844,16 +1973,19 @@
         <v>32</v>
       </c>
       <c r="M16" s="4">
-        <v>-0.07564403783779672</v>
+        <v>-0.07184743132806692</v>
       </c>
       <c r="N16" s="4">
-        <v>62.6</v>
-      </c>
-      <c r="O16" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+        <v>62.2</v>
+      </c>
+      <c r="O16" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="P16" s="4">
+        <v>-0.4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>16</v>
       </c>
@@ -1870,19 +2002,19 @@
         <v>4.52</v>
       </c>
       <c r="F17" s="1">
-        <v>0.11748865655087395</v>
+        <v>0.11892421787726136</v>
       </c>
       <c r="G17" s="1">
         <v>0.17</v>
       </c>
       <c r="H17" s="1">
-        <v>56.43</v>
+        <v>56.42</v>
       </c>
       <c r="I17" s="1">
-        <v>15.38</v>
+        <v>15.37</v>
       </c>
       <c r="J17" s="1">
-        <v>-0.0025026903760530404</v>
+        <v>-0.0024820169527348685</v>
       </c>
       <c r="K17" s="1" t="b">
         <v>0</v>
@@ -1891,16 +2023,19 @@
         <v>94</v>
       </c>
       <c r="M17" s="1">
-        <v>0.09684119973452066</v>
+        <v>0.09960299428025676</v>
       </c>
       <c r="N17" s="1">
         <v>48.99999999999999</v>
       </c>
-      <c r="O17" s="1">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O17" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="P17" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>17</v>
       </c>
@@ -1917,19 +2052,19 @@
         <v>-1.85</v>
       </c>
       <c r="F18" s="4">
-        <v>-0.0675655590646727</v>
+        <v>-0.06216288328514526</v>
       </c>
       <c r="G18" s="4">
         <v>1.14</v>
       </c>
       <c r="H18" s="4">
-        <v>69.08</v>
+        <v>68.57</v>
       </c>
       <c r="I18" s="4">
-        <v>4.38</v>
+        <v>4.14</v>
       </c>
       <c r="J18" s="4">
-        <v>-0.0007267240423029835</v>
+        <v>-0.0006459754597089684</v>
       </c>
       <c r="K18" s="4" t="b">
         <v>0</v>
@@ -1938,16 +2073,19 @@
         <v>4</v>
       </c>
       <c r="M18" s="4">
-        <v>-0.0640828555052878</v>
+        <v>-0.058903881714566175</v>
       </c>
       <c r="N18" s="4">
-        <v>54.2</v>
-      </c>
-      <c r="O18" s="4">
+        <v>54.4</v>
+      </c>
+      <c r="O18" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="P18" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>18</v>
       </c>
@@ -1964,19 +2102,19 @@
         <v>3.37</v>
       </c>
       <c r="F19" s="1">
-        <v>-0.055505071827900376</v>
+        <v>-0.05935038914566073</v>
       </c>
       <c r="G19" s="1">
         <v>1.31</v>
       </c>
       <c r="H19" s="1">
-        <v>43.15</v>
+        <v>42.55</v>
       </c>
       <c r="I19" s="1">
-        <v>-6.89</v>
+        <v>-7.32</v>
       </c>
       <c r="J19" s="1">
-        <v>-0.027605050492327275</v>
+        <v>-0.0277028045198283</v>
       </c>
       <c r="K19" s="1" t="b">
         <v>1</v>
@@ -1985,16 +2123,19 @@
         <v>-7</v>
       </c>
       <c r="M19" s="1">
-        <v>-0.047793371089262404</v>
+        <v>-0.052134028525092746</v>
       </c>
       <c r="N19" s="1">
         <v>42.8</v>
       </c>
-      <c r="O19" s="1">
-        <v>-0.2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O19" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="P19" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>19</v>
       </c>
@@ -2011,19 +2152,19 @@
         <v>8.76</v>
       </c>
       <c r="F20" s="3">
-        <v>-0.05948272480163863</v>
+        <v>-0.046129321572840026</v>
       </c>
       <c r="G20" s="3">
         <v>3.67</v>
       </c>
       <c r="H20" s="3">
-        <v>69.53</v>
+        <v>69.32</v>
       </c>
       <c r="I20" s="3">
-        <v>-30.43</v>
+        <v>-30.52</v>
       </c>
       <c r="J20" s="3">
-        <v>0.023095206533151898</v>
+        <v>0.02327639229910378</v>
       </c>
       <c r="K20" s="3" t="b">
         <v>1</v>
@@ -2032,16 +2173,19 @@
         <v>-44</v>
       </c>
       <c r="M20" s="3">
-        <v>0.006937407366630399</v>
+        <v>0.01602449409463258</v>
       </c>
       <c r="N20" s="3">
-        <v>27.400000000000002</v>
-      </c>
-      <c r="O20" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+        <v>27.6</v>
+      </c>
+      <c r="O20" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="P20" s="3">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>20</v>
       </c>
@@ -2058,19 +2202,19 @@
         <v>12.21</v>
       </c>
       <c r="F21" s="3">
-        <v>-0.4405830197438053</v>
+        <v>-0.43978668983249797</v>
       </c>
       <c r="G21" s="3">
         <v>2.31</v>
       </c>
       <c r="H21" s="3">
-        <v>53.95</v>
+        <v>52.84</v>
       </c>
       <c r="I21" s="3">
-        <v>-55.29</v>
+        <v>-55.91</v>
       </c>
       <c r="J21" s="3">
-        <v>-0.03561172296348668</v>
+        <v>-0.035698987635985606</v>
       </c>
       <c r="K21" s="3" t="b">
         <v>1</v>
@@ -2079,16 +2223,19 @@
         <v>17</v>
       </c>
       <c r="M21" s="3">
-        <v>-0.40799486500956095</v>
+        <v>-0.4092917465649365</v>
       </c>
       <c r="N21" s="3">
         <v>25.799999999999994</v>
       </c>
-      <c r="O21" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O21" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="P21" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
@@ -2105,19 +2252,19 @@
         <v>5.89</v>
       </c>
       <c r="F22" s="1">
-        <v>-0.1655971450178095</v>
+        <v>-0.15052865140437732</v>
       </c>
       <c r="G22" s="1">
         <v>3.13</v>
       </c>
       <c r="H22" s="1">
-        <v>72.8</v>
+        <v>74.05</v>
       </c>
       <c r="I22" s="1">
-        <v>0.29</v>
+        <v>1.2</v>
       </c>
       <c r="J22" s="1">
-        <v>0.031117144788648583</v>
+        <v>0.031426437562972816</v>
       </c>
       <c r="K22" s="1" t="b">
         <v>1</v>
@@ -2126,16 +2273,19 @@
         <v>43</v>
       </c>
       <c r="M22" s="1">
-        <v>-0.11261029800716793</v>
+        <v>-0.1009452703662812</v>
       </c>
       <c r="N22" s="1">
-        <v>46.400000000000006</v>
-      </c>
-      <c r="O22" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+        <v>47.400000000000006</v>
+      </c>
+      <c r="O22" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="P22" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>22</v>
       </c>
@@ -2152,19 +2302,19 @@
         <v>1.42</v>
       </c>
       <c r="F23" s="3">
-        <v>-0.46051095944106835</v>
+        <v>-0.4583078229640903</v>
       </c>
       <c r="G23" s="3">
         <v>2.65</v>
       </c>
       <c r="H23" s="3">
-        <v>49.67</v>
+        <v>49.05</v>
       </c>
       <c r="I23" s="3">
-        <v>-33.89</v>
+        <v>-34.15</v>
       </c>
       <c r="J23" s="3">
-        <v>-0.012349525627281642</v>
+        <v>-0.012412428446676022</v>
       </c>
       <c r="K23" s="3" t="b">
         <v>0</v>
@@ -2173,16 +2323,19 @@
         <v>37</v>
       </c>
       <c r="M23" s="3">
-        <v>-0.41946481034831784</v>
+        <v>-0.419898161596551</v>
       </c>
       <c r="N23" s="3">
         <v>24.599999999999998</v>
       </c>
-      <c r="O23" s="3">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O23" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="P23" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>23</v>
       </c>
@@ -2199,16 +2352,16 @@
         <v>3.54</v>
       </c>
       <c r="F24" s="3">
-        <v>-0.400598246421679</v>
+        <v>-0.39542114325217326</v>
       </c>
       <c r="G24" s="3">
         <v>3.24</v>
       </c>
       <c r="H24" s="3">
-        <v>52.34</v>
+        <v>51.83</v>
       </c>
       <c r="I24" s="3">
-        <v>-30.64</v>
+        <v>-30.9</v>
       </c>
       <c r="J24" s="3">
         <v>-0.014752019382312919</v>
@@ -2220,16 +2373,19 @@
         <v>60</v>
       </c>
       <c r="M24" s="3">
-        <v>-0.34487498947152073</v>
+        <v>-0.34327711812290784</v>
       </c>
       <c r="N24" s="3">
         <v>23.200000000000003</v>
       </c>
-      <c r="O24" s="3">
-        <v>-0.4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O24" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="P24" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
         <v>24</v>
       </c>
@@ -2246,19 +2402,19 @@
         <v>2.21</v>
       </c>
       <c r="F25" s="4">
-        <v>-0.31542297047728074</v>
+        <v>-0.31406975227847667</v>
       </c>
       <c r="G25" s="4">
         <v>2.32</v>
       </c>
       <c r="H25" s="4">
-        <v>63.1</v>
+        <v>62.37</v>
       </c>
       <c r="I25" s="4">
-        <v>-19.91</v>
+        <v>-20.18</v>
       </c>
       <c r="J25" s="4">
-        <v>-0.009865523158916659</v>
+        <v>-0.009931549509908096</v>
       </c>
       <c r="K25" s="4" t="b">
         <v>0</v>
@@ -2267,16 +2423,19 @@
         <v>70</v>
       </c>
       <c r="M25" s="4">
-        <v>-0.28258605120308034</v>
+        <v>-0.28334202318444524</v>
       </c>
       <c r="N25" s="4">
         <v>51</v>
       </c>
-      <c r="O25" s="4">
-        <v>-0.2</v>
-      </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O25" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="P25" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
         <v>25</v>
       </c>
@@ -2293,19 +2452,19 @@
         <v>2.07</v>
       </c>
       <c r="F26" s="4">
-        <v>-0.15608369211525974</v>
+        <v>-0.14998950535265979</v>
       </c>
       <c r="G26" s="4">
         <v>1.2</v>
       </c>
       <c r="H26" s="4">
-        <v>54.45</v>
+        <v>54.33</v>
       </c>
       <c r="I26" s="4">
-        <v>0.38</v>
+        <v>0.33</v>
       </c>
       <c r="J26" s="4">
-        <v>-0.006401082366864428</v>
+        <v>-0.006306767977628789</v>
       </c>
       <c r="K26" s="4" t="b">
         <v>0</v>
@@ -2314,16 +2473,19 @@
         <v>116</v>
       </c>
       <c r="M26" s="4">
-        <v>-0.15110840131613845</v>
+        <v>-0.1453337888232611</v>
       </c>
       <c r="N26" s="4">
-        <v>60.400000000000006</v>
-      </c>
-      <c r="O26" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+        <v>60.6</v>
+      </c>
+      <c r="O26" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="P26" s="4">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>26</v>
       </c>
@@ -2340,7 +2502,7 @@
         <v>0.39</v>
       </c>
       <c r="F27" s="2">
-        <v>0.1639470722757364</v>
+        <v>0.16645374549769174</v>
       </c>
       <c r="G27" s="2">
         <v>1.39</v>
@@ -2352,7 +2514,7 @@
         <v>19.93</v>
       </c>
       <c r="J27" s="2">
-        <v>0.024386229289761436</v>
+        <v>0.024392011769108306</v>
       </c>
       <c r="K27" s="2" t="b">
         <v>0</v>
@@ -2361,16 +2523,19 @@
         <v>412</v>
       </c>
       <c r="M27" s="2">
-        <v>0.1736488893340229</v>
+        <v>0.1755323927300192</v>
       </c>
       <c r="N27" s="2">
         <v>75.2</v>
       </c>
-      <c r="O27" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O27" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="P27" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>27</v>
       </c>
@@ -2387,19 +2552,19 @@
         <v>2.29</v>
       </c>
       <c r="F28" s="1">
-        <v>0.0041394910754501135</v>
+        <v>0.015812694343517494</v>
       </c>
       <c r="G28" s="1">
         <v>1.69</v>
       </c>
       <c r="H28" s="1">
-        <v>62.1</v>
+        <v>62.03</v>
       </c>
       <c r="I28" s="1">
-        <v>12.57</v>
+        <v>12.51</v>
       </c>
       <c r="J28" s="1">
-        <v>0.016701733911623943</v>
+        <v>0.016891229929873873</v>
       </c>
       <c r="K28" s="1" t="b">
         <v>0</v>
@@ -2408,63 +2573,69 @@
         <v>44</v>
       </c>
       <c r="M28" s="1">
-        <v>0.02130424433241851</v>
+        <v>0.031874916369942996</v>
       </c>
       <c r="N28" s="1">
-        <v>43.800000000000004</v>
-      </c>
-      <c r="O28" s="1">
+        <v>44.800000000000004</v>
+      </c>
+      <c r="O28" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="P28" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29" s="1">
+        <v>7.4</v>
+      </c>
+      <c r="C29" s="1">
+        <v>88</v>
+      </c>
+      <c r="D29" s="1">
+        <v>1.2283783783783782</v>
+      </c>
+      <c r="E29" s="1">
+        <v>-0.84</v>
+      </c>
+      <c r="F29" s="1">
+        <v>-0.09305921798036683</v>
+      </c>
+      <c r="G29" s="1">
+        <v>1.1</v>
+      </c>
+      <c r="H29" s="1">
+        <v>41.45</v>
+      </c>
+      <c r="I29" s="1">
+        <v>-15.14</v>
+      </c>
+      <c r="J29" s="1">
+        <v>0.010710945690364857</v>
+      </c>
+      <c r="K29" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L29" s="1">
+        <v>149</v>
+      </c>
+      <c r="M29" s="1">
+        <v>-0.09073135971566748</v>
+      </c>
+      <c r="N29" s="1">
+        <v>49.599999999999994</v>
+      </c>
+      <c r="O29" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="P29" s="1">
         <v>-0.8</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A29" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B29" s="4">
-        <v>7.4</v>
-      </c>
-      <c r="C29" s="4">
-        <v>88</v>
-      </c>
-      <c r="D29" s="4">
-        <v>1.2283783783783782</v>
-      </c>
-      <c r="E29" s="4">
-        <v>-0.84</v>
-      </c>
-      <c r="F29" s="4">
-        <v>-0.09146541819570014</v>
-      </c>
-      <c r="G29" s="4">
-        <v>1.1</v>
-      </c>
-      <c r="H29" s="4">
-        <v>42.45</v>
-      </c>
-      <c r="I29" s="4">
-        <v>-14.49</v>
-      </c>
-      <c r="J29" s="4">
-        <v>0.010778051501450026</v>
-      </c>
-      <c r="K29" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="L29" s="4">
-        <v>149</v>
-      </c>
-      <c r="M29" s="4">
-        <v>-0.0889777727961395</v>
-      </c>
-      <c r="N29" s="4">
-        <v>50.4</v>
-      </c>
-      <c r="O29" s="4">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
         <v>29</v>
       </c>
@@ -2481,19 +2652,19 @@
         <v>-0.09</v>
       </c>
       <c r="F30" s="4">
-        <v>-0.11776489135020235</v>
+        <v>-0.11302898548426081</v>
       </c>
       <c r="G30" s="4">
         <v>1.43</v>
       </c>
       <c r="H30" s="4">
-        <v>68.13</v>
+        <v>67.76</v>
       </c>
       <c r="I30" s="4">
-        <v>-15.24</v>
+        <v>-15.34</v>
       </c>
       <c r="J30" s="4">
-        <v>0.01682745320942556</v>
+        <v>0.0168881689085666</v>
       </c>
       <c r="K30" s="4" t="b">
         <v>0</v>
@@ -2502,16 +2673,19 @@
         <v>-63</v>
       </c>
       <c r="M30" s="4">
-        <v>-0.1070680161320916</v>
+        <v>-0.1030191949460536</v>
       </c>
       <c r="N30" s="4">
-        <v>53.39999999999999</v>
-      </c>
-      <c r="O30" s="4">
-        <v>-0.6</v>
-      </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+        <v>53.199999999999996</v>
+      </c>
+      <c r="O30" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="P30" s="4">
+        <v>-0.2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
         <v>30</v>
       </c>
@@ -2528,19 +2702,19 @@
         <v>1.22</v>
       </c>
       <c r="F31" s="4">
-        <v>-0.020539826332099193</v>
+        <v>-0.016987291083692936</v>
       </c>
       <c r="G31" s="4">
         <v>1.05</v>
       </c>
       <c r="H31" s="4">
-        <v>62.82</v>
+        <v>62.25</v>
       </c>
       <c r="I31" s="4">
-        <v>-1.92</v>
+        <v>-2.43</v>
       </c>
       <c r="J31" s="4">
-        <v>0.004328291007456379</v>
+        <v>0.004369199174233781</v>
       </c>
       <c r="K31" s="4" t="b">
         <v>0</v>
@@ -2549,16 +2723,19 @@
         <v>93</v>
       </c>
       <c r="M31" s="4">
-        <v>-0.01929600363231887</v>
+        <v>-0.015823361951343262</v>
       </c>
       <c r="N31" s="4">
         <v>50</v>
       </c>
-      <c r="O31" s="4">
-        <v>-0.8</v>
-      </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O31" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="P31" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
         <v>31</v>
       </c>
@@ -2575,19 +2752,19 @@
         <v>-4.72</v>
       </c>
       <c r="F32" s="4">
-        <v>0.13313544243322997</v>
+        <v>0.12824337554007453</v>
       </c>
       <c r="G32" s="4">
         <v>1.36</v>
       </c>
       <c r="H32" s="4">
-        <v>74.22</v>
+        <v>71.41</v>
       </c>
       <c r="I32" s="4">
-        <v>12.57</v>
+        <v>11.65</v>
       </c>
       <c r="J32" s="4">
-        <v>0.022292434755870626</v>
+        <v>0.02214932376640168</v>
       </c>
       <c r="K32" s="4" t="b">
         <v>0</v>
@@ -2596,16 +2773,19 @@
         <v>-11</v>
       </c>
       <c r="M32" s="4">
-        <v>0.14209096587164827</v>
+        <v>0.1366236652929922</v>
       </c>
       <c r="N32" s="4">
-        <v>68.39999999999999</v>
-      </c>
-      <c r="O32" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+        <v>67.19999999999999</v>
+      </c>
+      <c r="O32" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="P32" s="4">
+        <v>-1.2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>32</v>
       </c>
@@ -2622,19 +2802,19 @@
         <v>13.14</v>
       </c>
       <c r="F33" s="1">
-        <v>0.0794475694006667</v>
+        <v>0.07059457453548217</v>
       </c>
       <c r="G33" s="1">
         <v>0</v>
       </c>
       <c r="H33" s="1">
-        <v>61.98</v>
+        <v>60.46</v>
       </c>
       <c r="I33" s="1">
-        <v>-7.32</v>
+        <v>-8.24</v>
       </c>
       <c r="J33" s="1">
-        <v>0.044189170511191735</v>
+        <v>0.04398916632335539</v>
       </c>
       <c r="K33" s="1" t="b">
         <v>0</v>
@@ -2643,16 +2823,19 @@
         <v>20</v>
       </c>
       <c r="M33" s="1">
-        <v>0.05457111540506032</v>
+        <v>0.04731599188848867</v>
       </c>
       <c r="N33" s="1">
-        <v>48.2</v>
-      </c>
-      <c r="O33" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+        <v>48.400000000000006</v>
+      </c>
+      <c r="O33" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="P33" s="1">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>33</v>
       </c>
@@ -2669,19 +2852,19 @@
         <v>-1.38</v>
       </c>
       <c r="F34" s="1">
-        <v>-0.28006059158760466</v>
+        <v>-0.27623013916963984</v>
       </c>
       <c r="G34" s="1">
         <v>0.91</v>
       </c>
       <c r="H34" s="1">
-        <v>55.97</v>
+        <v>55.45</v>
       </c>
       <c r="I34" s="1">
-        <v>-32.6</v>
+        <v>-32.78</v>
       </c>
       <c r="J34" s="1">
-        <v>-0.010815020008760702</v>
+        <v>-0.010753220837419914</v>
       </c>
       <c r="K34" s="1" t="b">
         <v>0</v>
@@ -2690,16 +2873,19 @@
         <v>3</v>
       </c>
       <c r="M34" s="1">
-        <v>-0.2822994724472092</v>
+        <v>-0.27832521160786927</v>
       </c>
       <c r="N34" s="1">
-        <v>42.2</v>
-      </c>
-      <c r="O34" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+      <c r="O34" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="P34" s="1">
+        <v>-0.2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>34</v>
       </c>
@@ -2716,19 +2902,19 @@
         <v>0.4</v>
       </c>
       <c r="F35" s="1">
-        <v>0.04342695466623904</v>
+        <v>0.04095073687320342</v>
       </c>
       <c r="G35" s="1">
         <v>0.38</v>
       </c>
       <c r="H35" s="1">
-        <v>41.35</v>
+        <v>40.8</v>
       </c>
       <c r="I35" s="1">
-        <v>3.54</v>
+        <v>3.38</v>
       </c>
       <c r="J35" s="1">
-        <v>0.006968933733247495</v>
+        <v>0.0069113389259549875</v>
       </c>
       <c r="K35" s="1" t="b">
         <v>0</v>
@@ -2737,16 +2923,19 @@
         <v>28</v>
       </c>
       <c r="M35" s="1">
-        <v>0.028003553188963082</v>
+        <v>0.02651801563206746</v>
       </c>
       <c r="N35" s="1">
         <v>46.599999999999994</v>
       </c>
-      <c r="O35" s="1">
-        <v>-0.4</v>
-      </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O35" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="P35" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
         <v>35</v>
       </c>
@@ -2763,19 +2952,19 @@
         <v>5.89</v>
       </c>
       <c r="F36" s="4">
-        <v>-0.06133460065223531</v>
+        <v>-0.05131459596580723</v>
       </c>
       <c r="G36" s="4">
         <v>1.38</v>
       </c>
       <c r="H36" s="4">
-        <v>55.75</v>
+        <v>55.82</v>
       </c>
       <c r="I36" s="4">
-        <v>-10.45</v>
+        <v>-10.4</v>
       </c>
       <c r="J36" s="4">
-        <v>0.01739455982384013</v>
+        <v>0.017564761001367033</v>
       </c>
       <c r="K36" s="4" t="b">
         <v>1</v>
@@ -2784,16 +2973,19 @@
         <v>31</v>
       </c>
       <c r="M36" s="4">
-        <v>-0.05188154813390489</v>
+        <v>-0.042468734559949706</v>
       </c>
       <c r="N36" s="4">
-        <v>61</v>
-      </c>
-      <c r="O36" s="4">
-        <v>-0.6</v>
-      </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+        <v>61.2</v>
+      </c>
+      <c r="O36" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="P36" s="4">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
         <v>36</v>
       </c>
@@ -2810,19 +3002,19 @@
         <v>-0.72</v>
       </c>
       <c r="F37" s="4">
-        <v>-0.16146366087670874</v>
+        <v>-0.15726381840375436</v>
       </c>
       <c r="G37" s="4">
         <v>2.78</v>
       </c>
       <c r="H37" s="4">
-        <v>60.56</v>
+        <v>59.88</v>
       </c>
       <c r="I37" s="4">
-        <v>-6.56</v>
+        <v>-6.95</v>
       </c>
       <c r="J37" s="4">
-        <v>0.010724473081475675</v>
+        <v>0.01071865794972338</v>
       </c>
       <c r="K37" s="4" t="b">
         <v>0</v>
@@ -2831,16 +3023,19 @@
         <v>134</v>
       </c>
       <c r="M37" s="4">
-        <v>-0.1171835727645294</v>
+        <v>-0.11582794129210594</v>
       </c>
       <c r="N37" s="4">
         <v>56.6</v>
       </c>
-      <c r="O37" s="4">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O37" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="P37" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>37</v>
       </c>
@@ -2857,19 +3052,19 @@
         <v>-1.19</v>
       </c>
       <c r="F38" s="2">
-        <v>0.7522690315963407</v>
+        <v>0.74731533337892</v>
       </c>
       <c r="G38" s="2">
         <v>2.08</v>
       </c>
       <c r="H38" s="2">
-        <v>68.69</v>
+        <v>67.47</v>
       </c>
       <c r="I38" s="2">
-        <v>72.68</v>
+        <v>70.51</v>
       </c>
       <c r="J38" s="2">
-        <v>0.04788231480104818</v>
+        <v>0.047766385700810945</v>
       </c>
       <c r="K38" s="2" t="b">
         <v>0</v>
@@ -2878,16 +3073,19 @@
         <v>234</v>
       </c>
       <c r="M38" s="2">
-        <v>0.7791356019115956</v>
+        <v>0.7724562026376729</v>
       </c>
       <c r="N38" s="2">
-        <v>73.4</v>
-      </c>
-      <c r="O38" s="2">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+        <v>72.80000000000001</v>
+      </c>
+      <c r="O38" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="P38" s="2">
+        <v>-0.6</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>38</v>
       </c>
@@ -2904,19 +3102,19 @@
         <v>3.31</v>
       </c>
       <c r="F39" s="2">
-        <v>0.4187112698573938</v>
+        <v>0.3944700233220165</v>
       </c>
       <c r="G39" s="2">
         <v>3.47</v>
       </c>
       <c r="H39" s="2">
-        <v>73.66</v>
+        <v>72.31</v>
       </c>
       <c r="I39" s="2">
-        <v>118.84</v>
+        <v>112.87</v>
       </c>
       <c r="J39" s="2">
-        <v>0.04296879405972401</v>
+        <v>0.04237675278565152</v>
       </c>
       <c r="K39" s="2" t="b">
         <v>0</v>
@@ -2925,16 +3123,19 @@
         <v>211</v>
       </c>
       <c r="M39" s="2">
-        <v>0.48015611122654156</v>
+        <v>0.45196812246009044</v>
       </c>
       <c r="N39" s="2">
-        <v>74.39999999999999</v>
-      </c>
-      <c r="O39" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+      <c r="O39" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="P39" s="2">
+        <v>-0.4</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>39</v>
       </c>
@@ -2951,19 +3152,19 @@
         <v>3.34</v>
       </c>
       <c r="F40" s="1">
-        <v>-0.2007982514277325</v>
+        <v>-0.20392777540910845</v>
       </c>
       <c r="G40" s="1">
         <v>1.68</v>
       </c>
       <c r="H40" s="1">
-        <v>43.52</v>
+        <v>44.13</v>
       </c>
       <c r="I40" s="1">
-        <v>-5.97</v>
+        <v>-5.41</v>
       </c>
       <c r="J40" s="1">
-        <v>-0.011845693448925713</v>
+        <v>-0.011969732030883737</v>
       </c>
       <c r="K40" s="1" t="b">
         <v>0</v>
@@ -2972,16 +3173,19 @@
         <v>11</v>
       </c>
       <c r="M40" s="1">
-        <v>-0.18388226271072017</v>
+        <v>-0.18809833920915286</v>
       </c>
       <c r="N40" s="1">
-        <v>45.400000000000006</v>
-      </c>
-      <c r="O40" s="1">
-        <v>-0.2</v>
-      </c>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+        <v>45.6</v>
+      </c>
+      <c r="O40" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="P40" s="1">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>40</v>
       </c>
@@ -2998,19 +3202,19 @@
         <v>16.88</v>
       </c>
       <c r="F41" s="3">
-        <v>0.16678258034043136</v>
+        <v>0.15531506095359726</v>
       </c>
       <c r="G41" s="3">
         <v>1.95</v>
       </c>
       <c r="H41" s="3">
-        <v>71.02</v>
+        <v>70.88</v>
       </c>
       <c r="I41" s="3">
-        <v>32.21</v>
+        <v>31.85</v>
       </c>
       <c r="J41" s="3">
-        <v>-0.012003514083289334</v>
+        <v>-0.012303602701941448</v>
       </c>
       <c r="K41" s="3" t="b">
         <v>1</v>
@@ -3019,16 +3223,19 @@
         <v>83</v>
       </c>
       <c r="M41" s="3">
-        <v>0.1904152116362574</v>
+        <v>0.17742971446824107</v>
       </c>
       <c r="N41" s="3">
         <v>25.800000000000004</v>
       </c>
-      <c r="O41" s="3">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O41" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="P41" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
         <v>41</v>
       </c>
@@ -3045,19 +3252,19 @@
         <v>-0.19</v>
       </c>
       <c r="F42" s="4">
-        <v>0.11162120817244162</v>
+        <v>0.11213940405695273</v>
       </c>
       <c r="G42" s="4">
         <v>1.85</v>
       </c>
       <c r="H42" s="4">
-        <v>59.95</v>
+        <v>58.87</v>
       </c>
       <c r="I42" s="4">
-        <v>55.15</v>
+        <v>54.14</v>
       </c>
       <c r="J42" s="4">
-        <v>0.01700763705192206</v>
+        <v>0.016960356829298147</v>
       </c>
       <c r="K42" s="4" t="b">
         <v>0</v>
@@ -3066,16 +3273,19 @@
         <v>300</v>
       </c>
       <c r="M42" s="4">
-        <v>0.13276619406870704</v>
+        <v>0.1319261993068972</v>
       </c>
       <c r="N42" s="4">
         <v>64.39999999999999</v>
       </c>
-      <c r="O42" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O42" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="P42" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>42</v>
       </c>
@@ -3092,19 +3302,19 @@
         <v>7.72</v>
       </c>
       <c r="F43" s="1">
-        <v>-0.3845729028929534</v>
+        <v>-0.37991373552278257</v>
       </c>
       <c r="G43" s="1">
         <v>2.61</v>
       </c>
       <c r="H43" s="1">
-        <v>54.93</v>
+        <v>54.08</v>
       </c>
       <c r="I43" s="1">
-        <v>-32.36</v>
+        <v>-32.74</v>
       </c>
       <c r="J43" s="1">
-        <v>-0.01893993006080149</v>
+        <v>-0.018925796809681986</v>
       </c>
       <c r="K43" s="1" t="b">
         <v>1</v>
@@ -3113,16 +3323,19 @@
         <v>64</v>
       </c>
       <c r="M43" s="1">
-        <v>-0.3445218119600272</v>
+        <v>-0.34243521746112304</v>
       </c>
       <c r="N43" s="1">
-        <v>31.599999999999998</v>
-      </c>
-      <c r="O43" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+      <c r="O43" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="P43" s="1">
+        <v>-0.6</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
         <v>43</v>
       </c>
@@ -3145,10 +3358,10 @@
         <v>1.41</v>
       </c>
       <c r="H44" s="4">
-        <v>62.96</v>
+        <v>62.46</v>
       </c>
       <c r="I44" s="4">
-        <v>-3.92</v>
+        <v>-4.31</v>
       </c>
       <c r="J44" s="4">
         <v>0</v>
@@ -3163,15 +3376,18 @@
         <v>0</v>
       </c>
       <c r="N44" s="4">
-        <v>55.199999999999996</v>
-      </c>
-      <c r="O44" s="4">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+        <v>55.599999999999994</v>
+      </c>
+      <c r="O44" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="P44" s="4">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>58</v>
+        <v>83</v>
       </c>
       <c r="B45" s="2">
         <v>0.95</v>
@@ -3186,19 +3402,19 @@
         <v>2.01</v>
       </c>
       <c r="F45" s="2">
-        <v>0.31197289663961014</v>
+        <v>0.31318031069321284</v>
       </c>
       <c r="G45" s="2">
         <v>0.8</v>
       </c>
       <c r="H45" s="2">
-        <v>83.89</v>
+        <v>84.07</v>
       </c>
       <c r="I45" s="2">
-        <v>36.93</v>
+        <v>36.96</v>
       </c>
       <c r="J45" s="2">
-        <v>0.026610161244824973</v>
+        <v>0.026608906205351935</v>
       </c>
       <c r="K45" s="2" t="b">
         <v>0</v>
@@ -3207,18 +3423,21 @@
         <v>11</v>
       </c>
       <c r="M45" s="2">
-        <v>0.30699760584048885</v>
+        <v>0.30852459416381417</v>
       </c>
       <c r="N45" s="2">
         <v>72</v>
       </c>
-      <c r="O45" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O45" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="P45" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>59</v>
+        <v>84</v>
       </c>
       <c r="B46" s="4">
         <v>6.11</v>
@@ -3233,19 +3452,19 @@
         <v>-2.35</v>
       </c>
       <c r="F46" s="4">
-        <v>0.2268171383624703</v>
+        <v>0.22139772405707542</v>
       </c>
       <c r="G46" s="4">
         <v>0.87</v>
       </c>
       <c r="H46" s="4">
-        <v>70.66</v>
+        <v>69.45</v>
       </c>
       <c r="I46" s="4">
-        <v>21.83</v>
+        <v>21.49</v>
       </c>
       <c r="J46" s="4">
-        <v>0.014065204785143063</v>
+        <v>0.01394367813026002</v>
       </c>
       <c r="K46" s="4" t="b">
         <v>0</v>
@@ -3254,18 +3473,21 @@
         <v>0</v>
       </c>
       <c r="M46" s="4">
-        <v>0.2235831993430415</v>
+        <v>0.21837150831296626</v>
       </c>
       <c r="N46" s="4">
-        <v>58.8</v>
-      </c>
-      <c r="O46" s="4">
-        <v>-0.4</v>
-      </c>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+        <v>59</v>
+      </c>
+      <c r="O46" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="P46" s="4">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="B47" s="4">
         <v>1.94</v>
@@ -3280,19 +3502,19 @@
         <v>0.54</v>
       </c>
       <c r="F47" s="4">
-        <v>0.04217143679343387</v>
+        <v>0.04059263864824124</v>
       </c>
       <c r="G47" s="4">
         <v>0.74</v>
       </c>
       <c r="H47" s="4">
-        <v>69.66</v>
+        <v>68.48</v>
       </c>
       <c r="I47" s="4">
-        <v>22.32</v>
+        <v>21.65</v>
       </c>
       <c r="J47" s="4">
-        <v>0.008776966289988017</v>
+        <v>0.008718581588879152</v>
       </c>
       <c r="K47" s="4" t="b">
         <v>0</v>
@@ -3301,18 +3523,21 @@
         <v>23</v>
       </c>
       <c r="M47" s="4">
-        <v>0.0357035587545762</v>
+        <v>0.03454020716002293</v>
       </c>
       <c r="N47" s="4">
-        <v>53.2</v>
-      </c>
-      <c r="O47" s="4">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+      <c r="O47" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="P47" s="4">
+        <v>-0.2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>61</v>
+        <v>87</v>
       </c>
       <c r="B48" s="4">
         <v>2.84</v>
@@ -3327,19 +3552,19 @@
         <v>0.95</v>
       </c>
       <c r="F48" s="4">
-        <v>0.1842640237296823</v>
+        <v>0.18894345727710396</v>
       </c>
       <c r="G48" s="4">
         <v>0.88</v>
       </c>
       <c r="H48" s="4">
-        <v>73.46</v>
+        <v>73.31</v>
       </c>
       <c r="I48" s="4">
-        <v>20.33</v>
+        <v>20.2</v>
       </c>
       <c r="J48" s="4">
-        <v>0.004501832495174733</v>
+        <v>0.0045619145858679455</v>
       </c>
       <c r="K48" s="4" t="b">
         <v>0</v>
@@ -3348,18 +3573,21 @@
         <v>248</v>
       </c>
       <c r="M48" s="4">
-        <v>0.18127884925020954</v>
+        <v>0.18615002735946473</v>
       </c>
       <c r="N48" s="4">
-        <v>57.400000000000006</v>
-      </c>
-      <c r="O48" s="4">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
+        <v>57.60000000000001</v>
+      </c>
+      <c r="O48" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="P48" s="4">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
-        <v>62</v>
+        <v>89</v>
       </c>
       <c r="B49" s="4">
         <v>20.88</v>
@@ -3374,19 +3602,19 @@
         <v>-0.3</v>
       </c>
       <c r="F49" s="4">
-        <v>0.002233231868567248</v>
+        <v>0.0027278534074316116</v>
       </c>
       <c r="G49" s="4">
         <v>1.05</v>
       </c>
       <c r="H49" s="4">
-        <v>63.33</v>
+        <v>62.28</v>
       </c>
       <c r="I49" s="4">
-        <v>3.52</v>
+        <v>3.26</v>
       </c>
       <c r="J49" s="4">
-        <v>-0.0010066168117376939</v>
+        <v>-0.001030523403426859</v>
       </c>
       <c r="K49" s="4" t="b">
         <v>0</v>
@@ -3395,18 +3623,21 @@
         <v>318</v>
       </c>
       <c r="M49" s="4">
-        <v>0.0034770545683475707</v>
+        <v>0.0038917825397812855</v>
       </c>
       <c r="N49" s="4">
-        <v>50.4</v>
-      </c>
-      <c r="O49" s="4">
-        <v>-0.2</v>
-      </c>
-    </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+      <c r="O49" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="P49" s="4">
+        <v>-0.4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>63</v>
+        <v>91</v>
       </c>
       <c r="B50" s="2">
         <v>8.72</v>
@@ -3421,19 +3652,19 @@
         <v>6.35</v>
       </c>
       <c r="F50" s="2">
-        <v>0.8831681458235491</v>
+        <v>0.8930752718250653</v>
       </c>
       <c r="G50" s="2">
         <v>0.96</v>
       </c>
       <c r="H50" s="2">
-        <v>72.55</v>
+        <v>72.72</v>
       </c>
       <c r="I50" s="2">
-        <v>53.49</v>
+        <v>53.86</v>
       </c>
       <c r="J50" s="2">
-        <v>0.05283941505704367</v>
+        <v>0.05296561844851371</v>
       </c>
       <c r="K50" s="2" t="b">
         <v>0</v>
@@ -3442,18 +3673,21 @@
         <v>115</v>
       </c>
       <c r="M50" s="2">
-        <v>0.8821730876637248</v>
+        <v>0.8921441285191856</v>
       </c>
       <c r="N50" s="2">
-        <v>72.39999999999999</v>
-      </c>
-      <c r="O50" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
+        <v>72.8</v>
+      </c>
+      <c r="O50" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="P50" s="2">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
-        <v>64</v>
+        <v>92</v>
       </c>
       <c r="B51" s="4">
         <v>10.45</v>
@@ -3468,19 +3702,19 @@
         <v>-0.36</v>
       </c>
       <c r="F51" s="4">
-        <v>0.1777696584470837</v>
+        <v>0.18291586187730532</v>
       </c>
       <c r="G51" s="4">
         <v>1.2</v>
       </c>
       <c r="H51" s="4">
-        <v>68.11</v>
+        <v>67.86</v>
       </c>
       <c r="I51" s="4">
-        <v>14.17</v>
+        <v>13.98</v>
       </c>
       <c r="J51" s="4">
-        <v>0.0106861724220283</v>
+        <v>0.010745172978275826</v>
       </c>
       <c r="K51" s="4" t="b">
         <v>0</v>
@@ -3489,13 +3723,16 @@
         <v>133</v>
       </c>
       <c r="M51" s="4">
-        <v>0.182744949246205</v>
+        <v>0.18757157840670402</v>
       </c>
       <c r="N51" s="4">
-        <v>57.80000000000001</v>
-      </c>
-      <c r="O51" s="4">
-        <v>0</v>
+        <v>58.8</v>
+      </c>
+      <c r="O51" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="P51" s="4">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -3511,10 +3748,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>65</v>
+        <v>94</v>
       </c>
       <c r="B1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -3546,7 +3783,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>50.800000000000004</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -3562,7 +3799,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>61</v>
+        <v>61.6</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -3570,7 +3807,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>63.599999999999994</v>
+        <v>62.99999999999999</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -3586,7 +3823,7 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>48.4</v>
+        <v>48.00000000000001</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -3602,7 +3839,7 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>40.2</v>
+        <v>40.400000000000006</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -3626,7 +3863,7 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>36.400000000000006</v>
+        <v>35.8</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -3634,7 +3871,7 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>62.6</v>
+        <v>62.2</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -3650,7 +3887,7 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>54.2</v>
+        <v>54.4</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -3666,7 +3903,7 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>27.400000000000002</v>
+        <v>27.6</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -3682,7 +3919,7 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>46.400000000000006</v>
+        <v>47.400000000000006</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -3714,7 +3951,7 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>60.400000000000006</v>
+        <v>60.6</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -3730,7 +3967,7 @@
         <v>27</v>
       </c>
       <c r="B28">
-        <v>43.800000000000004</v>
+        <v>44.800000000000004</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -3738,7 +3975,7 @@
         <v>28</v>
       </c>
       <c r="B29">
-        <v>50.4</v>
+        <v>49.599999999999994</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -3746,7 +3983,7 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>53.39999999999999</v>
+        <v>53.199999999999996</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
@@ -3762,7 +3999,7 @@
         <v>31</v>
       </c>
       <c r="B32">
-        <v>68.39999999999999</v>
+        <v>67.19999999999999</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
@@ -3770,7 +4007,7 @@
         <v>32</v>
       </c>
       <c r="B33">
-        <v>48.2</v>
+        <v>48.400000000000006</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
@@ -3778,7 +4015,7 @@
         <v>33</v>
       </c>
       <c r="B34">
-        <v>42.2</v>
+        <v>42</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
@@ -3794,7 +4031,7 @@
         <v>35</v>
       </c>
       <c r="B36">
-        <v>61</v>
+        <v>61.2</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
@@ -3810,7 +4047,7 @@
         <v>37</v>
       </c>
       <c r="B38">
-        <v>73.4</v>
+        <v>72.80000000000001</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
@@ -3818,7 +4055,7 @@
         <v>38</v>
       </c>
       <c r="B39">
-        <v>74.39999999999999</v>
+        <v>74</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
@@ -3826,7 +4063,7 @@
         <v>39</v>
       </c>
       <c r="B40">
-        <v>45.400000000000006</v>
+        <v>45.6</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
@@ -3850,7 +4087,7 @@
         <v>42</v>
       </c>
       <c r="B43">
-        <v>31.599999999999998</v>
+        <v>31</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
@@ -3858,12 +4095,12 @@
         <v>43</v>
       </c>
       <c r="B44">
-        <v>55.199999999999996</v>
+        <v>55.599999999999994</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>58</v>
+        <v>83</v>
       </c>
       <c r="B45">
         <v>72</v>
@@ -3871,50 +4108,50 @@
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>84</v>
+      </c>
+      <c r="B46">
         <v>59</v>
-      </c>
-      <c r="B46">
-        <v>58.8</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="B47">
-        <v>53.2</v>
+        <v>53</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>61</v>
+        <v>87</v>
       </c>
       <c r="B48">
-        <v>57.400000000000006</v>
+        <v>57.60000000000001</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>62</v>
+        <v>89</v>
       </c>
       <c r="B49">
-        <v>50.4</v>
+        <v>50</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>63</v>
+        <v>91</v>
       </c>
       <c r="B50">
-        <v>72.39999999999999</v>
+        <v>72.8</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>64</v>
+        <v>92</v>
       </c>
       <c r="B51">
-        <v>57.80000000000001</v>
+        <v>58.8</v>
       </c>
     </row>
   </sheetData>
@@ -3933,131 +4170,131 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>67</v>
+        <v>95</v>
       </c>
       <c r="D1" t="s">
-        <v>68</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>58</v>
+        <v>83</v>
       </c>
       <c r="C2" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="D2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>59</v>
+        <v>84</v>
       </c>
       <c r="C3" t="s">
-        <v>70</v>
+        <v>98</v>
       </c>
       <c r="D3" t="s">
-        <v>71</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="C4" t="s">
-        <v>72</v>
+        <v>100</v>
       </c>
       <c r="D4" t="s">
-        <v>73</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>74</v>
+        <v>102</v>
       </c>
       <c r="D5" t="s">
-        <v>75</v>
+        <v>103</v>
       </c>
     </row>
     <row r="6" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>76</v>
+        <v>104</v>
       </c>
       <c r="D6" t="s">
-        <v>77</v>
+        <v>105</v>
       </c>
     </row>
     <row r="7" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>78</v>
+        <v>106</v>
       </c>
       <c r="D7" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>80</v>
+        <v>108</v>
       </c>
       <c r="D8" t="s">
-        <v>81</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>82</v>
+        <v>110</v>
       </c>
       <c r="D9" t="s">
-        <v>83</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>84</v>
+        <v>112</v>
       </c>
       <c r="D10" t="s">
-        <v>85</v>
+        <v>113</v>
       </c>
     </row>
     <row r="11" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>86</v>
+        <v>114</v>
       </c>
       <c r="D11" t="s">
-        <v>87</v>
+        <v>115</v>
       </c>
     </row>
     <row r="12" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>88</v>
+        <v>116</v>
       </c>
       <c r="D12" t="s">
-        <v>89</v>
+        <v>117</v>
       </c>
     </row>
     <row r="13" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>90</v>
+        <v>118</v>
       </c>
       <c r="D13" t="s">
-        <v>91</v>
+        <v>119</v>
       </c>
     </row>
     <row r="14" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>92</v>
+        <v>120</v>
       </c>
       <c r="D14" t="s">
-        <v>93</v>
+        <v>121</v>
       </c>
     </row>
     <row r="15" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="D15" t="s">
-        <v>95</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -4076,120 +4313,120 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>67</v>
+        <v>95</v>
       </c>
       <c r="D1" t="s">
-        <v>68</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>87</v>
       </c>
       <c r="C2" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="D2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>89</v>
       </c>
       <c r="C3" t="s">
-        <v>70</v>
+        <v>98</v>
       </c>
       <c r="D3" t="s">
-        <v>96</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>74</v>
+        <v>102</v>
       </c>
       <c r="D4" t="s">
-        <v>97</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>76</v>
+        <v>104</v>
       </c>
       <c r="D5" t="s">
-        <v>98</v>
+        <v>126</v>
       </c>
     </row>
     <row r="6" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>78</v>
+        <v>106</v>
       </c>
       <c r="D6" t="s">
-        <v>99</v>
+        <v>127</v>
       </c>
     </row>
     <row r="7" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>80</v>
+        <v>108</v>
       </c>
       <c r="D7" t="s">
-        <v>81</v>
+        <v>109</v>
       </c>
     </row>
     <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>82</v>
+        <v>110</v>
       </c>
       <c r="D8" t="s">
-        <v>100</v>
+        <v>128</v>
       </c>
     </row>
     <row r="9" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>84</v>
+        <v>112</v>
       </c>
       <c r="D9" t="s">
-        <v>85</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>86</v>
+        <v>114</v>
       </c>
       <c r="D10" t="s">
-        <v>101</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>88</v>
+        <v>116</v>
       </c>
       <c r="D11" t="s">
-        <v>89</v>
+        <v>117</v>
       </c>
     </row>
     <row r="12" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>90</v>
+        <v>118</v>
       </c>
       <c r="D12" t="s">
-        <v>91</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>92</v>
+        <v>120</v>
       </c>
       <c r="D13" t="s">
-        <v>93</v>
+        <v>121</v>
       </c>
     </row>
     <row r="14" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="D14" t="s">
-        <v>102</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -4208,117 +4445,117 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>67</v>
+        <v>95</v>
       </c>
       <c r="D1" t="s">
-        <v>68</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>87</v>
       </c>
       <c r="C2" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="D2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
-        <v>70</v>
+        <v>98</v>
       </c>
       <c r="D3" t="s">
-        <v>103</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>74</v>
+        <v>102</v>
       </c>
       <c r="D4" t="s">
-        <v>97</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>76</v>
+        <v>104</v>
       </c>
       <c r="D5" t="s">
-        <v>77</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>78</v>
+        <v>106</v>
       </c>
       <c r="D6" t="s">
-        <v>104</v>
+        <v>132</v>
       </c>
     </row>
     <row r="7" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>80</v>
+        <v>108</v>
       </c>
       <c r="D7" t="s">
-        <v>81</v>
+        <v>109</v>
       </c>
     </row>
     <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>82</v>
+        <v>110</v>
       </c>
       <c r="D8" t="s">
-        <v>83</v>
+        <v>111</v>
       </c>
     </row>
     <row r="9" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>84</v>
+        <v>112</v>
       </c>
       <c r="D9" t="s">
-        <v>105</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>86</v>
+        <v>114</v>
       </c>
       <c r="D10" t="s">
-        <v>87</v>
+        <v>115</v>
       </c>
     </row>
     <row r="11" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>88</v>
+        <v>116</v>
       </c>
       <c r="D11" t="s">
-        <v>89</v>
+        <v>117</v>
       </c>
     </row>
     <row r="12" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>90</v>
+        <v>118</v>
       </c>
       <c r="D12" t="s">
-        <v>91</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>92</v>
+        <v>120</v>
       </c>
       <c r="D13" t="s">
-        <v>93</v>
+        <v>121</v>
       </c>
     </row>
     <row r="14" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="D14" t="s">
-        <v>106</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -4337,128 +4574,128 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>67</v>
+        <v>95</v>
       </c>
       <c r="D1" t="s">
-        <v>68</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>63</v>
+        <v>91</v>
       </c>
       <c r="C2" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="D2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>64</v>
+        <v>92</v>
       </c>
       <c r="C3" t="s">
-        <v>70</v>
+        <v>98</v>
       </c>
       <c r="D3" t="s">
-        <v>107</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>72</v>
+        <v>100</v>
       </c>
       <c r="D4" t="s">
-        <v>108</v>
+        <v>136</v>
       </c>
     </row>
     <row r="5" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>74</v>
+        <v>102</v>
       </c>
       <c r="D5" t="s">
-        <v>97</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>76</v>
+        <v>104</v>
       </c>
       <c r="D6" t="s">
-        <v>109</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>78</v>
+        <v>106</v>
       </c>
       <c r="D7" t="s">
-        <v>110</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>80</v>
+        <v>108</v>
       </c>
       <c r="D8" t="s">
-        <v>81</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>82</v>
+        <v>110</v>
       </c>
       <c r="D9" t="s">
-        <v>83</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>84</v>
+        <v>112</v>
       </c>
       <c r="D10" t="s">
-        <v>85</v>
+        <v>113</v>
       </c>
     </row>
     <row r="11" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>86</v>
+        <v>114</v>
       </c>
       <c r="D11" t="s">
-        <v>87</v>
+        <v>115</v>
       </c>
     </row>
     <row r="12" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>88</v>
+        <v>116</v>
       </c>
       <c r="D12" t="s">
-        <v>89</v>
+        <v>117</v>
       </c>
     </row>
     <row r="13" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>90</v>
+        <v>118</v>
       </c>
       <c r="D13" t="s">
-        <v>91</v>
+        <v>119</v>
       </c>
     </row>
     <row r="14" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>92</v>
+        <v>120</v>
       </c>
       <c r="D14" t="s">
-        <v>93</v>
+        <v>121</v>
       </c>
     </row>
     <row r="15" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
-        <v>94</v>
+        <v>122</v>
       </c>
       <c r="D15" t="s">
-        <v>102</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -4474,16 +4711,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>111</v>
+        <v>139</v>
       </c>
       <c r="B1" t="s">
-        <v>112</v>
+        <v>140</v>
       </c>
       <c r="C1" t="s">
-        <v>113</v>
+        <v>141</v>
       </c>
       <c r="D1" t="s">
-        <v>114</v>
+        <v>142</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -4491,209 +4728,209 @@
         <v>45</v>
       </c>
       <c r="B2" t="s">
-        <v>115</v>
+        <v>143</v>
       </c>
       <c r="C2" t="s">
-        <v>116</v>
+        <v>144</v>
       </c>
       <c r="D2" t="s">
-        <v>117</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="B3" t="s">
-        <v>115</v>
+        <v>143</v>
       </c>
       <c r="C3" t="s">
-        <v>119</v>
+        <v>147</v>
       </c>
       <c r="D3" t="s">
-        <v>117</v>
+        <v>145</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>120</v>
+        <v>148</v>
       </c>
       <c r="B4" t="s">
-        <v>121</v>
+        <v>149</v>
       </c>
       <c r="C4" t="s">
-        <v>122</v>
+        <v>150</v>
       </c>
       <c r="D4" t="s">
-        <v>123</v>
+        <v>151</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>124</v>
+        <v>152</v>
       </c>
       <c r="B5" t="s">
-        <v>125</v>
+        <v>153</v>
       </c>
       <c r="C5" t="s">
-        <v>126</v>
+        <v>154</v>
       </c>
       <c r="D5" t="s">
-        <v>117</v>
+        <v>145</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>127</v>
+        <v>155</v>
       </c>
       <c r="B6" t="s">
-        <v>125</v>
+        <v>153</v>
       </c>
       <c r="C6" t="s">
-        <v>128</v>
+        <v>156</v>
       </c>
       <c r="D6" t="s">
-        <v>117</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
       <c r="B7" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
       <c r="C7" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
       <c r="D7" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>130</v>
+        <v>158</v>
       </c>
       <c r="B8" t="s">
-        <v>131</v>
+        <v>159</v>
       </c>
       <c r="C8" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
       <c r="D8" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
       <c r="B9" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
       <c r="C9" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
       <c r="D9" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>132</v>
+        <v>160</v>
       </c>
       <c r="B10" t="s">
-        <v>133</v>
+        <v>161</v>
       </c>
       <c r="C10" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
       <c r="D10" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>134</v>
+        <v>162</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>135</v>
+        <v>163</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>136</v>
+        <v>164</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>137</v>
+        <v>165</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>138</v>
+        <v>166</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>139</v>
+        <v>167</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>140</v>
+        <v>168</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>141</v>
+        <v>169</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
       <c r="B15" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
       <c r="C15" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
       <c r="D15" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>142</v>
+        <v>170</v>
       </c>
       <c r="B16" t="s">
-        <v>143</v>
+        <v>171</v>
       </c>
       <c r="C16" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
       <c r="D16" t="s">
-        <v>129</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated stocks.xlsx and report.html with latest corrections
</commit_message>
<xml_diff>
--- a/data/stocks.xlsx
+++ b/data/stocks.xlsx
@@ -12,13 +12,14 @@
     <sheet sheetId="6" name="Dow_Jones" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="Nasdaq" state="visible" r:id="rId10"/>
     <sheet sheetId="8" name="SP_100" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="Composite_Formula" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="121">
   <si>
     <t>Ticker</t>
   </si>
@@ -200,13 +201,187 @@
     <t>Composite_Score</t>
   </si>
   <si>
+    <t>Earnings_Date</t>
+  </si>
+  <si>
     <t>Daily_Composite_Score_delta</t>
   </si>
   <si>
+    <t>2026-05-01</t>
+  </si>
+  <si>
+    <t>2026-05-05</t>
+  </si>
+  <si>
+    <t>2027-02-25</t>
+  </si>
+  <si>
+    <t>2026-04-22</t>
+  </si>
+  <si>
+    <t>2026-04-16</t>
+  </si>
+  <si>
+    <t>2026-04-21</t>
+  </si>
+  <si>
+    <t>2026-05-04</t>
+  </si>
+  <si>
+    <t>2026-05-06</t>
+  </si>
+  <si>
+    <t>2027-03-10</t>
+  </si>
+  <si>
+    <t>2027-03-04</t>
+  </si>
+  <si>
+    <t>2026-04-23</t>
+  </si>
+  <si>
+    <t>2027-02-26</t>
+  </si>
+  <si>
+    <t>2027-02-12</t>
+  </si>
+  <si>
+    <t>2026-04-30</t>
+  </si>
+  <si>
+    <t>2026-04-29</t>
+  </si>
+  <si>
+    <t>2026-04-28</t>
+  </si>
+  <si>
+    <t>2026-05-07</t>
+  </si>
+  <si>
+    <t>2027-03-02</t>
+  </si>
+  <si>
+    <t>2027-02-24</t>
+  </si>
+  <si>
+    <t>2027-03-03</t>
+  </si>
+  <si>
+    <t>2027-02-18</t>
+  </si>
+  <si>
+    <t>2027-02-05</t>
+  </si>
+  <si>
+    <t>2027-03-05</t>
+  </si>
+  <si>
+    <t>2027-02-27</t>
+  </si>
+  <si>
+    <t>2026-03-30</t>
+  </si>
+  <si>
     <t>_date_</t>
   </si>
   <si>
+    <t>Component</t>
+  </si>
+  <si>
+    <t>Weight</t>
+  </si>
+  <si>
+    <t>Signal Type</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>30%</t>
+  </si>
+  <si>
+    <t>Earnings quality vs peers</t>
+  </si>
+  <si>
+    <t>Finviz</t>
+  </si>
+  <si>
+    <t>P(EPS_Fwd_Growth)</t>
+  </si>
+  <si>
+    <t>Earnings acceleration</t>
+  </si>
+  <si>
+    <t>P(MA_Slope_50)</t>
+  </si>
+  <si>
+    <t>20%</t>
+  </si>
+  <si>
+    <t>Medium-term price trend</t>
+  </si>
+  <si>
+    <t>Yahoo Finance prices</t>
+  </si>
+  <si>
+    <t>P(RSI_14)</t>
+  </si>
+  <si>
+    <t>10%</t>
+  </si>
+  <si>
+    <t>Short-term momentum strength</t>
+  </si>
+  <si>
+    <t>P(SMA200_Dist)</t>
+  </si>
+  <si>
+    <t>Long-term trend confirmation</t>
+  </si>
+  <si>
     <t/>
+  </si>
+  <si>
+    <t>Formula</t>
+  </si>
+  <si>
+    <t>Composite = 0.30 × P(EPS_Univ) + 0.30 × P(Fwd_Growth) + 0.20 × P(MA_Slope_50) + 0.10 × P(RSI_14) + 0.10 × P(SMA200_Dist)</t>
+  </si>
+  <si>
+    <t>Score Range</t>
+  </si>
+  <si>
+    <t>Signal</t>
+  </si>
+  <si>
+    <t>≥ 70</t>
+  </si>
+  <si>
+    <t>Strong Buy candidate</t>
+  </si>
+  <si>
+    <t>50 – 70</t>
+  </si>
+  <si>
+    <t>Hold / Monitor</t>
+  </si>
+  <si>
+    <t>30 – 50</t>
+  </si>
+  <si>
+    <t>Weak / Neutral</t>
+  </si>
+  <si>
+    <t>&lt; 30</t>
+  </si>
+  <si>
+    <t>Consider reducing position</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>All P(x) values are percentile ranks within the current universe (0-100). Score is relative, not absolute.</t>
   </si>
 </sst>
 </file>
@@ -222,12 +397,32 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -242,8 +437,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -788,7 +987,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -839,16 +1038,16 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:P47"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -894,29 +1093,2700 @@
       <c r="O1" t="s">
         <v>60</v>
       </c>
+      <c r="P1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1">
+        <v>6.69</v>
+      </c>
+      <c r="C2" s="1">
+        <v>84.78260869565217</v>
+      </c>
+      <c r="D2" s="1">
+        <v>-0.9805680119581465</v>
+      </c>
+      <c r="E2" s="1">
+        <v>-0.01</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0.09996892429925061</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0.19</v>
+      </c>
+      <c r="H2" s="1">
+        <v>41.06</v>
+      </c>
+      <c r="I2" s="1">
+        <v>17.69</v>
+      </c>
+      <c r="J2" s="1">
+        <v>0.0007479023153258213</v>
+      </c>
+      <c r="K2" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L2" s="1">
+        <v>357</v>
+      </c>
+      <c r="M2" s="1">
+        <v>0.08156342940660632</v>
+      </c>
+      <c r="N2" s="1">
+        <v>45.434782608695656</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="P2" s="1">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2">
+        <v>2.64</v>
+      </c>
+      <c r="C3" s="2">
+        <v>67.3913043478261</v>
+      </c>
+      <c r="D3" s="2">
+        <v>23.181818181818183</v>
+      </c>
+      <c r="E3" s="2">
+        <v>2.75</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0.12599842043116044</v>
+      </c>
+      <c r="G3" s="2">
+        <v>2.13</v>
+      </c>
+      <c r="H3" s="2">
+        <v>82.11</v>
+      </c>
+      <c r="I3" s="2">
+        <v>44.96</v>
+      </c>
+      <c r="J3" s="2">
+        <v>0.03363390125374692</v>
+      </c>
+      <c r="K3" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L3" s="2">
+        <v>361</v>
+      </c>
+      <c r="M3" s="2">
+        <v>0.15167522194805927</v>
+      </c>
+      <c r="N3" s="2">
+        <v>77.3913043478261</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="P3" s="2">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3">
+        <v>-3.95</v>
+      </c>
+      <c r="C4" s="3">
+        <v>8.695652173913043</v>
+      </c>
+      <c r="D4" s="3">
+        <v>9.721518987341772</v>
+      </c>
+      <c r="E4" s="3">
+        <v>4.7</v>
+      </c>
+      <c r="F4" s="3">
+        <v>-0.28808071658688233</v>
+      </c>
+      <c r="G4" s="3">
+        <v>1.19</v>
+      </c>
+      <c r="H4" s="3">
+        <v>51.41</v>
+      </c>
+      <c r="I4" s="3">
+        <v>-26.3</v>
+      </c>
+      <c r="J4" s="3">
+        <v>-0.011637421455963387</v>
+      </c>
+      <c r="K4" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L4" s="3">
+        <v>46</v>
+      </c>
+      <c r="M4" s="3">
+        <v>-0.2837633782787312</v>
+      </c>
+      <c r="N4" s="3">
+        <v>25.434782608695652</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="P4" s="3">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4">
+        <v>1.08</v>
+      </c>
+      <c r="C5" s="4">
+        <v>58.69565217391305</v>
+      </c>
+      <c r="D5" s="4">
+        <v>28.39814814814815</v>
+      </c>
+      <c r="E5" s="4">
+        <v>0.58</v>
+      </c>
+      <c r="F5" s="4">
+        <v>-0.14718748257773764</v>
+      </c>
+      <c r="G5" s="4">
+        <v>1.86</v>
+      </c>
+      <c r="H5" s="4">
+        <v>55.23</v>
+      </c>
+      <c r="I5" s="4">
+        <v>-2.35</v>
+      </c>
+      <c r="J5" s="4">
+        <v>-0.004825343870562308</v>
+      </c>
+      <c r="K5" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L5" s="4">
+        <v>283</v>
+      </c>
+      <c r="M5" s="4">
+        <v>-0.12764584602505358</v>
+      </c>
+      <c r="N5" s="4">
+        <v>52.608695652173914</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="P5" s="4">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1">
+        <v>3.09</v>
+      </c>
+      <c r="C6" s="1">
+        <v>69.56521739130434</v>
+      </c>
+      <c r="D6" s="1">
+        <v>1.5663430420711975</v>
+      </c>
+      <c r="E6" s="1">
+        <v>-2.3</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0.041782884097026574</v>
+      </c>
+      <c r="G6" s="1">
+        <v>1.6</v>
+      </c>
+      <c r="H6" s="1">
+        <v>41.49</v>
+      </c>
+      <c r="I6" s="1">
+        <v>-11.77</v>
+      </c>
+      <c r="J6" s="1">
+        <v>0.017751614246319332</v>
+      </c>
+      <c r="K6" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L6" s="1">
+        <v>144</v>
+      </c>
+      <c r="M6" s="1">
+        <v>0.05541658401750382</v>
+      </c>
+      <c r="N6" s="1">
+        <v>46.95652173913043</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="P6" s="1">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4">
+        <v>4.9</v>
+      </c>
+      <c r="C7" s="4">
+        <v>78.26086956521739</v>
+      </c>
+      <c r="D7" s="4">
+        <v>6.042857142857143</v>
+      </c>
+      <c r="E7" s="4">
+        <v>0.37</v>
+      </c>
+      <c r="F7" s="4">
+        <v>0.03441707862937263</v>
+      </c>
+      <c r="G7" s="4">
+        <v>2.3</v>
+      </c>
+      <c r="H7" s="4">
+        <v>68.73</v>
+      </c>
+      <c r="I7" s="4">
+        <v>10.28</v>
+      </c>
+      <c r="J7" s="4">
+        <v>0.011107263617018194</v>
+      </c>
+      <c r="K7" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L7" s="4">
+        <v>410</v>
+      </c>
+      <c r="M7" s="4">
+        <v>0.06395676179040666</v>
+      </c>
+      <c r="N7" s="4">
+        <v>61.52173913043478</v>
+      </c>
+      <c r="O7" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="P7" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4">
+        <v>13.24</v>
+      </c>
+      <c r="C8" s="4">
+        <v>97.82608695652173</v>
+      </c>
+      <c r="D8" s="4">
+        <v>-0.031722054380664645</v>
+      </c>
+      <c r="E8" s="4">
+        <v>0.43</v>
+      </c>
+      <c r="F8" s="4">
+        <v>-0.0022726769078958084</v>
+      </c>
+      <c r="G8" s="4">
+        <v>0.54</v>
+      </c>
+      <c r="H8" s="4">
+        <v>81.59</v>
+      </c>
+      <c r="I8" s="4">
+        <v>13.2</v>
+      </c>
+      <c r="J8" s="4">
+        <v>0.019984041201728593</v>
+      </c>
+      <c r="K8" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L8" s="4">
+        <v>48</v>
+      </c>
+      <c r="M8" s="4">
+        <v>-0.012725180180261697</v>
+      </c>
+      <c r="N8" s="4">
+        <v>65.8695652173913</v>
+      </c>
+      <c r="O8" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="P8" s="4">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4">
+        <v>0.63</v>
+      </c>
+      <c r="C9" s="4">
+        <v>54.347826086956516</v>
+      </c>
+      <c r="D9" s="4">
+        <v>67.1111111111111</v>
+      </c>
+      <c r="E9" s="4">
+        <v>1.75</v>
+      </c>
+      <c r="F9" s="4">
+        <v>-0.1326937351573292</v>
+      </c>
+      <c r="G9" s="4">
+        <v>1.62</v>
+      </c>
+      <c r="H9" s="4">
+        <v>56.62</v>
+      </c>
+      <c r="I9" s="4">
+        <v>-8.06</v>
+      </c>
+      <c r="J9" s="4">
+        <v>0.0036242846020889314</v>
+      </c>
+      <c r="K9" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L9" s="4">
+        <v>181</v>
+      </c>
+      <c r="M9" s="4">
+        <v>-0.11860557857283605</v>
+      </c>
+      <c r="N9" s="4">
+        <v>55.65217391304348</v>
+      </c>
+      <c r="O9" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="P9" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1">
+        <v>6.79</v>
+      </c>
+      <c r="C10" s="1">
+        <v>86.95652173913044</v>
+      </c>
+      <c r="D10" s="1">
+        <v>0.6435935198821797</v>
+      </c>
+      <c r="E10" s="1">
+        <v>0.88</v>
+      </c>
+      <c r="F10" s="1">
+        <v>-0.11941150605596082</v>
+      </c>
+      <c r="G10" s="1">
+        <v>1.45</v>
+      </c>
+      <c r="H10" s="1">
+        <v>61.49</v>
+      </c>
+      <c r="I10" s="1">
+        <v>-5.1</v>
+      </c>
+      <c r="J10" s="1">
+        <v>-0.0013125148616111757</v>
+      </c>
+      <c r="K10" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L10" s="1">
+        <v>42</v>
+      </c>
+      <c r="M10" s="1">
+        <v>-0.10918623111560288</v>
+      </c>
+      <c r="N10" s="1">
+        <v>48.69565217391304</v>
+      </c>
+      <c r="O10" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="P10" s="1">
+        <v>-0.65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="C11" s="3">
+        <v>47.82608695652174</v>
+      </c>
+      <c r="D11" s="3">
+        <v>-1653.5</v>
+      </c>
+      <c r="E11" s="3">
+        <v>10.01</v>
+      </c>
+      <c r="F11" s="3">
+        <v>-0.2613708318770846</v>
+      </c>
+      <c r="G11" s="3">
+        <v>1.42</v>
+      </c>
+      <c r="H11" s="3">
+        <v>50.91</v>
+      </c>
+      <c r="I11" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="J11" s="3">
+        <v>-0.012710329593127003</v>
+      </c>
+      <c r="K11" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L11" s="3">
+        <v>28</v>
+      </c>
+      <c r="M11" s="3">
+        <v>-0.2518272419327505</v>
+      </c>
+      <c r="N11" s="3">
+        <v>25</v>
+      </c>
+      <c r="O11" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="P11" s="3">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1">
+        <v>1.31</v>
+      </c>
+      <c r="C12" s="1">
+        <v>63.04347826086957</v>
+      </c>
+      <c r="D12" s="1">
+        <v>7.5114503816793885</v>
+      </c>
+      <c r="E12" s="1">
+        <v>0.13</v>
+      </c>
+      <c r="F12" s="1">
+        <v>-0.157856292551665</v>
+      </c>
+      <c r="G12" s="1">
+        <v>0.65</v>
+      </c>
+      <c r="H12" s="1">
+        <v>53.93</v>
+      </c>
+      <c r="I12" s="1">
+        <v>-10.77</v>
+      </c>
+      <c r="J12" s="1">
+        <v>-0.012330698631726643</v>
+      </c>
+      <c r="K12" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L12" s="1">
+        <v>14</v>
+      </c>
+      <c r="M12" s="1">
+        <v>-0.1658092841719434</v>
+      </c>
+      <c r="N12" s="1">
+        <v>41.08695652173913</v>
+      </c>
+      <c r="O12" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="P12" s="1">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2">
+        <v>-0.08</v>
+      </c>
+      <c r="C13" s="2">
+        <v>41.30434782608695</v>
+      </c>
+      <c r="D13" s="2">
+        <v>1166</v>
+      </c>
+      <c r="E13" s="2">
+        <v>6.17</v>
+      </c>
+      <c r="F13" s="2">
+        <v>0.1663195259495343</v>
+      </c>
+      <c r="G13" s="2">
+        <v>1.65</v>
+      </c>
+      <c r="H13" s="2">
+        <v>70.76</v>
+      </c>
+      <c r="I13" s="2">
+        <v>74.53</v>
+      </c>
+      <c r="J13" s="2">
+        <v>0.03647987497816678</v>
+      </c>
+      <c r="K13" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L13" s="2">
+        <v>250</v>
+      </c>
+      <c r="M13" s="2">
+        <v>0.18108936753005134</v>
+      </c>
+      <c r="N13" s="2">
+        <v>76.95652173913044</v>
+      </c>
+      <c r="O13" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="P13" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="4">
+        <v>-3.83</v>
+      </c>
+      <c r="C14" s="4">
+        <v>10.869565217391305</v>
+      </c>
+      <c r="D14" s="4">
+        <v>12.668407310704959</v>
+      </c>
+      <c r="E14" s="4">
+        <v>2.52</v>
+      </c>
+      <c r="F14" s="4">
+        <v>0.09331850547452526</v>
+      </c>
+      <c r="G14" s="4">
+        <v>2.07</v>
+      </c>
+      <c r="H14" s="4">
+        <v>68.78</v>
+      </c>
+      <c r="I14" s="4">
+        <v>24.28</v>
+      </c>
+      <c r="J14" s="4">
+        <v>0.022103908627329315</v>
+      </c>
+      <c r="K14" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L14" s="4">
+        <v>24</v>
+      </c>
+      <c r="M14" s="4">
+        <v>0.11763193699937635</v>
+      </c>
+      <c r="N14" s="4">
+        <v>52.608695652173914</v>
+      </c>
+      <c r="O14" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="P14" s="4">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1">
+        <v>-6.51</v>
+      </c>
+      <c r="C15" s="1">
+        <v>4.3478260869565215</v>
+      </c>
+      <c r="D15" s="1">
+        <v>4.411674347158218</v>
+      </c>
+      <c r="E15" s="1">
+        <v>4.53</v>
+      </c>
+      <c r="F15" s="1">
+        <v>-0.03840923881066992</v>
+      </c>
+      <c r="G15" s="1">
+        <v>1.82</v>
+      </c>
+      <c r="H15" s="1">
+        <v>57.02</v>
+      </c>
+      <c r="I15" s="1">
+        <v>-2.37</v>
+      </c>
+      <c r="J15" s="1">
+        <v>0.013897275697783682</v>
+      </c>
+      <c r="K15" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L15" s="1">
+        <v>42</v>
+      </c>
+      <c r="M15" s="1">
+        <v>-0.019776515586017673</v>
+      </c>
+      <c r="N15" s="1">
+        <v>33.47826086956522</v>
+      </c>
+      <c r="O15" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="P15" s="1">
+        <v>-0.65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="4">
+        <v>-0.01</v>
+      </c>
+      <c r="C16" s="4">
+        <v>45.65217391304348</v>
+      </c>
+      <c r="D16" s="4">
+        <v>18685</v>
+      </c>
+      <c r="E16" s="4">
+        <v>11.11</v>
+      </c>
+      <c r="F16" s="4">
+        <v>-0.1397593578045052</v>
+      </c>
+      <c r="G16" s="4">
+        <v>1.22</v>
+      </c>
+      <c r="H16" s="4">
+        <v>58.5</v>
+      </c>
+      <c r="I16" s="4">
+        <v>17.19</v>
+      </c>
+      <c r="J16" s="4">
+        <v>-0.001842040615125081</v>
+      </c>
+      <c r="K16" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L16" s="4">
+        <v>31</v>
+      </c>
+      <c r="M16" s="4">
+        <v>-0.1347603345003302</v>
+      </c>
+      <c r="N16" s="4">
+        <v>63.04347826086957</v>
+      </c>
+      <c r="O16" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="P16" s="4">
+        <v>-1.74</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4">
+        <v>8.81</v>
+      </c>
+      <c r="C17" s="4">
+        <v>93.47826086956522</v>
+      </c>
+      <c r="D17" s="4">
+        <v>-0.2542565266742338</v>
+      </c>
+      <c r="E17" s="4">
+        <v>4.52</v>
+      </c>
+      <c r="F17" s="4">
+        <v>0.08708899278369829</v>
+      </c>
+      <c r="G17" s="4">
+        <v>0.18</v>
+      </c>
+      <c r="H17" s="4">
+        <v>59.05</v>
+      </c>
+      <c r="I17" s="4">
+        <v>16.86</v>
+      </c>
+      <c r="J17" s="4">
+        <v>-0.0031876764959356445</v>
+      </c>
+      <c r="K17" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L17" s="4">
+        <v>95</v>
+      </c>
+      <c r="M17" s="4">
+        <v>0.06845626955904605</v>
+      </c>
+      <c r="N17" s="4">
+        <v>50.869565217391305</v>
+      </c>
+      <c r="O17" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="P17" s="4">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="4">
+        <v>27.92</v>
+      </c>
+      <c r="C18" s="4">
+        <v>100</v>
+      </c>
+      <c r="D18" s="4">
+        <v>-0.5508595988538683</v>
+      </c>
+      <c r="E18" s="4">
+        <v>-1.85</v>
+      </c>
+      <c r="F18" s="4">
+        <v>-0.07398723892664896</v>
+      </c>
+      <c r="G18" s="4">
+        <v>1.15</v>
+      </c>
+      <c r="H18" s="4">
+        <v>63.15</v>
+      </c>
+      <c r="I18" s="4">
+        <v>2.9</v>
+      </c>
+      <c r="J18" s="4">
+        <v>-0.00012401714498254583</v>
+      </c>
+      <c r="K18" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L18" s="4">
+        <v>5</v>
+      </c>
+      <c r="M18" s="4">
+        <v>-0.07057881394652965</v>
+      </c>
+      <c r="N18" s="4">
+        <v>53.47826086956522</v>
+      </c>
+      <c r="O18" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="P18" s="4">
+        <v>-1.09</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="1">
+        <v>1.29</v>
+      </c>
+      <c r="C19" s="1">
+        <v>60.86956521739131</v>
+      </c>
+      <c r="D19" s="1">
+        <v>15.51937984496124</v>
+      </c>
+      <c r="E19" s="1">
+        <v>3.37</v>
+      </c>
+      <c r="F19" s="1">
+        <v>-0.07071837006175516</v>
+      </c>
+      <c r="G19" s="1">
+        <v>1.33</v>
+      </c>
+      <c r="H19" s="1">
+        <v>46.58</v>
+      </c>
+      <c r="I19" s="1">
+        <v>-4.49</v>
+      </c>
+      <c r="J19" s="1">
+        <v>-0.03319969783581741</v>
+      </c>
+      <c r="K19" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L19" s="1">
+        <v>-8</v>
+      </c>
+      <c r="M19" s="1">
+        <v>-0.06321983510549267</v>
+      </c>
+      <c r="N19" s="1">
+        <v>43.913043478260875</v>
+      </c>
+      <c r="O19" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="P19" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="1">
+        <v>-18.39</v>
+      </c>
+      <c r="C20" s="1">
+        <v>2.1739130434782608</v>
+      </c>
+      <c r="D20" s="1">
+        <v>-4.206090266449157</v>
+      </c>
+      <c r="E20" s="1">
+        <v>8.76</v>
+      </c>
+      <c r="F20" s="1">
+        <v>0.008381790563761982</v>
+      </c>
+      <c r="G20" s="1">
+        <v>3.65</v>
+      </c>
+      <c r="H20" s="1">
+        <v>72.85</v>
+      </c>
+      <c r="I20" s="1">
+        <v>-24.91</v>
+      </c>
+      <c r="J20" s="1">
+        <v>0.028378167283443965</v>
+      </c>
+      <c r="K20" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L20" s="1">
+        <v>-46</v>
+      </c>
+      <c r="M20" s="1">
+        <v>0.06859729854586982</v>
+      </c>
+      <c r="N20" s="1">
+        <v>30</v>
+      </c>
+      <c r="O20" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="P20" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3">
+        <v>-2.25</v>
+      </c>
+      <c r="C21" s="3">
+        <v>19.565217391304348</v>
+      </c>
+      <c r="D21" s="3">
+        <v>10.44</v>
+      </c>
+      <c r="E21" s="3">
+        <v>12.21</v>
+      </c>
+      <c r="F21" s="3">
+        <v>-0.4329896693257033</v>
+      </c>
+      <c r="G21" s="3">
+        <v>2.26</v>
+      </c>
+      <c r="H21" s="3">
+        <v>56.52</v>
+      </c>
+      <c r="I21" s="3">
+        <v>-53.26</v>
+      </c>
+      <c r="J21" s="3">
+        <v>-0.03706634906145761</v>
+      </c>
+      <c r="K21" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L21" s="3">
+        <v>25</v>
+      </c>
+      <c r="M21" s="3">
+        <v>-0.4043588994927011</v>
+      </c>
+      <c r="N21" s="3">
+        <v>25.8695652173913</v>
+      </c>
+      <c r="O21" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="P21" s="3">
+        <v>-0.65</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1">
+        <v>-2.38</v>
+      </c>
+      <c r="C22" s="1">
+        <v>17.391304347826086</v>
+      </c>
+      <c r="D22" s="1">
+        <v>1.4705882352941178</v>
+      </c>
+      <c r="E22" s="1">
+        <v>5.89</v>
+      </c>
+      <c r="F22" s="1">
+        <v>-0.08508151333094409</v>
+      </c>
+      <c r="G22" s="1">
+        <v>3.08</v>
+      </c>
+      <c r="H22" s="1">
+        <v>73.98</v>
+      </c>
+      <c r="I22" s="1">
+        <v>3.85</v>
+      </c>
+      <c r="J22" s="1">
+        <v>0.03554625294757561</v>
+      </c>
+      <c r="K22" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L22" s="1">
+        <v>48</v>
+      </c>
+      <c r="M22" s="1">
+        <v>-0.03781802027328962</v>
+      </c>
+      <c r="N22" s="1">
+        <v>46.73913043478261</v>
+      </c>
+      <c r="O22" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="P22" s="1">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3">
+        <v>-1.13</v>
+      </c>
+      <c r="C23" s="3">
+        <v>21.73913043478261</v>
+      </c>
+      <c r="D23" s="3">
+        <v>5.7522123893805315</v>
+      </c>
+      <c r="E23" s="3">
+        <v>1.42</v>
+      </c>
+      <c r="F23" s="3">
+        <v>-0.44182211533809623</v>
+      </c>
+      <c r="G23" s="3">
+        <v>2.66</v>
+      </c>
+      <c r="H23" s="3">
+        <v>49.4</v>
+      </c>
+      <c r="I23" s="3">
+        <v>-33.99</v>
+      </c>
+      <c r="J23" s="3">
+        <v>-0.0131462304015791</v>
+      </c>
+      <c r="K23" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L23" s="3">
+        <v>39</v>
+      </c>
+      <c r="M23" s="3">
+        <v>-0.4041022122247758</v>
+      </c>
+      <c r="N23" s="3">
+        <v>22.391304347826086</v>
+      </c>
+      <c r="O23" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="P23" s="3">
+        <v>-0.43</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3">
+        <v>-0.99</v>
+      </c>
+      <c r="C24" s="3">
+        <v>23.91304347826087</v>
+      </c>
+      <c r="D24" s="3">
+        <v>3.04040404040404</v>
+      </c>
+      <c r="E24" s="3">
+        <v>3.54</v>
+      </c>
+      <c r="F24" s="3">
+        <v>-0.37303787031193114</v>
+      </c>
+      <c r="G24" s="3">
+        <v>3.24</v>
+      </c>
+      <c r="H24" s="3">
+        <v>53.56</v>
+      </c>
+      <c r="I24" s="3">
+        <v>-29.81</v>
+      </c>
+      <c r="J24" s="3">
+        <v>-0.016038272851735914</v>
+      </c>
+      <c r="K24" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L24" s="3">
+        <v>61</v>
+      </c>
+      <c r="M24" s="3">
+        <v>-0.3221387239421494</v>
+      </c>
+      <c r="N24" s="3">
+        <v>22.60869565217391</v>
+      </c>
+      <c r="O24" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="P24" s="3">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25" s="4">
+        <v>0.38</v>
+      </c>
+      <c r="C25" s="4">
+        <v>50</v>
+      </c>
+      <c r="D25" s="4">
+        <v>89.71052631578947</v>
+      </c>
+      <c r="E25" s="4">
+        <v>2.21</v>
+      </c>
+      <c r="F25" s="4">
+        <v>-0.32237288207287773</v>
+      </c>
+      <c r="G25" s="4">
+        <v>2.3</v>
+      </c>
+      <c r="H25" s="4">
+        <v>61.11</v>
+      </c>
+      <c r="I25" s="4">
+        <v>-20.43</v>
+      </c>
+      <c r="J25" s="4">
+        <v>-0.009277359455133173</v>
+      </c>
+      <c r="K25" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L25" s="4">
+        <v>62</v>
+      </c>
+      <c r="M25" s="4">
+        <v>-0.2928331989118437</v>
+      </c>
+      <c r="N25" s="4">
+        <v>51.73913043478261</v>
+      </c>
+      <c r="O25" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="P25" s="4">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" s="4">
+        <v>1.9</v>
+      </c>
+      <c r="C26" s="4">
+        <v>65.21739130434783</v>
+      </c>
+      <c r="D26" s="4">
+        <v>2990.236842105264</v>
+      </c>
+      <c r="E26" s="4">
+        <v>2.07</v>
+      </c>
+      <c r="F26" s="4">
+        <v>-0.119567320339584</v>
+      </c>
+      <c r="G26" s="4">
+        <v>1.19</v>
+      </c>
+      <c r="H26" s="4">
+        <v>62.01</v>
+      </c>
+      <c r="I26" s="4">
+        <v>5.11</v>
+      </c>
+      <c r="J26" s="4">
+        <v>-0.007049404183546274</v>
+      </c>
+      <c r="K26" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L26" s="4">
+        <v>101</v>
+      </c>
+      <c r="M26" s="4">
+        <v>-0.11524998203143288</v>
+      </c>
+      <c r="N26" s="4">
+        <v>66.08695652173913</v>
+      </c>
+      <c r="O26" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="P26" s="4">
+        <v>2.39</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2">
+        <v>5.13</v>
+      </c>
+      <c r="C27" s="2">
+        <v>80.43478260869566</v>
+      </c>
+      <c r="D27" s="2">
+        <v>10.491228070175438</v>
+      </c>
+      <c r="E27" s="2">
+        <v>0.39</v>
+      </c>
+      <c r="F27" s="2">
+        <v>0.2229490479703709</v>
+      </c>
+      <c r="G27" s="2">
+        <v>1.4</v>
+      </c>
+      <c r="H27" s="2">
+        <v>78.01</v>
+      </c>
+      <c r="I27" s="2">
+        <v>24.35</v>
+      </c>
+      <c r="J27" s="2">
+        <v>0.02468420475262018</v>
+      </c>
+      <c r="K27" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L27" s="2">
+        <v>386</v>
+      </c>
+      <c r="M27" s="2">
+        <v>0.2320381812506891</v>
+      </c>
+      <c r="N27" s="2">
+        <v>76.08695652173913</v>
+      </c>
+      <c r="O27" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="P27" s="2">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28" s="1">
+        <v>-3.07</v>
+      </c>
+      <c r="C28" s="1">
+        <v>13.043478260869565</v>
+      </c>
+      <c r="D28" s="1">
+        <v>8.671009771986972</v>
+      </c>
+      <c r="E28" s="1">
+        <v>2.29</v>
+      </c>
+      <c r="F28" s="1">
+        <v>0.04116510893404747</v>
+      </c>
+      <c r="G28" s="1">
+        <v>1.71</v>
+      </c>
+      <c r="H28" s="1">
+        <v>66.88</v>
+      </c>
+      <c r="I28" s="1">
+        <v>17.06</v>
+      </c>
+      <c r="J28" s="1">
+        <v>0.018451170252593203</v>
+      </c>
+      <c r="K28" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L28" s="1">
+        <v>44</v>
+      </c>
+      <c r="M28" s="1">
+        <v>0.05729832050661221</v>
+      </c>
+      <c r="N28" s="1">
+        <v>47.173913043478265</v>
+      </c>
+      <c r="O28" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="P28" s="1">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29" s="1">
+        <v>7.4</v>
+      </c>
+      <c r="C29" s="1">
+        <v>91.30434782608695</v>
+      </c>
+      <c r="D29" s="1">
+        <v>1.2256756756756755</v>
+      </c>
+      <c r="E29" s="1">
+        <v>-0.84</v>
+      </c>
+      <c r="F29" s="1">
+        <v>-0.05617212154524295</v>
+      </c>
+      <c r="G29" s="1">
+        <v>1.09</v>
+      </c>
+      <c r="H29" s="1">
+        <v>47.34</v>
+      </c>
+      <c r="I29" s="1">
+        <v>-12.27</v>
+      </c>
+      <c r="J29" s="1">
+        <v>0.010107613393399483</v>
+      </c>
+      <c r="K29" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L29" s="1">
+        <v>124</v>
+      </c>
+      <c r="M29" s="1">
+        <v>-0.054127066557171366</v>
+      </c>
+      <c r="N29" s="1">
+        <v>49.99999999999999</v>
+      </c>
+      <c r="O29" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="P29" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30" s="4">
+        <v>5.41</v>
+      </c>
+      <c r="C30" s="4">
+        <v>82.6086956521739</v>
+      </c>
+      <c r="D30" s="4">
+        <v>0.6487985212569316</v>
+      </c>
+      <c r="E30" s="4">
+        <v>-0.09</v>
+      </c>
+      <c r="F30" s="4">
+        <v>-0.12979399564621946</v>
+      </c>
+      <c r="G30" s="4">
+        <v>1.42</v>
+      </c>
+      <c r="H30" s="4">
+        <v>67.38</v>
+      </c>
+      <c r="I30" s="4">
+        <v>-15.19</v>
+      </c>
+      <c r="J30" s="4">
+        <v>0.022425463705878987</v>
+      </c>
+      <c r="K30" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L30" s="4">
+        <v>-63</v>
+      </c>
+      <c r="M30" s="4">
+        <v>-0.12025040570188539</v>
+      </c>
+      <c r="N30" s="4">
+        <v>56.08695652173913</v>
+      </c>
+      <c r="O30" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="P30" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A31" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31" s="4">
+        <v>-0.74</v>
+      </c>
+      <c r="C31" s="4">
+        <v>28.26086956521739</v>
+      </c>
+      <c r="D31" s="4">
+        <v>36.608108108108105</v>
+      </c>
+      <c r="E31" s="4">
+        <v>1.22</v>
+      </c>
+      <c r="F31" s="4">
+        <v>0.0016923626016362228</v>
+      </c>
+      <c r="G31" s="4">
+        <v>1.08</v>
+      </c>
+      <c r="H31" s="4">
+        <v>65.35</v>
+      </c>
+      <c r="I31" s="4">
+        <v>0.49</v>
+      </c>
+      <c r="J31" s="4">
+        <v>0.008364888116717522</v>
+      </c>
+      <c r="K31" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L31" s="4">
+        <v>90</v>
+      </c>
+      <c r="M31" s="4">
+        <v>0.0035101892576998583</v>
+      </c>
+      <c r="N31" s="4">
+        <v>53.26086956521739</v>
+      </c>
+      <c r="O31" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="P31" s="4">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A32" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32" s="4">
+        <v>-0.18</v>
+      </c>
+      <c r="C32" s="4">
+        <v>39.130434782608695</v>
+      </c>
+      <c r="D32" s="4">
+        <v>105.33333333333334</v>
+      </c>
+      <c r="E32" s="4">
+        <v>-4.72</v>
+      </c>
+      <c r="F32" s="4">
+        <v>0.12212126696351888</v>
+      </c>
+      <c r="G32" s="4">
+        <v>1.36</v>
+      </c>
+      <c r="H32" s="4">
+        <v>71.01</v>
+      </c>
+      <c r="I32" s="4">
+        <v>11.54</v>
+      </c>
+      <c r="J32" s="4">
+        <v>0.02288485019404691</v>
+      </c>
+      <c r="K32" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L32" s="4">
+        <v>-11</v>
+      </c>
+      <c r="M32" s="4">
+        <v>0.13030148691580523</v>
+      </c>
+      <c r="N32" s="4">
+        <v>68.47826086956522</v>
+      </c>
+      <c r="O32" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="P32" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A33" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33" s="4">
+        <v>-4.08</v>
+      </c>
+      <c r="C33" s="4">
+        <v>6.521739130434782</v>
+      </c>
+      <c r="D33" s="4">
+        <v>14.372549019607844</v>
+      </c>
+      <c r="E33" s="4">
+        <v>13.14</v>
+      </c>
+      <c r="F33" s="4">
+        <v>0.10965664256424805</v>
+      </c>
+      <c r="G33" s="4">
+        <v>0</v>
+      </c>
+      <c r="H33" s="4">
+        <v>63.5</v>
+      </c>
+      <c r="I33" s="4">
+        <v>-5.4</v>
+      </c>
+      <c r="J33" s="4">
+        <v>0.042413988359607684</v>
+      </c>
+      <c r="K33" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L33" s="4">
+        <v>19</v>
+      </c>
+      <c r="M33" s="4">
+        <v>0.08693380936345263</v>
+      </c>
+      <c r="N33" s="4">
+        <v>50</v>
+      </c>
+      <c r="O33" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="P33" s="4">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34" s="1">
+        <v>-0.48</v>
+      </c>
+      <c r="C34" s="1">
+        <v>30.434782608695656</v>
+      </c>
+      <c r="D34" s="1">
+        <v>85.89583333333333</v>
+      </c>
+      <c r="E34" s="1">
+        <v>-1.38</v>
+      </c>
+      <c r="F34" s="1">
+        <v>-0.30901152829805545</v>
+      </c>
+      <c r="G34" s="1">
+        <v>0.87</v>
+      </c>
+      <c r="H34" s="1">
+        <v>54.87</v>
+      </c>
+      <c r="I34" s="1">
+        <v>-32.68</v>
+      </c>
+      <c r="J34" s="1">
+        <v>-0.010910532801692763</v>
+      </c>
+      <c r="K34" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L34" s="1">
+        <v>2</v>
+      </c>
+      <c r="M34" s="1">
+        <v>-0.31196549661415884</v>
+      </c>
+      <c r="N34" s="1">
+        <v>40.869565217391305</v>
+      </c>
+      <c r="O34" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="P34" s="1">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35" s="1">
+        <v>3.52</v>
+      </c>
+      <c r="C35" s="1">
+        <v>73.91304347826086</v>
+      </c>
+      <c r="D35" s="1">
+        <v>1.1988636363636365</v>
+      </c>
+      <c r="E35" s="1">
+        <v>0.4</v>
+      </c>
+      <c r="F35" s="1">
+        <v>0.03780598225516454</v>
+      </c>
+      <c r="G35" s="1">
+        <v>0.38</v>
+      </c>
+      <c r="H35" s="1">
+        <v>41.11</v>
+      </c>
+      <c r="I35" s="1">
+        <v>3.29</v>
+      </c>
+      <c r="J35" s="1">
+        <v>0.005840482007137134</v>
+      </c>
+      <c r="K35" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L35" s="1">
+        <v>30</v>
+      </c>
+      <c r="M35" s="1">
+        <v>0.023717825670671377</v>
+      </c>
+      <c r="N35" s="1">
+        <v>45.43478260869564</v>
+      </c>
+      <c r="O35" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="P35" s="1">
+        <v>-0.65</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36" s="4">
+        <v>-0.02</v>
+      </c>
+      <c r="C36" s="4">
+        <v>43.47826086956522</v>
+      </c>
+      <c r="D36" s="4">
+        <v>1215</v>
+      </c>
+      <c r="E36" s="4">
+        <v>5.89</v>
+      </c>
+      <c r="F36" s="4">
+        <v>-0.042474722199229806</v>
+      </c>
+      <c r="G36" s="4">
+        <v>1.41</v>
+      </c>
+      <c r="H36" s="4">
+        <v>57.13</v>
+      </c>
+      <c r="I36" s="4">
+        <v>-9.3</v>
+      </c>
+      <c r="J36" s="4">
+        <v>0.018793031669813467</v>
+      </c>
+      <c r="K36" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L36" s="4">
+        <v>29</v>
+      </c>
+      <c r="M36" s="4">
+        <v>-0.03315836058690369</v>
+      </c>
+      <c r="N36" s="4">
+        <v>63.04347826086957</v>
+      </c>
+      <c r="O36" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="P36" s="4">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A37" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37" s="4">
+        <v>0.94</v>
+      </c>
+      <c r="C37" s="4">
+        <v>56.52173913043478</v>
+      </c>
+      <c r="D37" s="4">
+        <v>31.03191489361702</v>
+      </c>
+      <c r="E37" s="4">
+        <v>-0.72</v>
+      </c>
+      <c r="F37" s="4">
+        <v>-0.11748082100577148</v>
+      </c>
+      <c r="G37" s="4">
+        <v>2.78</v>
+      </c>
+      <c r="H37" s="4">
+        <v>60.16</v>
+      </c>
+      <c r="I37" s="4">
+        <v>-6.59</v>
+      </c>
+      <c r="J37" s="4">
+        <v>0.013611002135374714</v>
+      </c>
+      <c r="K37" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L37" s="4">
+        <v>118</v>
+      </c>
+      <c r="M37" s="4">
+        <v>-0.07703417790835565</v>
+      </c>
+      <c r="N37" s="4">
+        <v>59.34782608695652</v>
+      </c>
+      <c r="O37" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="P37" s="4">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A38" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B38" s="4">
+        <v>7.17</v>
+      </c>
+      <c r="C38" s="4">
+        <v>89.13043478260869</v>
+      </c>
+      <c r="D38" s="4">
+        <v>2.0557880055788007</v>
+      </c>
+      <c r="E38" s="4">
+        <v>0.78</v>
+      </c>
+      <c r="F38" s="4">
+        <v>0.04783567841319197</v>
+      </c>
+      <c r="G38" s="4">
+        <v>1.42</v>
+      </c>
+      <c r="H38" s="4">
+        <v>75.45</v>
+      </c>
+      <c r="I38" s="4">
+        <v>11.74</v>
+      </c>
+      <c r="J38" s="4">
+        <v>0.01286416800260734</v>
+      </c>
+      <c r="K38" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L38" s="4">
+        <v>402</v>
+      </c>
+      <c r="M38" s="4">
+        <v>0.05737926835752605</v>
+      </c>
+      <c r="N38" s="4">
+        <v>64.78260869565219</v>
+      </c>
+      <c r="O38" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="P38" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A39" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B39" s="4">
+        <v>-0.38</v>
+      </c>
+      <c r="C39" s="4">
+        <v>34.78260869565217</v>
+      </c>
+      <c r="D39" s="4">
+        <v>882.7368421052631</v>
+      </c>
+      <c r="E39" s="4">
+        <v>0.68</v>
+      </c>
+      <c r="F39" s="4">
+        <v>-0.10456414799775396</v>
+      </c>
+      <c r="G39" s="4">
+        <v>1.51</v>
+      </c>
+      <c r="H39" s="4">
+        <v>58.98</v>
+      </c>
+      <c r="I39" s="4">
+        <v>28.59</v>
+      </c>
+      <c r="J39" s="4">
+        <v>-0.005237698966110143</v>
+      </c>
+      <c r="K39" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L39" s="4">
+        <v>28</v>
+      </c>
+      <c r="M39" s="4">
+        <v>-0.0929755030653483</v>
+      </c>
+      <c r="N39" s="4">
+        <v>56.95652173913044</v>
+      </c>
+      <c r="O39" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="P39" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A40" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40" s="4">
+        <v>11.94</v>
+      </c>
+      <c r="C40" s="4">
+        <v>95.65217391304348</v>
+      </c>
+      <c r="D40" s="4">
+        <v>0.9145728643216081</v>
+      </c>
+      <c r="E40" s="4">
+        <v>-1</v>
+      </c>
+      <c r="F40" s="4">
+        <v>0.08168919683414534</v>
+      </c>
+      <c r="G40" s="4">
+        <v>1.71</v>
+      </c>
+      <c r="H40" s="4">
+        <v>67.32</v>
+      </c>
+      <c r="I40" s="4">
+        <v>15.79</v>
+      </c>
+      <c r="J40" s="4">
+        <v>0.007987304885088326</v>
+      </c>
+      <c r="K40" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L40" s="4">
+        <v>19</v>
+      </c>
+      <c r="M40" s="4">
+        <v>0.09782240840671008</v>
+      </c>
+      <c r="N40" s="4">
+        <v>60.000000000000014</v>
+      </c>
+      <c r="O40" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="P40" s="4">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2">
+        <v>3.41</v>
+      </c>
+      <c r="C41" s="2">
+        <v>71.73913043478261</v>
+      </c>
+      <c r="D41" s="2">
+        <v>8.926686217008797</v>
+      </c>
+      <c r="E41" s="2">
+        <v>-1.19</v>
+      </c>
+      <c r="F41" s="2">
+        <v>0.6153054797879739</v>
+      </c>
+      <c r="G41" s="2">
+        <v>2.08</v>
+      </c>
+      <c r="H41" s="2">
+        <v>60.93</v>
+      </c>
+      <c r="I41" s="2">
+        <v>63.79</v>
+      </c>
+      <c r="J41" s="2">
+        <v>0.04627481066076709</v>
+      </c>
+      <c r="K41" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L41" s="2">
+        <v>235</v>
+      </c>
+      <c r="M41" s="2">
+        <v>0.639846139644833</v>
+      </c>
+      <c r="N41" s="2">
+        <v>71.30434782608695</v>
+      </c>
+      <c r="O41" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="P41" s="2">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2">
+        <v>-0.38</v>
+      </c>
+      <c r="C42" s="2">
+        <v>34.78260869565217</v>
+      </c>
+      <c r="D42" s="2">
+        <v>322.6315789473684</v>
+      </c>
+      <c r="E42" s="2">
+        <v>3.31</v>
+      </c>
+      <c r="F42" s="2">
+        <v>0.4198218532481703</v>
+      </c>
+      <c r="G42" s="2">
+        <v>3.48</v>
+      </c>
+      <c r="H42" s="2">
+        <v>73.18</v>
+      </c>
+      <c r="I42" s="2">
+        <v>114.18</v>
+      </c>
+      <c r="J42" s="2">
+        <v>0.04333575444785875</v>
+      </c>
+      <c r="K42" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L42" s="2">
+        <v>211</v>
+      </c>
+      <c r="M42" s="2">
+        <v>0.4761744795861429</v>
+      </c>
+      <c r="N42" s="2">
+        <v>75.43478260869566</v>
+      </c>
+      <c r="O42" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="P42" s="2">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B43" s="1">
+        <v>-0.32</v>
+      </c>
+      <c r="C43" s="1">
+        <v>36.95652173913043</v>
+      </c>
+      <c r="D43" s="1">
+        <v>228.28125</v>
+      </c>
+      <c r="E43" s="1">
+        <v>3.34</v>
+      </c>
+      <c r="F43" s="1">
+        <v>-0.20299411633949566</v>
+      </c>
+      <c r="G43" s="1">
+        <v>1.68</v>
+      </c>
+      <c r="H43" s="1">
+        <v>44.09</v>
+      </c>
+      <c r="I43" s="1">
+        <v>-5.45</v>
+      </c>
+      <c r="J43" s="1">
+        <v>-0.012991047223777473</v>
+      </c>
+      <c r="K43" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L43" s="1">
+        <v>12</v>
+      </c>
+      <c r="M43" s="1">
+        <v>-0.1875425897629548</v>
+      </c>
+      <c r="N43" s="1">
+        <v>44.130434782608695</v>
+      </c>
+      <c r="O43" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="P43" s="1">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A44" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B44" s="3">
+        <v>-2.92</v>
+      </c>
+      <c r="C44" s="3">
+        <v>15.217391304347828</v>
+      </c>
+      <c r="D44" s="3">
+        <v>-23.77054794520548</v>
+      </c>
+      <c r="E44" s="3">
+        <v>16.88</v>
+      </c>
+      <c r="F44" s="3">
+        <v>0.24188821420172246</v>
+      </c>
+      <c r="G44" s="3">
+        <v>1.95</v>
+      </c>
+      <c r="H44" s="3">
+        <v>74.63</v>
+      </c>
+      <c r="I44" s="3">
+        <v>41.35</v>
+      </c>
+      <c r="J44" s="3">
+        <v>-0.006994511996842627</v>
+      </c>
+      <c r="K44" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L44" s="3">
+        <v>82</v>
+      </c>
+      <c r="M44" s="3">
+        <v>0.2634749057424781</v>
+      </c>
+      <c r="N44" s="3">
+        <v>29.565217391304344</v>
+      </c>
+      <c r="O44" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="P44" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A45" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B45" s="4">
+        <v>4.88</v>
+      </c>
+      <c r="C45" s="4">
+        <v>76.08695652173914</v>
+      </c>
+      <c r="D45" s="4">
+        <v>6.172131147540984</v>
+      </c>
+      <c r="E45" s="4">
+        <v>-0.19</v>
+      </c>
+      <c r="F45" s="4">
+        <v>0.09383436891822006</v>
+      </c>
+      <c r="G45" s="4">
+        <v>1.84</v>
+      </c>
+      <c r="H45" s="4">
+        <v>59.99</v>
+      </c>
+      <c r="I45" s="4">
+        <v>54.98</v>
+      </c>
+      <c r="J45" s="4">
+        <v>0.017261853058808306</v>
+      </c>
+      <c r="K45" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L45" s="4">
+        <v>304</v>
+      </c>
+      <c r="M45" s="4">
+        <v>0.1129215488068882</v>
+      </c>
+      <c r="N45" s="4">
+        <v>63.47826086956522</v>
+      </c>
+      <c r="O45" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="P45" s="4">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A46" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B46" s="1">
+        <v>-0.76</v>
+      </c>
+      <c r="C46" s="1">
+        <v>26.08695652173913</v>
+      </c>
+      <c r="D46" s="1">
+        <v>13.236842105263158</v>
+      </c>
+      <c r="E46" s="1">
+        <v>7.72</v>
+      </c>
+      <c r="F46" s="1">
+        <v>-0.4166629597611616</v>
+      </c>
+      <c r="G46" s="1">
+        <v>2.61</v>
+      </c>
+      <c r="H46" s="1">
+        <v>57.47</v>
+      </c>
+      <c r="I46" s="1">
+        <v>-30.83</v>
+      </c>
+      <c r="J46" s="1">
+        <v>-0.020525779216574738</v>
+      </c>
+      <c r="K46" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L46" s="1">
+        <v>65</v>
+      </c>
+      <c r="M46" s="1">
+        <v>-0.38007919830788095</v>
+      </c>
+      <c r="N46" s="1">
+        <v>32.173913043478265</v>
+      </c>
+      <c r="O46" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="P46" s="1">
+        <v>0.87</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A47" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B47" s="4">
+        <v>0.54</v>
+      </c>
+      <c r="C47" s="4">
+        <v>52.17391304347826</v>
+      </c>
+      <c r="D47" s="4">
+        <v>41.629629629629626</v>
+      </c>
+      <c r="E47" s="4">
+        <v>0</v>
+      </c>
+      <c r="F47" s="4">
+        <v>-0.07112210226546752</v>
+      </c>
+      <c r="G47" s="4">
+        <v>1.43</v>
+      </c>
+      <c r="H47" s="4">
+        <v>63.64</v>
+      </c>
+      <c r="I47" s="4">
+        <v>-3.52</v>
+      </c>
+      <c r="J47" s="4">
+        <v>-0.001118055836978989</v>
+      </c>
+      <c r="K47" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L47" s="4">
+        <v>47</v>
+      </c>
+      <c r="M47" s="4">
+        <v>-0.06135128398912548</v>
+      </c>
+      <c r="N47" s="4">
+        <v>57.608695652173914</v>
+      </c>
+      <c r="O47" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="P47" s="4">
+        <v>0.65</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>61</v>
+        <v>87</v>
       </c>
       <c r="B1" t="s">
-        <v>62</v>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>45.434782608695656</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>77.3913043478261</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>25.434782608695652</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>52.608695652173914</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>46.95652173913043</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>61.52173913043478</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>65.8695652173913</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>55.65217391304348</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>48.69565217391304</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>41.08695652173913</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>76.95652173913044</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>52.608695652173914</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>33.47826086956522</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>63.04347826086957</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>50.869565217391305</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18">
+        <v>53.47826086956522</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19">
+        <v>43.913043478260875</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <v>25.8695652173913</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22">
+        <v>46.73913043478261</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23">
+        <v>22.391304347826086</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24">
+        <v>22.60869565217391</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25">
+        <v>51.73913043478261</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26">
+        <v>66.08695652173913</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27">
+        <v>76.08695652173913</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28">
+        <v>47.173913043478265</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29">
+        <v>49.99999999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <v>56.08695652173913</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31">
+        <v>53.26086956521739</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32">
+        <v>68.47826086956522</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <v>40.869565217391305</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>45.43478260869564</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <v>63.04347826086957</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37">
+        <v>59.34782608695652</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <v>64.78260869565219</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>38</v>
+      </c>
+      <c r="B39">
+        <v>56.95652173913044</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <v>60.000000000000014</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <v>71.30434782608695</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>41</v>
+      </c>
+      <c r="B42">
+        <v>75.43478260869566</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>42</v>
+      </c>
+      <c r="B43">
+        <v>44.130434782608695</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>43</v>
+      </c>
+      <c r="B44">
+        <v>29.565217391304344</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>44</v>
+      </c>
+      <c r="B45">
+        <v>63.47826086956522</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>45</v>
+      </c>
+      <c r="B46">
+        <v>32.173913043478265</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>46</v>
+      </c>
+      <c r="B47">
+        <v>57.608695652173914</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -932,7 +3802,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -948,7 +3818,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -964,7 +3834,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -980,6 +3850,241 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C3" t="s">
+        <v>96</v>
+      </c>
+      <c r="D3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C4" t="s">
+        <v>99</v>
+      </c>
+      <c r="D4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5" t="s">
+        <v>103</v>
+      </c>
+      <c r="D5" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6" t="s">
+        <v>105</v>
+      </c>
+      <c r="D6" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>106</v>
+      </c>
+      <c r="B7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" t="s">
+        <v>106</v>
+      </c>
+      <c r="D7" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>107</v>
+      </c>
+      <c r="B8" t="s">
+        <v>108</v>
+      </c>
+      <c r="C8" t="s">
+        <v>106</v>
+      </c>
+      <c r="D8" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>106</v>
+      </c>
+      <c r="B9" t="s">
+        <v>106</v>
+      </c>
+      <c r="C9" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>109</v>
+      </c>
+      <c r="B10" t="s">
+        <v>110</v>
+      </c>
+      <c r="C10" t="s">
+        <v>106</v>
+      </c>
+      <c r="D10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>106</v>
+      </c>
+      <c r="B15" t="s">
+        <v>106</v>
+      </c>
+      <c r="C15" t="s">
+        <v>106</v>
+      </c>
+      <c r="D15" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>119</v>
+      </c>
+      <c r="B16" t="s">
+        <v>120</v>
+      </c>
+      <c r="C16" t="s">
+        <v>106</v>
+      </c>
+      <c r="D16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated visualizer.js to reflect build information to check freshenss of data
</commit_message>
<xml_diff>
--- a/data/stocks.xlsx
+++ b/data/stocks.xlsx
@@ -12,13 +12,14 @@
     <sheet sheetId="6" name="Dow_Jones" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="Nasdaq" state="visible" r:id="rId10"/>
     <sheet sheetId="8" name="SP_100" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="Composite_Formula" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="121">
   <si>
     <t>Ticker</t>
   </si>
@@ -200,13 +201,187 @@
     <t>Composite_Score</t>
   </si>
   <si>
+    <t>Earnings_Date</t>
+  </si>
+  <si>
     <t>Daily_Composite_Score_delta</t>
   </si>
   <si>
+    <t>2026-05-01</t>
+  </si>
+  <si>
+    <t>2026-05-05</t>
+  </si>
+  <si>
+    <t>2027-02-25</t>
+  </si>
+  <si>
+    <t>2026-04-22</t>
+  </si>
+  <si>
+    <t>2026-04-16</t>
+  </si>
+  <si>
+    <t>2026-04-21</t>
+  </si>
+  <si>
+    <t>2026-05-04</t>
+  </si>
+  <si>
+    <t>2026-05-06</t>
+  </si>
+  <si>
+    <t>2027-03-10</t>
+  </si>
+  <si>
+    <t>2027-03-04</t>
+  </si>
+  <si>
+    <t>2026-04-23</t>
+  </si>
+  <si>
+    <t>2027-02-26</t>
+  </si>
+  <si>
+    <t>2027-02-12</t>
+  </si>
+  <si>
+    <t>2026-04-30</t>
+  </si>
+  <si>
+    <t>2026-04-29</t>
+  </si>
+  <si>
+    <t>2026-04-28</t>
+  </si>
+  <si>
+    <t>2026-05-07</t>
+  </si>
+  <si>
+    <t>2027-03-02</t>
+  </si>
+  <si>
+    <t>2027-02-24</t>
+  </si>
+  <si>
+    <t>2027-03-03</t>
+  </si>
+  <si>
+    <t>2027-02-18</t>
+  </si>
+  <si>
+    <t>2027-02-05</t>
+  </si>
+  <si>
+    <t>2027-03-05</t>
+  </si>
+  <si>
+    <t>2027-02-27</t>
+  </si>
+  <si>
+    <t>2026-03-30</t>
+  </si>
+  <si>
     <t>_date_</t>
   </si>
   <si>
+    <t>Component</t>
+  </si>
+  <si>
+    <t>Weight</t>
+  </si>
+  <si>
+    <t>Signal Type</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>30%</t>
+  </si>
+  <si>
+    <t>Earnings quality vs peers</t>
+  </si>
+  <si>
+    <t>Finviz</t>
+  </si>
+  <si>
+    <t>P(EPS_Fwd_Growth)</t>
+  </si>
+  <si>
+    <t>Earnings acceleration</t>
+  </si>
+  <si>
+    <t>P(MA_Slope_50)</t>
+  </si>
+  <si>
+    <t>20%</t>
+  </si>
+  <si>
+    <t>Medium-term price trend</t>
+  </si>
+  <si>
+    <t>Yahoo Finance prices</t>
+  </si>
+  <si>
+    <t>P(RSI_14)</t>
+  </si>
+  <si>
+    <t>10%</t>
+  </si>
+  <si>
+    <t>Short-term momentum strength</t>
+  </si>
+  <si>
+    <t>P(SMA200_Dist)</t>
+  </si>
+  <si>
+    <t>Long-term trend confirmation</t>
+  </si>
+  <si>
     <t/>
+  </si>
+  <si>
+    <t>Formula</t>
+  </si>
+  <si>
+    <t>Composite = 0.30 × P(EPS_Univ) + 0.30 × P(Fwd_Growth) + 0.20 × P(MA_Slope_50) + 0.10 × P(RSI_14) + 0.10 × P(SMA200_Dist)</t>
+  </si>
+  <si>
+    <t>Score Range</t>
+  </si>
+  <si>
+    <t>Signal</t>
+  </si>
+  <si>
+    <t>≥ 70</t>
+  </si>
+  <si>
+    <t>Strong Buy candidate</t>
+  </si>
+  <si>
+    <t>50 – 70</t>
+  </si>
+  <si>
+    <t>Hold / Monitor</t>
+  </si>
+  <si>
+    <t>30 – 50</t>
+  </si>
+  <si>
+    <t>Weak / Neutral</t>
+  </si>
+  <si>
+    <t>&lt; 30</t>
+  </si>
+  <si>
+    <t>Consider reducing position</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>All P(x) values are percentile ranks within the current universe (0-100). Score is relative, not absolute.</t>
   </si>
 </sst>
 </file>
@@ -222,12 +397,32 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -242,8 +437,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -845,10 +1044,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:P47"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -893,6 +1092,2309 @@
       </c>
       <c r="O1" t="s">
         <v>60</v>
+      </c>
+      <c r="P1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1">
+        <v>6.69</v>
+      </c>
+      <c r="C2" s="1">
+        <v>84.78260869565217</v>
+      </c>
+      <c r="D2" s="1">
+        <v>-0.9805680119581465</v>
+      </c>
+      <c r="E2" s="1">
+        <v>-0.01</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0.1008274762122777</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0.19</v>
+      </c>
+      <c r="H2" s="1">
+        <v>41.04</v>
+      </c>
+      <c r="I2" s="1">
+        <v>17.69</v>
+      </c>
+      <c r="J2" s="1">
+        <v>0.000767312784949413</v>
+      </c>
+      <c r="K2" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L2" s="1">
+        <v>357</v>
+      </c>
+      <c r="M2" s="1">
+        <v>0.08129571015627968</v>
+      </c>
+      <c r="N2" s="1">
+        <v>45.652173913043484</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="P2" s="1">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2">
+        <v>2.64</v>
+      </c>
+      <c r="C3" s="2">
+        <v>67.3913043478261</v>
+      </c>
+      <c r="D3" s="2">
+        <v>23.181818181818183</v>
+      </c>
+      <c r="E3" s="2">
+        <v>2.75</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0.13554675226258095</v>
+      </c>
+      <c r="G3" s="2">
+        <v>2.13</v>
+      </c>
+      <c r="H3" s="2">
+        <v>82.76</v>
+      </c>
+      <c r="I3" s="2">
+        <v>46.67</v>
+      </c>
+      <c r="J3" s="2">
+        <v>0.033931736160777805</v>
+      </c>
+      <c r="K3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L3" s="2">
+        <v>361</v>
+      </c>
+      <c r="M3" s="2">
+        <v>0.16279477157526956</v>
+      </c>
+      <c r="N3" s="2">
+        <v>77.3913043478261</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="P3" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3">
+        <v>-3.95</v>
+      </c>
+      <c r="C4" s="3">
+        <v>8.695652173913043</v>
+      </c>
+      <c r="D4" s="3">
+        <v>9.721518987341772</v>
+      </c>
+      <c r="E4" s="3">
+        <v>4.7</v>
+      </c>
+      <c r="F4" s="3">
+        <v>-0.2926409604404942</v>
+      </c>
+      <c r="G4" s="3">
+        <v>1.19</v>
+      </c>
+      <c r="H4" s="3">
+        <v>51.36</v>
+      </c>
+      <c r="I4" s="3">
+        <v>-26.33</v>
+      </c>
+      <c r="J4" s="3">
+        <v>-0.011710159872109282</v>
+      </c>
+      <c r="K4" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L4" s="3">
+        <v>46</v>
+      </c>
+      <c r="M4" s="3">
+        <v>-0.2880594350693342</v>
+      </c>
+      <c r="N4" s="3">
+        <v>25.217391304347828</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="P4" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4">
+        <v>1.08</v>
+      </c>
+      <c r="C5" s="4">
+        <v>58.69565217391305</v>
+      </c>
+      <c r="D5" s="4">
+        <v>28.39814814814815</v>
+      </c>
+      <c r="E5" s="4">
+        <v>0.58</v>
+      </c>
+      <c r="F5" s="4">
+        <v>-0.15459476807109435</v>
+      </c>
+      <c r="G5" s="4">
+        <v>1.86</v>
+      </c>
+      <c r="H5" s="4">
+        <v>54.55</v>
+      </c>
+      <c r="I5" s="4">
+        <v>-2.78</v>
+      </c>
+      <c r="J5" s="4">
+        <v>-0.004931709406969973</v>
+      </c>
+      <c r="K5" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L5" s="4">
+        <v>283</v>
+      </c>
+      <c r="M5" s="4">
+        <v>-0.1338573374437384</v>
+      </c>
+      <c r="N5" s="4">
+        <v>51.73913043478261</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="P5" s="4">
+        <v>-0.65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1">
+        <v>3.09</v>
+      </c>
+      <c r="C6" s="1">
+        <v>69.56521739130434</v>
+      </c>
+      <c r="D6" s="1">
+        <v>1.5663430420711975</v>
+      </c>
+      <c r="E6" s="1">
+        <v>-2.3</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0.040289182066815615</v>
+      </c>
+      <c r="G6" s="1">
+        <v>1.6</v>
+      </c>
+      <c r="H6" s="1">
+        <v>41.93</v>
+      </c>
+      <c r="I6" s="1">
+        <v>-11.58</v>
+      </c>
+      <c r="J6" s="1">
+        <v>0.01776532060850231</v>
+      </c>
+      <c r="K6" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L6" s="1">
+        <v>144</v>
+      </c>
+      <c r="M6" s="1">
+        <v>0.05475715692311045</v>
+      </c>
+      <c r="N6" s="1">
+        <v>46.95652173913043</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="P6" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4">
+        <v>4.9</v>
+      </c>
+      <c r="C7" s="4">
+        <v>78.26086956521739</v>
+      </c>
+      <c r="D7" s="4">
+        <v>6.042857142857143</v>
+      </c>
+      <c r="E7" s="4">
+        <v>0.37</v>
+      </c>
+      <c r="F7" s="4">
+        <v>0.03386742167029862</v>
+      </c>
+      <c r="G7" s="4">
+        <v>2.3</v>
+      </c>
+      <c r="H7" s="4">
+        <v>69.62</v>
+      </c>
+      <c r="I7" s="4">
+        <v>10.87</v>
+      </c>
+      <c r="J7" s="4">
+        <v>0.011160502632594714</v>
+      </c>
+      <c r="K7" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L7" s="4">
+        <v>410</v>
+      </c>
+      <c r="M7" s="4">
+        <v>0.06521470052560407</v>
+      </c>
+      <c r="N7" s="4">
+        <v>61.95652173913042</v>
+      </c>
+      <c r="O7" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="P7" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4">
+        <v>13.24</v>
+      </c>
+      <c r="C8" s="4">
+        <v>97.82608695652173</v>
+      </c>
+      <c r="D8" s="4">
+        <v>-0.024169184290030232</v>
+      </c>
+      <c r="E8" s="4">
+        <v>0.43</v>
+      </c>
+      <c r="F8" s="4">
+        <v>-0.010226989146141601</v>
+      </c>
+      <c r="G8" s="4">
+        <v>0.54</v>
+      </c>
+      <c r="H8" s="4">
+        <v>81.17</v>
+      </c>
+      <c r="I8" s="4">
+        <v>12.61</v>
+      </c>
+      <c r="J8" s="4">
+        <v>0.01980807368851632</v>
+      </c>
+      <c r="K8" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L8" s="4">
+        <v>48</v>
+      </c>
+      <c r="M8" s="4">
+        <v>-0.021319103202634304</v>
+      </c>
+      <c r="N8" s="4">
+        <v>65.8695652173913</v>
+      </c>
+      <c r="O8" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="P8" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4">
+        <v>0.63</v>
+      </c>
+      <c r="C9" s="4">
+        <v>54.347826086956516</v>
+      </c>
+      <c r="D9" s="4">
+        <v>67.1111111111111</v>
+      </c>
+      <c r="E9" s="4">
+        <v>1.75</v>
+      </c>
+      <c r="F9" s="4">
+        <v>-0.13310152654710197</v>
+      </c>
+      <c r="G9" s="4">
+        <v>1.62</v>
+      </c>
+      <c r="H9" s="4">
+        <v>57.31</v>
+      </c>
+      <c r="I9" s="4">
+        <v>-7.56</v>
+      </c>
+      <c r="J9" s="4">
+        <v>0.0036667583722992786</v>
+      </c>
+      <c r="K9" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L9" s="4">
+        <v>181</v>
+      </c>
+      <c r="M9" s="4">
+        <v>-0.11815128586226398</v>
+      </c>
+      <c r="N9" s="4">
+        <v>55.65217391304348</v>
+      </c>
+      <c r="O9" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="P9" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1">
+        <v>6.79</v>
+      </c>
+      <c r="C10" s="1">
+        <v>86.95652173913044</v>
+      </c>
+      <c r="D10" s="1">
+        <v>0.6435935198821797</v>
+      </c>
+      <c r="E10" s="1">
+        <v>0.88</v>
+      </c>
+      <c r="F10" s="1">
+        <v>-0.12398974230389055</v>
+      </c>
+      <c r="G10" s="1">
+        <v>1.45</v>
+      </c>
+      <c r="H10" s="1">
+        <v>61.31</v>
+      </c>
+      <c r="I10" s="1">
+        <v>-5.16</v>
+      </c>
+      <c r="J10" s="1">
+        <v>-0.0013695809862560113</v>
+      </c>
+      <c r="K10" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L10" s="1">
+        <v>42</v>
+      </c>
+      <c r="M10" s="1">
+        <v>-0.11313876116166943</v>
+      </c>
+      <c r="N10" s="1">
+        <v>48.47826086956522</v>
+      </c>
+      <c r="O10" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="P10" s="1">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="C11" s="3">
+        <v>47.82608695652174</v>
+      </c>
+      <c r="D11" s="3">
+        <v>-1653.5</v>
+      </c>
+      <c r="E11" s="3">
+        <v>10.01</v>
+      </c>
+      <c r="F11" s="3">
+        <v>-0.25701617436476676</v>
+      </c>
+      <c r="G11" s="3">
+        <v>1.42</v>
+      </c>
+      <c r="H11" s="3">
+        <v>52.4</v>
+      </c>
+      <c r="I11" s="3">
+        <v>1.71</v>
+      </c>
+      <c r="J11" s="3">
+        <v>-0.012555010041612849</v>
+      </c>
+      <c r="K11" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L11" s="3">
+        <v>28</v>
+      </c>
+      <c r="M11" s="3">
+        <v>-0.2468885919653604</v>
+      </c>
+      <c r="N11" s="3">
+        <v>25.434782608695652</v>
+      </c>
+      <c r="O11" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="P11" s="3">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1">
+        <v>1.31</v>
+      </c>
+      <c r="C12" s="1">
+        <v>63.04347826086957</v>
+      </c>
+      <c r="D12" s="1">
+        <v>7.5114503816793885</v>
+      </c>
+      <c r="E12" s="1">
+        <v>0.13</v>
+      </c>
+      <c r="F12" s="1">
+        <v>-0.1505522723541079</v>
+      </c>
+      <c r="G12" s="1">
+        <v>0.65</v>
+      </c>
+      <c r="H12" s="1">
+        <v>55.4</v>
+      </c>
+      <c r="I12" s="1">
+        <v>-9.57</v>
+      </c>
+      <c r="J12" s="1">
+        <v>-0.012143051089573783</v>
+      </c>
+      <c r="K12" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L12" s="1">
+        <v>14</v>
+      </c>
+      <c r="M12" s="1">
+        <v>-0.1589919243536132</v>
+      </c>
+      <c r="N12" s="1">
+        <v>41.52173913043479</v>
+      </c>
+      <c r="O12" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="P12" s="1">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2">
+        <v>-0.08</v>
+      </c>
+      <c r="C13" s="2">
+        <v>41.30434782608695</v>
+      </c>
+      <c r="D13" s="2">
+        <v>1166</v>
+      </c>
+      <c r="E13" s="2">
+        <v>6.17</v>
+      </c>
+      <c r="F13" s="2">
+        <v>0.1534630938967733</v>
+      </c>
+      <c r="G13" s="2">
+        <v>1.65</v>
+      </c>
+      <c r="H13" s="2">
+        <v>68.58</v>
+      </c>
+      <c r="I13" s="2">
+        <v>72.52</v>
+      </c>
+      <c r="J13" s="2">
+        <v>0.036242152949882776</v>
+      </c>
+      <c r="K13" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L13" s="2">
+        <v>250</v>
+      </c>
+      <c r="M13" s="2">
+        <v>0.16913673332442603</v>
+      </c>
+      <c r="N13" s="2">
+        <v>76.73913043478261</v>
+      </c>
+      <c r="O13" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="P13" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="4">
+        <v>-3.83</v>
+      </c>
+      <c r="C14" s="4">
+        <v>10.869565217391305</v>
+      </c>
+      <c r="D14" s="4">
+        <v>12.668407310704959</v>
+      </c>
+      <c r="E14" s="4">
+        <v>2.52</v>
+      </c>
+      <c r="F14" s="4">
+        <v>0.08438187589888259</v>
+      </c>
+      <c r="G14" s="4">
+        <v>2.07</v>
+      </c>
+      <c r="H14" s="4">
+        <v>67.8</v>
+      </c>
+      <c r="I14" s="4">
+        <v>22.8</v>
+      </c>
+      <c r="J14" s="4">
+        <v>0.02197442468749787</v>
+      </c>
+      <c r="K14" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L14" s="4">
+        <v>24</v>
+      </c>
+      <c r="M14" s="4">
+        <v>0.1101830977259417</v>
+      </c>
+      <c r="N14" s="4">
+        <v>51.95652173913044</v>
+      </c>
+      <c r="O14" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="P14" s="4">
+        <v>-0.43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1">
+        <v>-6.51</v>
+      </c>
+      <c r="C15" s="1">
+        <v>4.3478260869565215</v>
+      </c>
+      <c r="D15" s="1">
+        <v>4.411674347158218</v>
+      </c>
+      <c r="E15" s="1">
+        <v>4.53</v>
+      </c>
+      <c r="F15" s="1">
+        <v>-0.0412979929126466</v>
+      </c>
+      <c r="G15" s="1">
+        <v>1.82</v>
+      </c>
+      <c r="H15" s="1">
+        <v>57.34</v>
+      </c>
+      <c r="I15" s="1">
+        <v>-2.19</v>
+      </c>
+      <c r="J15" s="1">
+        <v>0.013889694610936927</v>
+      </c>
+      <c r="K15" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L15" s="1">
+        <v>42</v>
+      </c>
+      <c r="M15" s="1">
+        <v>-0.021525093942377005</v>
+      </c>
+      <c r="N15" s="1">
+        <v>33.69565217391305</v>
+      </c>
+      <c r="O15" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="P15" s="1">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="4">
+        <v>-0.01</v>
+      </c>
+      <c r="C16" s="4">
+        <v>45.65217391304348</v>
+      </c>
+      <c r="D16" s="4">
+        <v>18685</v>
+      </c>
+      <c r="E16" s="4">
+        <v>11.11</v>
+      </c>
+      <c r="F16" s="4">
+        <v>-0.14574757884685463</v>
+      </c>
+      <c r="G16" s="4">
+        <v>1.22</v>
+      </c>
+      <c r="H16" s="4">
+        <v>57.77</v>
+      </c>
+      <c r="I16" s="4">
+        <v>16.75</v>
+      </c>
+      <c r="J16" s="4">
+        <v>-0.0019455263977864303</v>
+      </c>
+      <c r="K16" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L16" s="4">
+        <v>31</v>
+      </c>
+      <c r="M16" s="4">
+        <v>-0.14044265473287987</v>
+      </c>
+      <c r="N16" s="4">
+        <v>62.82608695652174</v>
+      </c>
+      <c r="O16" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="P16" s="4">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4">
+        <v>8.81</v>
+      </c>
+      <c r="C17" s="4">
+        <v>93.47826086956522</v>
+      </c>
+      <c r="D17" s="4">
+        <v>-0.2542565266742338</v>
+      </c>
+      <c r="E17" s="4">
+        <v>4.52</v>
+      </c>
+      <c r="F17" s="4">
+        <v>0.08860564312184951</v>
+      </c>
+      <c r="G17" s="4">
+        <v>0.18</v>
+      </c>
+      <c r="H17" s="4">
+        <v>59.17</v>
+      </c>
+      <c r="I17" s="4">
+        <v>16.95</v>
+      </c>
+      <c r="J17" s="4">
+        <v>-0.003154923684622415</v>
+      </c>
+      <c r="K17" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L17" s="4">
+        <v>95</v>
+      </c>
+      <c r="M17" s="4">
+        <v>0.06883274415157992</v>
+      </c>
+      <c r="N17" s="4">
+        <v>51.08695652173914</v>
+      </c>
+      <c r="O17" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="P17" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="4">
+        <v>27.92</v>
+      </c>
+      <c r="C18" s="4">
+        <v>100</v>
+      </c>
+      <c r="D18" s="4">
+        <v>-0.5508595988538683</v>
+      </c>
+      <c r="E18" s="4">
+        <v>-1.85</v>
+      </c>
+      <c r="F18" s="4">
+        <v>-0.07768872066430293</v>
+      </c>
+      <c r="G18" s="4">
+        <v>1.15</v>
+      </c>
+      <c r="H18" s="4">
+        <v>63.12</v>
+      </c>
+      <c r="I18" s="4">
+        <v>2.9</v>
+      </c>
+      <c r="J18" s="4">
+        <v>-0.00017124448272952357</v>
+      </c>
+      <c r="K18" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L18" s="4">
+        <v>5</v>
+      </c>
+      <c r="M18" s="4">
+        <v>-0.07407172695022923</v>
+      </c>
+      <c r="N18" s="4">
+        <v>54.34782608695652</v>
+      </c>
+      <c r="O18" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="P18" s="4">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="1">
+        <v>1.29</v>
+      </c>
+      <c r="C19" s="1">
+        <v>60.86956521739131</v>
+      </c>
+      <c r="D19" s="1">
+        <v>15.51937984496124</v>
+      </c>
+      <c r="E19" s="1">
+        <v>3.37</v>
+      </c>
+      <c r="F19" s="1">
+        <v>-0.059362273386575806</v>
+      </c>
+      <c r="G19" s="1">
+        <v>1.33</v>
+      </c>
+      <c r="H19" s="1">
+        <v>47.16</v>
+      </c>
+      <c r="I19" s="1">
+        <v>-4.03</v>
+      </c>
+      <c r="J19" s="1">
+        <v>-0.032972728826274986</v>
+      </c>
+      <c r="K19" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L19" s="1">
+        <v>-8</v>
+      </c>
+      <c r="M19" s="1">
+        <v>-0.05140488721561365</v>
+      </c>
+      <c r="N19" s="1">
+        <v>44.1304347826087</v>
+      </c>
+      <c r="O19" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="P19" s="1">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="1">
+        <v>-18.39</v>
+      </c>
+      <c r="C20" s="1">
+        <v>2.1739130434782608</v>
+      </c>
+      <c r="D20" s="1">
+        <v>-4.206090266449157</v>
+      </c>
+      <c r="E20" s="1">
+        <v>8.76</v>
+      </c>
+      <c r="F20" s="1">
+        <v>-0.01879277749792678</v>
+      </c>
+      <c r="G20" s="1">
+        <v>3.65</v>
+      </c>
+      <c r="H20" s="1">
+        <v>72.27</v>
+      </c>
+      <c r="I20" s="1">
+        <v>-25.64</v>
+      </c>
+      <c r="J20" s="1">
+        <v>0.02783189594132707</v>
+      </c>
+      <c r="K20" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L20" s="1">
+        <v>-46</v>
+      </c>
+      <c r="M20" s="1">
+        <v>0.04510744478404205</v>
+      </c>
+      <c r="N20" s="1">
+        <v>30</v>
+      </c>
+      <c r="O20" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="P20" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3">
+        <v>-2.25</v>
+      </c>
+      <c r="C21" s="3">
+        <v>19.565217391304348</v>
+      </c>
+      <c r="D21" s="3">
+        <v>10.44</v>
+      </c>
+      <c r="E21" s="3">
+        <v>12.21</v>
+      </c>
+      <c r="F21" s="3">
+        <v>-0.4257523619448244</v>
+      </c>
+      <c r="G21" s="3">
+        <v>2.26</v>
+      </c>
+      <c r="H21" s="3">
+        <v>57.74</v>
+      </c>
+      <c r="I21" s="3">
+        <v>-52.37</v>
+      </c>
+      <c r="J21" s="3">
+        <v>-0.036738611374177825</v>
+      </c>
+      <c r="K21" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L21" s="3">
+        <v>25</v>
+      </c>
+      <c r="M21" s="3">
+        <v>-0.39536961474660526</v>
+      </c>
+      <c r="N21" s="3">
+        <v>26.739130434782606</v>
+      </c>
+      <c r="O21" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="P21" s="3">
+        <v>0.87</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1">
+        <v>-2.38</v>
+      </c>
+      <c r="C22" s="1">
+        <v>17.391304347826086</v>
+      </c>
+      <c r="D22" s="1">
+        <v>1.4705882352941178</v>
+      </c>
+      <c r="E22" s="1">
+        <v>5.89</v>
+      </c>
+      <c r="F22" s="1">
+        <v>-0.11802123762200953</v>
+      </c>
+      <c r="G22" s="1">
+        <v>3.08</v>
+      </c>
+      <c r="H22" s="1">
+        <v>72.74</v>
+      </c>
+      <c r="I22" s="1">
+        <v>1.33</v>
+      </c>
+      <c r="J22" s="1">
+        <v>0.03470869757352629</v>
+      </c>
+      <c r="K22" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L22" s="1">
+        <v>48</v>
+      </c>
+      <c r="M22" s="1">
+        <v>-0.06786559145352078</v>
+      </c>
+      <c r="N22" s="1">
+        <v>45.869565217391305</v>
+      </c>
+      <c r="O22" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="P22" s="1">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3">
+        <v>-1.13</v>
+      </c>
+      <c r="C23" s="3">
+        <v>21.73913043478261</v>
+      </c>
+      <c r="D23" s="3">
+        <v>5.7522123893805315</v>
+      </c>
+      <c r="E23" s="3">
+        <v>1.42</v>
+      </c>
+      <c r="F23" s="3">
+        <v>-0.4479682759646458</v>
+      </c>
+      <c r="G23" s="3">
+        <v>2.66</v>
+      </c>
+      <c r="H23" s="3">
+        <v>49.03</v>
+      </c>
+      <c r="I23" s="3">
+        <v>-34.14</v>
+      </c>
+      <c r="J23" s="3">
+        <v>-0.013220085323303233</v>
+      </c>
+      <c r="K23" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L23" s="3">
+        <v>39</v>
+      </c>
+      <c r="M23" s="3">
+        <v>-0.4079402121955634</v>
+      </c>
+      <c r="N23" s="3">
+        <v>22.391304347826086</v>
+      </c>
+      <c r="O23" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="P23" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3">
+        <v>-0.99</v>
+      </c>
+      <c r="C24" s="3">
+        <v>23.91304347826087</v>
+      </c>
+      <c r="D24" s="3">
+        <v>3.04040404040404</v>
+      </c>
+      <c r="E24" s="3">
+        <v>3.54</v>
+      </c>
+      <c r="F24" s="3">
+        <v>-0.3834461650194826</v>
+      </c>
+      <c r="G24" s="3">
+        <v>3.24</v>
+      </c>
+      <c r="H24" s="3">
+        <v>52.77</v>
+      </c>
+      <c r="I24" s="3">
+        <v>-30.24</v>
+      </c>
+      <c r="J24" s="3">
+        <v>-0.0161972256448195</v>
+      </c>
+      <c r="K24" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L24" s="3">
+        <v>61</v>
+      </c>
+      <c r="M24" s="3">
+        <v>-0.32943239222264853</v>
+      </c>
+      <c r="N24" s="3">
+        <v>22.60869565217391</v>
+      </c>
+      <c r="O24" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="P24" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25" s="4">
+        <v>0.38</v>
+      </c>
+      <c r="C25" s="4">
+        <v>50</v>
+      </c>
+      <c r="D25" s="4">
+        <v>89.71052631578947</v>
+      </c>
+      <c r="E25" s="4">
+        <v>2.21</v>
+      </c>
+      <c r="F25" s="4">
+        <v>-0.3271270914927164</v>
+      </c>
+      <c r="G25" s="4">
+        <v>2.3</v>
+      </c>
+      <c r="H25" s="4">
+        <v>61.04</v>
+      </c>
+      <c r="I25" s="4">
+        <v>-20.47</v>
+      </c>
+      <c r="J25" s="4">
+        <v>-0.009321426722427306</v>
+      </c>
+      <c r="K25" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L25" s="4">
+        <v>62</v>
+      </c>
+      <c r="M25" s="4">
+        <v>-0.29577981263741093</v>
+      </c>
+      <c r="N25" s="4">
+        <v>51.52173913043478</v>
+      </c>
+      <c r="O25" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="P25" s="4">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" s="4">
+        <v>1.9</v>
+      </c>
+      <c r="C26" s="4">
+        <v>65.21739130434783</v>
+      </c>
+      <c r="D26" s="4">
+        <v>2990.236842105264</v>
+      </c>
+      <c r="E26" s="4">
+        <v>2.07</v>
+      </c>
+      <c r="F26" s="4">
+        <v>-0.1137240652607237</v>
+      </c>
+      <c r="G26" s="4">
+        <v>1.19</v>
+      </c>
+      <c r="H26" s="4">
+        <v>62.57</v>
+      </c>
+      <c r="I26" s="4">
+        <v>5.52</v>
+      </c>
+      <c r="J26" s="4">
+        <v>-0.0068792273359546295</v>
+      </c>
+      <c r="K26" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L26" s="4">
+        <v>101</v>
+      </c>
+      <c r="M26" s="4">
+        <v>-0.10914253988956368</v>
+      </c>
+      <c r="N26" s="4">
+        <v>66.73913043478261</v>
+      </c>
+      <c r="O26" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="P26" s="4">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2">
+        <v>5.13</v>
+      </c>
+      <c r="C27" s="2">
+        <v>80.43478260869566</v>
+      </c>
+      <c r="D27" s="2">
+        <v>10.491228070175438</v>
+      </c>
+      <c r="E27" s="2">
+        <v>0.39</v>
+      </c>
+      <c r="F27" s="2">
+        <v>0.23160151071424817</v>
+      </c>
+      <c r="G27" s="2">
+        <v>1.4</v>
+      </c>
+      <c r="H27" s="2">
+        <v>78.63</v>
+      </c>
+      <c r="I27" s="2">
+        <v>25.29</v>
+      </c>
+      <c r="J27" s="2">
+        <v>0.02489548308240803</v>
+      </c>
+      <c r="K27" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L27" s="2">
+        <v>386</v>
+      </c>
+      <c r="M27" s="2">
+        <v>0.24124682728511138</v>
+      </c>
+      <c r="N27" s="2">
+        <v>76.08695652173913</v>
+      </c>
+      <c r="O27" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="P27" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28" s="1">
+        <v>-3.07</v>
+      </c>
+      <c r="C28" s="1">
+        <v>13.043478260869565</v>
+      </c>
+      <c r="D28" s="1">
+        <v>8.667752442996743</v>
+      </c>
+      <c r="E28" s="1">
+        <v>2.29</v>
+      </c>
+      <c r="F28" s="1">
+        <v>0.02300113273057261</v>
+      </c>
+      <c r="G28" s="1">
+        <v>1.71</v>
+      </c>
+      <c r="H28" s="1">
+        <v>66.58</v>
+      </c>
+      <c r="I28" s="1">
+        <v>16.73</v>
+      </c>
+      <c r="J28" s="1">
+        <v>0.01811225760128193</v>
+      </c>
+      <c r="K28" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L28" s="1">
+        <v>44</v>
+      </c>
+      <c r="M28" s="1">
+        <v>0.040121569643854826</v>
+      </c>
+      <c r="N28" s="1">
+        <v>46.95652173913044</v>
+      </c>
+      <c r="O28" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="P28" s="1">
+        <v>-1.09</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29" s="1">
+        <v>7.4</v>
+      </c>
+      <c r="C29" s="1">
+        <v>91.30434782608695</v>
+      </c>
+      <c r="D29" s="1">
+        <v>1.2256756756756755</v>
+      </c>
+      <c r="E29" s="1">
+        <v>-0.84</v>
+      </c>
+      <c r="F29" s="1">
+        <v>-0.06157745009525035</v>
+      </c>
+      <c r="G29" s="1">
+        <v>1.09</v>
+      </c>
+      <c r="H29" s="1">
+        <v>47.51</v>
+      </c>
+      <c r="I29" s="1">
+        <v>-12.18</v>
+      </c>
+      <c r="J29" s="1">
+        <v>0.010030126685428955</v>
+      </c>
+      <c r="K29" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L29" s="1">
+        <v>124</v>
+      </c>
+      <c r="M29" s="1">
+        <v>-0.05940725386680612</v>
+      </c>
+      <c r="N29" s="1">
+        <v>49.99999999999999</v>
+      </c>
+      <c r="O29" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="P29" s="1">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30" s="4">
+        <v>5.41</v>
+      </c>
+      <c r="C30" s="4">
+        <v>82.6086956521739</v>
+      </c>
+      <c r="D30" s="4">
+        <v>0.6487985212569316</v>
+      </c>
+      <c r="E30" s="4">
+        <v>-0.09</v>
+      </c>
+      <c r="F30" s="4">
+        <v>-0.13114399355140938</v>
+      </c>
+      <c r="G30" s="4">
+        <v>1.42</v>
+      </c>
+      <c r="H30" s="4">
+        <v>67.82</v>
+      </c>
+      <c r="I30" s="4">
+        <v>-14.94</v>
+      </c>
+      <c r="J30" s="4">
+        <v>0.02244117984151456</v>
+      </c>
+      <c r="K30" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L30" s="4">
+        <v>-63</v>
+      </c>
+      <c r="M30" s="4">
+        <v>-0.12101641115200301</v>
+      </c>
+      <c r="N30" s="4">
+        <v>56.08695652173913</v>
+      </c>
+      <c r="O30" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="P30" s="4">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A31" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31" s="4">
+        <v>-0.74</v>
+      </c>
+      <c r="C31" s="4">
+        <v>28.26086956521739</v>
+      </c>
+      <c r="D31" s="4">
+        <v>36.608108108108105</v>
+      </c>
+      <c r="E31" s="4">
+        <v>1.22</v>
+      </c>
+      <c r="F31" s="4">
+        <v>0.0027810480137657745</v>
+      </c>
+      <c r="G31" s="4">
+        <v>1.08</v>
+      </c>
+      <c r="H31" s="4">
+        <v>65.81</v>
+      </c>
+      <c r="I31" s="4">
+        <v>0.95</v>
+      </c>
+      <c r="J31" s="4">
+        <v>0.008421891102854916</v>
+      </c>
+      <c r="K31" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L31" s="4">
+        <v>90</v>
+      </c>
+      <c r="M31" s="4">
+        <v>0.0047101113279384155</v>
+      </c>
+      <c r="N31" s="4">
+        <v>53.26086956521739</v>
+      </c>
+      <c r="O31" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="P31" s="4">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A32" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32" s="4">
+        <v>-0.18</v>
+      </c>
+      <c r="C32" s="4">
+        <v>39.130434782608695</v>
+      </c>
+      <c r="D32" s="4">
+        <v>105.33333333333334</v>
+      </c>
+      <c r="E32" s="4">
+        <v>-4.72</v>
+      </c>
+      <c r="F32" s="4">
+        <v>0.11290929379608892</v>
+      </c>
+      <c r="G32" s="4">
+        <v>1.36</v>
+      </c>
+      <c r="H32" s="4">
+        <v>70.33</v>
+      </c>
+      <c r="I32" s="4">
+        <v>11.33</v>
+      </c>
+      <c r="J32" s="4">
+        <v>0.022736747770421565</v>
+      </c>
+      <c r="K32" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L32" s="4">
+        <v>-11</v>
+      </c>
+      <c r="M32" s="4">
+        <v>0.12159007870986582</v>
+      </c>
+      <c r="N32" s="4">
+        <v>68.47826086956522</v>
+      </c>
+      <c r="O32" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="P32" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33" s="1">
+        <v>-4.08</v>
+      </c>
+      <c r="C33" s="1">
+        <v>6.521739130434782</v>
+      </c>
+      <c r="D33" s="1">
+        <v>14.372549019607844</v>
+      </c>
+      <c r="E33" s="1">
+        <v>13.14</v>
+      </c>
+      <c r="F33" s="1">
+        <v>0.0948011949387904</v>
+      </c>
+      <c r="G33" s="1">
+        <v>0</v>
+      </c>
+      <c r="H33" s="1">
+        <v>62.13</v>
+      </c>
+      <c r="I33" s="1">
+        <v>-6.76</v>
+      </c>
+      <c r="J33" s="1">
+        <v>0.04208599862763582</v>
+      </c>
+      <c r="K33" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L33" s="1">
+        <v>19</v>
+      </c>
+      <c r="M33" s="1">
+        <v>0.07068790351163234</v>
+      </c>
+      <c r="N33" s="1">
+        <v>49.130434782608695</v>
+      </c>
+      <c r="O33" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="P33" s="1">
+        <v>-0.43</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34" s="1">
+        <v>-0.48</v>
+      </c>
+      <c r="C34" s="1">
+        <v>30.434782608695656</v>
+      </c>
+      <c r="D34" s="1">
+        <v>85.89583333333333</v>
+      </c>
+      <c r="E34" s="1">
+        <v>-1.38</v>
+      </c>
+      <c r="F34" s="1">
+        <v>-0.3115998911395332</v>
+      </c>
+      <c r="G34" s="1">
+        <v>0.87</v>
+      </c>
+      <c r="H34" s="1">
+        <v>53.46</v>
+      </c>
+      <c r="I34" s="1">
+        <v>-33.19</v>
+      </c>
+      <c r="J34" s="1">
+        <v>-0.010947727472033765</v>
+      </c>
+      <c r="K34" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L34" s="1">
+        <v>2</v>
+      </c>
+      <c r="M34" s="1">
+        <v>-0.3147346190250637</v>
+      </c>
+      <c r="N34" s="1">
+        <v>40.65217391304348</v>
+      </c>
+      <c r="O34" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="P34" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35" s="1">
+        <v>3.52</v>
+      </c>
+      <c r="C35" s="1">
+        <v>73.91304347826086</v>
+      </c>
+      <c r="D35" s="1">
+        <v>1.1988636363636365</v>
+      </c>
+      <c r="E35" s="1">
+        <v>0.4</v>
+      </c>
+      <c r="F35" s="1">
+        <v>0.02862922306194351</v>
+      </c>
+      <c r="G35" s="1">
+        <v>0.38</v>
+      </c>
+      <c r="H35" s="1">
+        <v>38.34</v>
+      </c>
+      <c r="I35" s="1">
+        <v>2.56</v>
+      </c>
+      <c r="J35" s="1">
+        <v>0.005678463488259859</v>
+      </c>
+      <c r="K35" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L35" s="1">
+        <v>30</v>
+      </c>
+      <c r="M35" s="1">
+        <v>0.01367898237710552</v>
+      </c>
+      <c r="N35" s="1">
+        <v>45.21739130434782</v>
+      </c>
+      <c r="O35" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="P35" s="1">
+        <v>-0.43</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36" s="4">
+        <v>-0.02</v>
+      </c>
+      <c r="C36" s="4">
+        <v>43.47826086956522</v>
+      </c>
+      <c r="D36" s="4">
+        <v>1215</v>
+      </c>
+      <c r="E36" s="4">
+        <v>5.89</v>
+      </c>
+      <c r="F36" s="4">
+        <v>-0.036259160275768546</v>
+      </c>
+      <c r="G36" s="4">
+        <v>1.41</v>
+      </c>
+      <c r="H36" s="4">
+        <v>57.49</v>
+      </c>
+      <c r="I36" s="4">
+        <v>-9.02</v>
+      </c>
+      <c r="J36" s="4">
+        <v>0.018969747496321538</v>
+      </c>
+      <c r="K36" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L36" s="4">
+        <v>29</v>
+      </c>
+      <c r="M36" s="4">
+        <v>-0.026372710790633747</v>
+      </c>
+      <c r="N36" s="4">
+        <v>63.04347826086957</v>
+      </c>
+      <c r="O36" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="P36" s="4">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A37" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37" s="4">
+        <v>0.94</v>
+      </c>
+      <c r="C37" s="4">
+        <v>56.52173913043478</v>
+      </c>
+      <c r="D37" s="4">
+        <v>31.03191489361702</v>
+      </c>
+      <c r="E37" s="4">
+        <v>-0.72</v>
+      </c>
+      <c r="F37" s="4">
+        <v>-0.12542455724540152</v>
+      </c>
+      <c r="G37" s="4">
+        <v>2.78</v>
+      </c>
+      <c r="H37" s="4">
+        <v>60.11</v>
+      </c>
+      <c r="I37" s="4">
+        <v>-6.63</v>
+      </c>
+      <c r="J37" s="4">
+        <v>0.01351706395763758</v>
+      </c>
+      <c r="K37" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L37" s="4">
+        <v>118</v>
+      </c>
+      <c r="M37" s="4">
+        <v>-0.08250289850506021</v>
+      </c>
+      <c r="N37" s="4">
+        <v>59.1304347826087</v>
+      </c>
+      <c r="O37" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="P37" s="4">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A38" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B38" s="4">
+        <v>7.17</v>
+      </c>
+      <c r="C38" s="4">
+        <v>89.13043478260869</v>
+      </c>
+      <c r="D38" s="4">
+        <v>2.0557880055788007</v>
+      </c>
+      <c r="E38" s="4">
+        <v>0.78</v>
+      </c>
+      <c r="F38" s="4">
+        <v>0.052951277478668554</v>
+      </c>
+      <c r="G38" s="4">
+        <v>1.42</v>
+      </c>
+      <c r="H38" s="4">
+        <v>76.19</v>
+      </c>
+      <c r="I38" s="4">
+        <v>12.39</v>
+      </c>
+      <c r="J38" s="4">
+        <v>0.01301767497237266</v>
+      </c>
+      <c r="K38" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L38" s="4">
+        <v>402</v>
+      </c>
+      <c r="M38" s="4">
+        <v>0.06307885987807493</v>
+      </c>
+      <c r="N38" s="4">
+        <v>64.78260869565219</v>
+      </c>
+      <c r="O38" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="P38" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A39" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B39" s="4">
+        <v>-0.38</v>
+      </c>
+      <c r="C39" s="4">
+        <v>34.78260869565217</v>
+      </c>
+      <c r="D39" s="4">
+        <v>882.7368421052631</v>
+      </c>
+      <c r="E39" s="4">
+        <v>0.68</v>
+      </c>
+      <c r="F39" s="4">
+        <v>-0.08623749324450543</v>
+      </c>
+      <c r="G39" s="4">
+        <v>1.51</v>
+      </c>
+      <c r="H39" s="4">
+        <v>60.23</v>
+      </c>
+      <c r="I39" s="4">
+        <v>30.43</v>
+      </c>
+      <c r="J39" s="4">
+        <v>-0.004777022686944814</v>
+      </c>
+      <c r="K39" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L39" s="4">
+        <v>28</v>
+      </c>
+      <c r="M39" s="4">
+        <v>-0.07393971461665483</v>
+      </c>
+      <c r="N39" s="4">
+        <v>57.826086956521735</v>
+      </c>
+      <c r="O39" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="P39" s="4">
+        <v>1.09</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A40" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40" s="4">
+        <v>11.94</v>
+      </c>
+      <c r="C40" s="4">
+        <v>95.65217391304348</v>
+      </c>
+      <c r="D40" s="4">
+        <v>0.9145728643216081</v>
+      </c>
+      <c r="E40" s="4">
+        <v>-1</v>
+      </c>
+      <c r="F40" s="4">
+        <v>0.08153386460991555</v>
+      </c>
+      <c r="G40" s="4">
+        <v>1.71</v>
+      </c>
+      <c r="H40" s="4">
+        <v>68.02</v>
+      </c>
+      <c r="I40" s="4">
+        <v>16.38</v>
+      </c>
+      <c r="J40" s="4">
+        <v>0.008029978850508778</v>
+      </c>
+      <c r="K40" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L40" s="4">
+        <v>19</v>
+      </c>
+      <c r="M40" s="4">
+        <v>0.09865430152319776</v>
+      </c>
+      <c r="N40" s="4">
+        <v>60.434782608695656</v>
+      </c>
+      <c r="O40" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="P40" s="4">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2">
+        <v>3.41</v>
+      </c>
+      <c r="C41" s="2">
+        <v>71.73913043478261</v>
+      </c>
+      <c r="D41" s="2">
+        <v>8.926686217008797</v>
+      </c>
+      <c r="E41" s="2">
+        <v>-1.19</v>
+      </c>
+      <c r="F41" s="2">
+        <v>0.6135308078325732</v>
+      </c>
+      <c r="G41" s="2">
+        <v>2.08</v>
+      </c>
+      <c r="H41" s="2">
+        <v>61.03</v>
+      </c>
+      <c r="I41" s="2">
+        <v>63.89</v>
+      </c>
+      <c r="J41" s="2">
+        <v>0.046290880944706556</v>
+      </c>
+      <c r="K41" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L41" s="2">
+        <v>235</v>
+      </c>
+      <c r="M41" s="2">
+        <v>0.6395731625739038</v>
+      </c>
+      <c r="N41" s="2">
+        <v>71.08695652173913</v>
+      </c>
+      <c r="O41" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="P41" s="2">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2">
+        <v>-0.38</v>
+      </c>
+      <c r="C42" s="2">
+        <v>34.78260869565217</v>
+      </c>
+      <c r="D42" s="2">
+        <v>322.6315789473684</v>
+      </c>
+      <c r="E42" s="2">
+        <v>3.31</v>
+      </c>
+      <c r="F42" s="2">
+        <v>0.43376294328765586</v>
+      </c>
+      <c r="G42" s="2">
+        <v>3.48</v>
+      </c>
+      <c r="H42" s="2">
+        <v>73.97</v>
+      </c>
+      <c r="I42" s="2">
+        <v>117.52</v>
+      </c>
+      <c r="J42" s="2">
+        <v>0.0437033287774922</v>
+      </c>
+      <c r="K42" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L42" s="2">
+        <v>211</v>
+      </c>
+      <c r="M42" s="2">
+        <v>0.49356390602700784</v>
+      </c>
+      <c r="N42" s="2">
+        <v>75.86956521739131</v>
+      </c>
+      <c r="O42" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="P42" s="2">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B43" s="1">
+        <v>-0.32</v>
+      </c>
+      <c r="C43" s="1">
+        <v>36.95652173913043</v>
+      </c>
+      <c r="D43" s="1">
+        <v>228.28125</v>
+      </c>
+      <c r="E43" s="1">
+        <v>3.34</v>
+      </c>
+      <c r="F43" s="1">
+        <v>-0.2024231122362621</v>
+      </c>
+      <c r="G43" s="1">
+        <v>1.68</v>
+      </c>
+      <c r="H43" s="1">
+        <v>44.47</v>
+      </c>
+      <c r="I43" s="1">
+        <v>-5.12</v>
+      </c>
+      <c r="J43" s="1">
+        <v>-0.012928889152724788</v>
+      </c>
+      <c r="K43" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L43" s="1">
+        <v>12</v>
+      </c>
+      <c r="M43" s="1">
+        <v>-0.18602607406579463</v>
+      </c>
+      <c r="N43" s="1">
+        <v>44.565217391304344</v>
+      </c>
+      <c r="O43" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="P43" s="1">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A44" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B44" s="3">
+        <v>-2.92</v>
+      </c>
+      <c r="C44" s="3">
+        <v>15.217391304347828</v>
+      </c>
+      <c r="D44" s="3">
+        <v>-23.77054794520548</v>
+      </c>
+      <c r="E44" s="3">
+        <v>16.88</v>
+      </c>
+      <c r="F44" s="3">
+        <v>0.23124094783320537</v>
+      </c>
+      <c r="G44" s="3">
+        <v>1.95</v>
+      </c>
+      <c r="H44" s="3">
+        <v>73.93</v>
+      </c>
+      <c r="I44" s="3">
+        <v>39.23</v>
+      </c>
+      <c r="J44" s="3">
+        <v>-0.007159582933150655</v>
+      </c>
+      <c r="K44" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L44" s="3">
+        <v>82</v>
+      </c>
+      <c r="M44" s="3">
+        <v>0.25414857468900554</v>
+      </c>
+      <c r="N44" s="3">
+        <v>28.913043478260867</v>
+      </c>
+      <c r="O44" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="P44" s="3">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A45" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B45" s="4">
+        <v>4.88</v>
+      </c>
+      <c r="C45" s="4">
+        <v>76.08695652173914</v>
+      </c>
+      <c r="D45" s="4">
+        <v>6.172131147540984</v>
+      </c>
+      <c r="E45" s="4">
+        <v>-0.19</v>
+      </c>
+      <c r="F45" s="4">
+        <v>0.09983578644763577</v>
+      </c>
+      <c r="G45" s="4">
+        <v>1.84</v>
+      </c>
+      <c r="H45" s="4">
+        <v>61.19</v>
+      </c>
+      <c r="I45" s="4">
+        <v>56.66</v>
+      </c>
+      <c r="J45" s="4">
+        <v>0.017431917254956325</v>
+      </c>
+      <c r="K45" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L45" s="4">
+        <v>304</v>
+      </c>
+      <c r="M45" s="4">
+        <v>0.12009095124644853</v>
+      </c>
+      <c r="N45" s="4">
+        <v>64.13043478260869</v>
+      </c>
+      <c r="O45" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="P45" s="4">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A46" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B46" s="1">
+        <v>-0.76</v>
+      </c>
+      <c r="C46" s="1">
+        <v>26.08695652173913</v>
+      </c>
+      <c r="D46" s="1">
+        <v>13.236842105263158</v>
+      </c>
+      <c r="E46" s="1">
+        <v>7.72</v>
+      </c>
+      <c r="F46" s="1">
+        <v>-0.4293418207008787</v>
+      </c>
+      <c r="G46" s="1">
+        <v>2.61</v>
+      </c>
+      <c r="H46" s="1">
+        <v>55.73</v>
+      </c>
+      <c r="I46" s="1">
+        <v>-31.83</v>
+      </c>
+      <c r="J46" s="1">
+        <v>-0.020809676287581447</v>
+      </c>
+      <c r="K46" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L46" s="1">
+        <v>65</v>
+      </c>
+      <c r="M46" s="1">
+        <v>-0.3905194215031542</v>
+      </c>
+      <c r="N46" s="1">
+        <v>31.30434782608696</v>
+      </c>
+      <c r="O46" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="P46" s="1">
+        <v>-0.43</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A47" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B47" s="4">
+        <v>0.54</v>
+      </c>
+      <c r="C47" s="4">
+        <v>52.17391304347826</v>
+      </c>
+      <c r="D47" s="4">
+        <v>41.629629629629626</v>
+      </c>
+      <c r="E47" s="4">
+        <v>0</v>
+      </c>
+      <c r="F47" s="4">
+        <v>-0.07729216133870549</v>
+      </c>
+      <c r="G47" s="4">
+        <v>1.43</v>
+      </c>
+      <c r="H47" s="4">
+        <v>62.92</v>
+      </c>
+      <c r="I47" s="4">
+        <v>-4.06</v>
+      </c>
+      <c r="J47" s="4">
+        <v>-0.0012099495887365832</v>
+      </c>
+      <c r="K47" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L47" s="4">
+        <v>47</v>
+      </c>
+      <c r="M47" s="4">
+        <v>-0.06692344602502753</v>
+      </c>
+      <c r="N47" s="4">
+        <v>57.17391304347826</v>
+      </c>
+      <c r="O47" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="P47" s="4">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -903,15 +3405,383 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>61</v>
+        <v>87</v>
       </c>
       <c r="B1" t="s">
-        <v>62</v>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>45.652173913043484</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>77.3913043478261</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>25.217391304347828</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>51.73913043478261</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>46.95652173913043</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>61.95652173913042</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>65.8695652173913</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>55.65217391304348</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>48.47826086956522</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>25.434782608695652</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>41.52173913043479</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>76.73913043478261</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>51.95652173913044</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>33.69565217391305</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>62.82608695652174</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>51.08695652173914</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18">
+        <v>54.34782608695652</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19">
+        <v>44.1304347826087</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <v>26.739130434782606</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22">
+        <v>45.869565217391305</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23">
+        <v>22.391304347826086</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24">
+        <v>22.60869565217391</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25">
+        <v>51.52173913043478</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26">
+        <v>66.73913043478261</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27">
+        <v>76.08695652173913</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28">
+        <v>46.95652173913044</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29">
+        <v>49.99999999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <v>56.08695652173913</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31">
+        <v>53.26086956521739</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32">
+        <v>68.47826086956522</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <v>49.130434782608695</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <v>40.65217391304348</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>45.21739130434782</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <v>63.04347826086957</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37">
+        <v>59.1304347826087</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <v>64.78260869565219</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>38</v>
+      </c>
+      <c r="B39">
+        <v>57.826086956521735</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <v>60.434782608695656</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <v>71.08695652173913</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>41</v>
+      </c>
+      <c r="B42">
+        <v>75.86956521739131</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>42</v>
+      </c>
+      <c r="B43">
+        <v>44.565217391304344</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>43</v>
+      </c>
+      <c r="B44">
+        <v>28.913043478260867</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>44</v>
+      </c>
+      <c r="B45">
+        <v>64.13043478260869</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>45</v>
+      </c>
+      <c r="B46">
+        <v>31.30434782608696</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>46</v>
+      </c>
+      <c r="B47">
+        <v>57.17391304347826</v>
       </c>
     </row>
   </sheetData>
@@ -982,4 +3852,239 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C3" t="s">
+        <v>96</v>
+      </c>
+      <c r="D3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C4" t="s">
+        <v>99</v>
+      </c>
+      <c r="D4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5" t="s">
+        <v>103</v>
+      </c>
+      <c r="D5" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6" t="s">
+        <v>105</v>
+      </c>
+      <c r="D6" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>106</v>
+      </c>
+      <c r="B7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" t="s">
+        <v>106</v>
+      </c>
+      <c r="D7" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>107</v>
+      </c>
+      <c r="B8" t="s">
+        <v>108</v>
+      </c>
+      <c r="C8" t="s">
+        <v>106</v>
+      </c>
+      <c r="D8" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>106</v>
+      </c>
+      <c r="B9" t="s">
+        <v>106</v>
+      </c>
+      <c r="C9" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>109</v>
+      </c>
+      <c r="B10" t="s">
+        <v>110</v>
+      </c>
+      <c r="C10" t="s">
+        <v>106</v>
+      </c>
+      <c r="D10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>106</v>
+      </c>
+      <c r="B15" t="s">
+        <v>106</v>
+      </c>
+      <c r="C15" t="s">
+        <v>106</v>
+      </c>
+      <c r="D15" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>119</v>
+      </c>
+      <c r="B16" t="s">
+        <v>120</v>
+      </c>
+      <c r="C16" t="s">
+        <v>106</v>
+      </c>
+      <c r="D16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update report generation to include build ID and timestamp in report.html and visualizer.js
</commit_message>
<xml_diff>
--- a/data/stocks.xlsx
+++ b/data/stocks.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="173">
   <si>
     <t>Ticker</t>
   </si>
@@ -283,6 +283,162 @@
   </si>
   <si>
     <t>_date_</t>
+  </si>
+  <si>
+    <t>Criteria</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>WSR</t>
+  </si>
+  <si>
+    <t>Last Run</t>
+  </si>
+  <si>
+    <t>BLX</t>
+  </si>
+  <si>
+    <t>Index</t>
+  </si>
+  <si>
+    <t>Russell 2000</t>
+  </si>
+  <si>
+    <t>OFG</t>
+  </si>
+  <si>
+    <t>Cap</t>
+  </si>
+  <si>
+    <t>Small ($300M–$2B)</t>
+  </si>
+  <si>
+    <t>Price min</t>
+  </si>
+  <si>
+    <t>&gt; $7</t>
+  </si>
+  <si>
+    <t>YTD perf min</t>
+  </si>
+  <si>
+    <t>&gt; +10%</t>
+  </si>
+  <si>
+    <t>P/E max</t>
+  </si>
+  <si>
+    <t>&lt; 28</t>
+  </si>
+  <si>
+    <t>EPS Q/Q</t>
+  </si>
+  <si>
+    <t>Positive</t>
+  </si>
+  <si>
+    <t>Sectors</t>
+  </si>
+  <si>
+    <t>Technology, Consumer Staples, Materials, Real Estate, Financials, Industrials, Consumer Discretionary</t>
+  </si>
+  <si>
+    <t>Beta range</t>
+  </si>
+  <si>
+    <t>0.7 – 1.2</t>
+  </si>
+  <si>
+    <t>RSI min</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>Alpha</t>
+  </si>
+  <si>
+    <t>&gt; 0</t>
+  </si>
+  <si>
+    <t>Ranked by</t>
+  </si>
+  <si>
+    <t>Alpha (highest first)</t>
+  </si>
+  <si>
+    <t>Top N</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>Results</t>
+  </si>
+  <si>
+    <t>3 of 3 qualified</t>
+  </si>
+  <si>
+    <t>CSCO</t>
+  </si>
+  <si>
+    <t>JPM</t>
+  </si>
+  <si>
+    <t>Dow Jones 30</t>
+  </si>
+  <si>
+    <t>&gt; $10</t>
+  </si>
+  <si>
+    <t>&gt; +5%</t>
+  </si>
+  <si>
+    <t>&lt; 35</t>
+  </si>
+  <si>
+    <t>All sectors</t>
+  </si>
+  <si>
+    <t>2 of 2 qualified</t>
+  </si>
+  <si>
+    <t>AAPL</t>
+  </si>
+  <si>
+    <t>Nasdaq 100</t>
+  </si>
+  <si>
+    <t>&lt; 50</t>
+  </si>
+  <si>
+    <t>0.7 – 1.3</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>DELL</t>
+  </si>
+  <si>
+    <t>ETN</t>
+  </si>
+  <si>
+    <t>S&amp;P 500 (large-cap subset)</t>
+  </si>
+  <si>
+    <t>UNP</t>
+  </si>
+  <si>
+    <t>Large (approx. S&amp;P 100)</t>
+  </si>
+  <si>
+    <t>&gt; +8%</t>
+  </si>
+  <si>
+    <t>&lt; 40</t>
   </si>
   <si>
     <t>Component</t>
@@ -3792,12 +3948,139 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="5" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>100</v>
+      </c>
+      <c r="D6" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="7" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D7" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="8" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>104</v>
+      </c>
+      <c r="D8" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="9" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
+        <v>108</v>
+      </c>
+      <c r="D10" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="11" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C11" t="s">
+        <v>110</v>
+      </c>
+      <c r="D11" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="12" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
+        <v>112</v>
+      </c>
+      <c r="D12" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="13" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C13" t="s">
+        <v>114</v>
+      </c>
+      <c r="D13" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="14" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C14" t="s">
+        <v>116</v>
+      </c>
+      <c r="D14" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="15" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C15" t="s">
+        <v>118</v>
+      </c>
+      <c r="D15" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -3808,12 +4091,128 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D3" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="4" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="5" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>100</v>
+      </c>
+      <c r="D5" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="6" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>102</v>
+      </c>
+      <c r="D6" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="7" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>104</v>
+      </c>
+      <c r="D7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="8" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>106</v>
+      </c>
+      <c r="D8" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="9" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
+        <v>108</v>
+      </c>
+      <c r="D9" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="10" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
+        <v>110</v>
+      </c>
+      <c r="D10" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="11" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C11" t="s">
+        <v>112</v>
+      </c>
+      <c r="D11" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="12" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
+        <v>114</v>
+      </c>
+      <c r="D12" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="13" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C13" t="s">
+        <v>116</v>
+      </c>
+      <c r="D13" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="14" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C14" t="s">
+        <v>118</v>
+      </c>
+      <c r="D14" t="s">
+        <v>127</v>
       </c>
     </row>
   </sheetData>
@@ -3824,12 +4223,128 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D3" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="4" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="5" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>100</v>
+      </c>
+      <c r="D5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="6" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>102</v>
+      </c>
+      <c r="D6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="7" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>104</v>
+      </c>
+      <c r="D7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="8" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>106</v>
+      </c>
+      <c r="D8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
+        <v>108</v>
+      </c>
+      <c r="D9" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="10" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
+        <v>110</v>
+      </c>
+      <c r="D10" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="11" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C11" t="s">
+        <v>112</v>
+      </c>
+      <c r="D11" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="12" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
+        <v>114</v>
+      </c>
+      <c r="D12" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="13" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C13" t="s">
+        <v>116</v>
+      </c>
+      <c r="D13" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="14" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C14" t="s">
+        <v>118</v>
+      </c>
+      <c r="D14" t="s">
+        <v>127</v>
       </c>
     </row>
   </sheetData>
@@ -3840,12 +4355,139 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D3" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D4" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="5" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D5" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="6" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>100</v>
+      </c>
+      <c r="D6" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="7" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D7" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="8" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>104</v>
+      </c>
+      <c r="D8" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="9" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
+        <v>108</v>
+      </c>
+      <c r="D10" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="11" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C11" t="s">
+        <v>110</v>
+      </c>
+      <c r="D11" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="12" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
+        <v>112</v>
+      </c>
+      <c r="D12" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="13" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C13" t="s">
+        <v>114</v>
+      </c>
+      <c r="D13" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="14" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C14" t="s">
+        <v>116</v>
+      </c>
+      <c r="D14" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="15" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C15" t="s">
+        <v>118</v>
+      </c>
+      <c r="D15" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -3861,16 +4503,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>88</v>
+        <v>140</v>
       </c>
       <c r="B1" t="s">
-        <v>89</v>
+        <v>141</v>
       </c>
       <c r="C1" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="D1" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -3878,209 +4520,209 @@
         <v>48</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="C2" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="D2" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>95</v>
+        <v>147</v>
       </c>
       <c r="B3" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
       <c r="C3" t="s">
-        <v>96</v>
+        <v>148</v>
       </c>
       <c r="D3" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>97</v>
+        <v>149</v>
       </c>
       <c r="B4" t="s">
-        <v>98</v>
+        <v>150</v>
       </c>
       <c r="C4" t="s">
-        <v>99</v>
+        <v>151</v>
       </c>
       <c r="D4" t="s">
-        <v>100</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>101</v>
+        <v>153</v>
       </c>
       <c r="B5" t="s">
-        <v>102</v>
+        <v>154</v>
       </c>
       <c r="C5" t="s">
-        <v>103</v>
+        <v>155</v>
       </c>
       <c r="D5" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>104</v>
+        <v>156</v>
       </c>
       <c r="B6" t="s">
-        <v>102</v>
+        <v>154</v>
       </c>
       <c r="C6" t="s">
-        <v>105</v>
+        <v>157</v>
       </c>
       <c r="D6" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
       <c r="B7" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
       <c r="C7" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
       <c r="D7" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>107</v>
+        <v>159</v>
       </c>
       <c r="B8" t="s">
-        <v>108</v>
+        <v>160</v>
       </c>
       <c r="C8" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
       <c r="D8" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
       <c r="B9" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
       <c r="C9" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
       <c r="D9" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>109</v>
+        <v>161</v>
       </c>
       <c r="B10" t="s">
-        <v>110</v>
+        <v>162</v>
       </c>
       <c r="C10" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
       <c r="D10" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>111</v>
+        <v>163</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>112</v>
+        <v>164</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>113</v>
+        <v>165</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>114</v>
+        <v>166</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>115</v>
+        <v>167</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>116</v>
+        <v>168</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>117</v>
+        <v>169</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>118</v>
+        <v>170</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
       <c r="B15" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
       <c r="C15" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
       <c r="D15" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>119</v>
+        <v>171</v>
       </c>
       <c r="B16" t="s">
-        <v>120</v>
+        <v>172</v>
       </c>
       <c r="C16" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
       <c r="D16" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update README.md to clarify clean-workbook script usage and enhance analytics engine description
</commit_message>
<xml_diff>
--- a/data/stocks.xlsx
+++ b/data/stocks.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="118">
   <si>
     <t>Ticker</t>
   </si>
@@ -282,6 +282,96 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>Criteria</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Last Run</t>
+  </si>
+  <si>
+    <t>2026-05-13</t>
+  </si>
+  <si>
+    <t>GOOG</t>
+  </si>
+  <si>
+    <t>Index</t>
+  </si>
+  <si>
+    <t>Nasdaq 100</t>
+  </si>
+  <si>
+    <t>CSCO</t>
+  </si>
+  <si>
+    <t>Price min</t>
+  </si>
+  <si>
+    <t>&gt; $10</t>
+  </si>
+  <si>
+    <t>YTD perf min</t>
+  </si>
+  <si>
+    <t>&gt; +10%</t>
+  </si>
+  <si>
+    <t>P/E max</t>
+  </si>
+  <si>
+    <t>&lt; 50</t>
+  </si>
+  <si>
+    <t>EPS Q/Q</t>
+  </si>
+  <si>
+    <t>Positive</t>
+  </si>
+  <si>
+    <t>Sectors</t>
+  </si>
+  <si>
+    <t>Technology, Consumer Staples, Materials, Real Estate, Financials, Industrials, Consumer Discretionary</t>
+  </si>
+  <si>
+    <t>Beta range</t>
+  </si>
+  <si>
+    <t>0.7 – 1.3</t>
+  </si>
+  <si>
+    <t>RSI min</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>Alpha</t>
+  </si>
+  <si>
+    <t>&gt; 0</t>
+  </si>
+  <si>
+    <t>Ranked by</t>
+  </si>
+  <si>
+    <t>Alpha (highest first)</t>
+  </si>
+  <si>
+    <t>Top N</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>Results</t>
+  </si>
+  <si>
+    <t>3 of 3 qualified</t>
   </si>
 </sst>
 </file>
@@ -898,7 +988,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1039,7 +1129,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1097,7 +1187,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1116,7 +1206,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1132,7 +1222,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1148,23 +1238,142 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
+      <c r="C1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="5" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>100</v>
+      </c>
+      <c r="D6" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="7" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D7" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="8" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>104</v>
+      </c>
+      <c r="D8" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="9" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
+        <v>108</v>
+      </c>
+      <c r="D10" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="11" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C11" t="s">
+        <v>110</v>
+      </c>
+      <c r="D11" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="12" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
+        <v>112</v>
+      </c>
+      <c r="D12" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="13" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C13" t="s">
+        <v>114</v>
+      </c>
+      <c r="D13" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="14" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C14" t="s">
+        <v>116</v>
+      </c>
+      <c r="D14" t="s">
+        <v>117</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1180,6 +1389,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
checkpoint: complete firebase auth pipeline (custom token → id token → middleware rbac)
</commit_message>
<xml_diff>
--- a/data/stocks.xlsx
+++ b/data/stocks.xlsx
@@ -337,7 +337,7 @@
     <t>2026-05-11</t>
   </si>
   <si>
-    <t>2026-04-30</t>
+    <t>2027-04-30</t>
   </si>
   <si>
     <t>2027-04-29</t>
@@ -1689,7 +1689,7 @@
         <v>43.291139240506325</v>
       </c>
       <c r="C30" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -1914,13 +1914,13 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>15</v>
+        <v>68</v>
       </c>
       <c r="B51">
-        <v>29.367088607594937</v>
+        <v>32.0253164556962</v>
       </c>
       <c r="C51" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
     </row>
   </sheetData>
@@ -4091,7 +4091,7 @@
         <v>0.006795185819069533</v>
       </c>
       <c r="K33" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L33" s="3">
         <v>5</v>
@@ -6323,7 +6323,7 @@
         <v>-0.0006359513945416026</v>
       </c>
       <c r="K69" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L69" s="3">
         <v>-60</v>

</xml_diff>

<commit_message>
WIP: checkpoint analytics pipeline & screenIndex changes
</commit_message>
<xml_diff>
--- a/data/stocks.xlsx
+++ b/data/stocks.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="234">
   <si>
     <t>Ticker</t>
   </si>
@@ -418,15 +418,24 @@
     <t>Value</t>
   </si>
   <si>
+    <t>RAPP</t>
+  </si>
+  <si>
     <t>Last Run</t>
   </si>
   <si>
+    <t>2026-05-31</t>
+  </si>
+  <si>
     <t>Index</t>
   </si>
   <si>
     <t>Russell 2000</t>
   </si>
   <si>
+    <t>OFG</t>
+  </si>
+  <si>
     <t>Cap</t>
   </si>
   <si>
@@ -496,7 +505,7 @@
     <t>Results</t>
   </si>
   <si>
-    <t>5 of 5 qualified</t>
+    <t>3 of 3 qualified</t>
   </si>
   <si>
     <t>Dow Jones 30</t>
@@ -514,37 +523,37 @@
     <t>All sectors</t>
   </si>
   <si>
+    <t>1 of 1 qualified</t>
+  </si>
+  <si>
+    <t>AAPL</t>
+  </si>
+  <si>
+    <t>Nasdaq 100</t>
+  </si>
+  <si>
+    <t>&lt; 50</t>
+  </si>
+  <si>
+    <t>0.7 – 1.3</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>S&amp;P 500 (large-cap subset)</t>
+  </si>
+  <si>
+    <t>Large (approx. S&amp;P 100)</t>
+  </si>
+  <si>
+    <t>&gt; +8%</t>
+  </si>
+  <si>
+    <t>&lt; 40</t>
+  </si>
+  <si>
     <t>0 of 0 qualified</t>
-  </si>
-  <si>
-    <t>Nasdaq 100</t>
-  </si>
-  <si>
-    <t>&lt; 50</t>
-  </si>
-  <si>
-    <t>0.7 – 1.3</t>
-  </si>
-  <si>
-    <t>60</t>
-  </si>
-  <si>
-    <t>3 of 3 qualified</t>
-  </si>
-  <si>
-    <t>S&amp;P 500 (large-cap subset)</t>
-  </si>
-  <si>
-    <t>Large (approx. S&amp;P 100)</t>
-  </si>
-  <si>
-    <t>&gt; +8%</t>
-  </si>
-  <si>
-    <t>&lt; 40</t>
-  </si>
-  <si>
-    <t>1 of 1 qualified</t>
   </si>
   <si>
     <t>Component</t>
@@ -1367,10 +1376,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="C1" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -1381,7 +1390,7 @@
         <v>72.08860759493672</v>
       </c>
       <c r="C2" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1392,7 +1401,7 @@
         <v>67.40506329113924</v>
       </c>
       <c r="C3" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1403,7 +1412,7 @@
         <v>67.34177215189875</v>
       </c>
       <c r="C4" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1414,7 +1423,7 @@
         <v>66.45569620253164</v>
       </c>
       <c r="C5" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1425,7 +1434,7 @@
         <v>65.37974683544304</v>
       </c>
       <c r="C6" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1436,7 +1445,7 @@
         <v>61.329113924050645</v>
       </c>
       <c r="C7" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1447,7 +1456,7 @@
         <v>61.13924050632911</v>
       </c>
       <c r="C8" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -1458,7 +1467,7 @@
         <v>60.8860759493671</v>
       </c>
       <c r="C9" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -1469,7 +1478,7 @@
         <v>60.88607594936709</v>
       </c>
       <c r="C10" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -1480,7 +1489,7 @@
         <v>58.41772151898735</v>
       </c>
       <c r="C11" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -1491,7 +1500,7 @@
         <v>57.59493670886076</v>
       </c>
       <c r="C12" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -1502,7 +1511,7 @@
         <v>55.949367088607595</v>
       </c>
       <c r="C13" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -1513,7 +1522,7 @@
         <v>55.8860759493671</v>
       </c>
       <c r="C14" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -1524,7 +1533,7 @@
         <v>55.822784810126585</v>
       </c>
       <c r="C15" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -1535,7 +1544,7 @@
         <v>55.063291139240505</v>
       </c>
       <c r="C16" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -1546,7 +1555,7 @@
         <v>55.063291139240505</v>
       </c>
       <c r="C17" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -1557,7 +1566,7 @@
         <v>53.98734177215191</v>
       </c>
       <c r="C18" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -1568,7 +1577,7 @@
         <v>53.9873417721519</v>
       </c>
       <c r="C19" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -1579,7 +1588,7 @@
         <v>53.164556962025316</v>
       </c>
       <c r="C20" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -1590,7 +1599,7 @@
         <v>52.65822784810126</v>
       </c>
       <c r="C21" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -1601,7 +1610,7 @@
         <v>52.40506329113924</v>
       </c>
       <c r="C22" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -1612,7 +1621,7 @@
         <v>51.139240506329116</v>
       </c>
       <c r="C23" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -1623,7 +1632,7 @@
         <v>48.79746835443037</v>
       </c>
       <c r="C24" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -1634,7 +1643,7 @@
         <v>47.21518987341773</v>
       </c>
       <c r="C25" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -1645,7 +1654,7 @@
         <v>46.835443037974684</v>
       </c>
       <c r="C26" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -1656,7 +1665,7 @@
         <v>46.835443037974684</v>
       </c>
       <c r="C27" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -1667,7 +1676,7 @@
         <v>46.39240506329114</v>
       </c>
       <c r="C28" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -1678,7 +1687,7 @@
         <v>46.265822784810126</v>
       </c>
       <c r="C29" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -1689,7 +1698,7 @@
         <v>43.291139240506325</v>
       </c>
       <c r="C30" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -1700,7 +1709,7 @@
         <v>43.164556962025316</v>
       </c>
       <c r="C31" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -1711,7 +1720,7 @@
         <v>42.53164556962026</v>
       </c>
       <c r="C32" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -1722,7 +1731,7 @@
         <v>42.53164556962026</v>
       </c>
       <c r="C33" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -1733,7 +1742,7 @@
         <v>42.08860759493671</v>
       </c>
       <c r="C34" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -1744,7 +1753,7 @@
         <v>41.89873417721519</v>
       </c>
       <c r="C35" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -1755,7 +1764,7 @@
         <v>41.64556962025317</v>
       </c>
       <c r="C36" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -1766,7 +1775,7 @@
         <v>41.265822784810126</v>
       </c>
       <c r="C37" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -1777,7 +1786,7 @@
         <v>40.632911392405056</v>
       </c>
       <c r="C38" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -1788,7 +1797,7 @@
         <v>39.43037974683544</v>
       </c>
       <c r="C39" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -1799,7 +1808,7 @@
         <v>37.848101265822784</v>
       </c>
       <c r="C40" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -1810,7 +1819,7 @@
         <v>37.215189873417714</v>
       </c>
       <c r="C41" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -1821,7 +1830,7 @@
         <v>36.075949367088604</v>
       </c>
       <c r="C42" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -1832,7 +1841,7 @@
         <v>35.69620253164557</v>
       </c>
       <c r="C43" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -1843,7 +1852,7 @@
         <v>35</v>
       </c>
       <c r="C44" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -1854,7 +1863,7 @@
         <v>34.49367088607595</v>
       </c>
       <c r="C45" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
@@ -1865,7 +1874,7 @@
         <v>33.79746835443038</v>
       </c>
       <c r="C46" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -1876,7 +1885,7 @@
         <v>33.164556962025316</v>
       </c>
       <c r="C47" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -1887,7 +1896,7 @@
         <v>33.10126582278481</v>
       </c>
       <c r="C48" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -1898,7 +1907,7 @@
         <v>33.10126582278481</v>
       </c>
       <c r="C49" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -1909,7 +1918,7 @@
         <v>32.53164556962025</v>
       </c>
       <c r="C50" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -1920,7 +1929,7 @@
         <v>32.0253164556962</v>
       </c>
       <c r="C51" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
   </sheetData>
@@ -7710,13 +7719,13 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="C2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D2" t="s">
-        <v>111</v>
+        <v>134</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -7724,21 +7733,21 @@
         <v>120</v>
       </c>
       <c r="C3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>122</v>
+        <v>137</v>
       </c>
       <c r="C4" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="D4" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -7746,10 +7755,10 @@
         <v>123</v>
       </c>
       <c r="C5" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D5" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -7757,82 +7766,82 @@
         <v>124</v>
       </c>
       <c r="C6" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D6" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
     </row>
     <row r="7" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D7" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="D8" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="9" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D9" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="D10" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="11" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="D11" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="12" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D12" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="13" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="D13" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="14" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D14" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="15" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="D15" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -7857,108 +7866,111 @@
         <v>131</v>
       </c>
     </row>
-    <row r="2" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
       <c r="C2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D2" t="s">
-        <v>111</v>
+        <v>134</v>
       </c>
     </row>
     <row r="3" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D3" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D4" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D5" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="6" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D6" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
     </row>
     <row r="7" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="D7" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D8" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="9" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="D9" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="10" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="D10" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="11" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D11" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="12" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="D12" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="13" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D13" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="14" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="D14" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -7985,115 +7997,115 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>126</v>
       </c>
       <c r="C2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D2" t="s">
-        <v>111</v>
+        <v>134</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>125</v>
+        <v>168</v>
       </c>
       <c r="C3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D3" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>126</v>
+        <v>32</v>
       </c>
       <c r="C4" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D4" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D5" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D6" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="7" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="D7" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D8" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="9" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="D9" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
     </row>
     <row r="10" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="D10" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
     </row>
     <row r="11" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D11" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="12" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="D12" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="13" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D13" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="14" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="D14" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -8123,114 +8135,114 @@
         <v>127</v>
       </c>
       <c r="C2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D2" t="s">
-        <v>111</v>
+        <v>134</v>
       </c>
     </row>
     <row r="3" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D3" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
     </row>
     <row r="4" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="D4" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D5" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D6" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D7" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
     </row>
     <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="D8" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="9" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D9" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="D10" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="11" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="D11" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="12" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D12" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="13" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="D13" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="14" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D14" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="15" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="D15" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
   </sheetData>
@@ -8246,212 +8258,212 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B1" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="C1" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="D1" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B2" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="D2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>186</v>
+      </c>
+      <c r="B3" t="s">
         <v>183</v>
       </c>
-      <c r="B3" t="s">
-        <v>180</v>
-      </c>
       <c r="C3" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D3" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B4" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C4" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D4" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B5" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="C5" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="D5" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>196</v>
+      </c>
+      <c r="B6" t="s">
         <v>193</v>
       </c>
-      <c r="B6" t="s">
-        <v>190</v>
-      </c>
       <c r="C6" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="D6" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B7" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="C7" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="D7" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B8" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C8" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D8" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="B9" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="C9" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D9" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B10" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C10" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D10" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>205</v>
+      </c>
+      <c r="B11" t="s">
+        <v>206</v>
+      </c>
+      <c r="C11" t="s">
         <v>202</v>
       </c>
-      <c r="B11" t="s">
-        <v>203</v>
-      </c>
-      <c r="C11" t="s">
-        <v>199</v>
-      </c>
       <c r="D11" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B12" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="C12" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D12" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B13" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="C13" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D13" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B14" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="C14" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D14" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="B15" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="C15" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D15" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(screenIndex): update Finviz ticker extraction for current DOM structure
- Select ticker from a.tab-link instead of concatenated anchor text

- Restore Russell screener functionality after Finviz HTML changes

- Preserve existing screening, ranking, and workbook generation behavior
</commit_message>
<xml_diff>
--- a/data/stocks.xlsx
+++ b/data/stocks.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="240">
   <si>
     <t>Ticker</t>
   </si>
@@ -445,130 +445,145 @@
     <t>Last Run</t>
   </si>
   <si>
+    <t>2026-07-24</t>
+  </si>
+  <si>
+    <t>XHR</t>
+  </si>
+  <si>
+    <t>Index</t>
+  </si>
+  <si>
+    <t>Russell 2000</t>
+  </si>
+  <si>
+    <t>LPG</t>
+  </si>
+  <si>
+    <t>Cap</t>
+  </si>
+  <si>
+    <t>Small ($300M–$2B)</t>
+  </si>
+  <si>
+    <t>RAPP</t>
+  </si>
+  <si>
+    <t>Price min</t>
+  </si>
+  <si>
+    <t>&gt; $7</t>
+  </si>
+  <si>
+    <t>YTD perf min</t>
+  </si>
+  <si>
+    <t>&gt; +10%</t>
+  </si>
+  <si>
+    <t>P/E max</t>
+  </si>
+  <si>
+    <t>&lt; 28</t>
+  </si>
+  <si>
+    <t>EPS Q/Q</t>
+  </si>
+  <si>
+    <t>Positive</t>
+  </si>
+  <si>
+    <t>Sectors</t>
+  </si>
+  <si>
+    <t>Technology, Consumer Staples, Materials, Real Estate, Financials, Industrials, Consumer Discretionary</t>
+  </si>
+  <si>
+    <t>Beta range</t>
+  </si>
+  <si>
+    <t>0.7 – 1.2</t>
+  </si>
+  <si>
+    <t>RSI min</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>Alpha</t>
+  </si>
+  <si>
+    <t>&gt; 0</t>
+  </si>
+  <si>
+    <t>Ranked by</t>
+  </si>
+  <si>
+    <t>Alpha (highest first)</t>
+  </si>
+  <si>
+    <t>Top N</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>Results</t>
+  </si>
+  <si>
+    <t>4 of 4 qualified</t>
+  </si>
+  <si>
+    <t>Dow Jones 30</t>
+  </si>
+  <si>
+    <t>&gt; $10</t>
+  </si>
+  <si>
+    <t>&gt; +5%</t>
+  </si>
+  <si>
+    <t>&lt; 35</t>
+  </si>
+  <si>
+    <t>All sectors</t>
+  </si>
+  <si>
+    <t>3 of 3 qualified</t>
+  </si>
+  <si>
+    <t>Nasdaq 100</t>
+  </si>
+  <si>
+    <t>&lt; 50</t>
+  </si>
+  <si>
+    <t>0.7 – 1.3</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>0 of 0 qualified</t>
+  </si>
+  <si>
     <t>2026-07-08</t>
   </si>
   <si>
-    <t>Index</t>
-  </si>
-  <si>
-    <t>Russell 2000</t>
-  </si>
-  <si>
-    <t>Cap</t>
-  </si>
-  <si>
-    <t>Small ($300M–$2B)</t>
-  </si>
-  <si>
-    <t>Price min</t>
-  </si>
-  <si>
-    <t>&gt; $7</t>
-  </si>
-  <si>
-    <t>YTD perf min</t>
-  </si>
-  <si>
-    <t>&gt; +10%</t>
-  </si>
-  <si>
-    <t>P/E max</t>
-  </si>
-  <si>
-    <t>&lt; 28</t>
-  </si>
-  <si>
-    <t>EPS Q/Q</t>
-  </si>
-  <si>
-    <t>Positive</t>
-  </si>
-  <si>
-    <t>Sectors</t>
-  </si>
-  <si>
-    <t>Technology, Consumer Staples, Materials, Real Estate, Financials, Industrials, Consumer Discretionary</t>
-  </si>
-  <si>
-    <t>Beta range</t>
-  </si>
-  <si>
-    <t>0.7 – 1.2</t>
-  </si>
-  <si>
-    <t>RSI min</t>
-  </si>
-  <si>
-    <t>50</t>
-  </si>
-  <si>
-    <t>Alpha</t>
-  </si>
-  <si>
-    <t>&gt; 0</t>
-  </si>
-  <si>
-    <t>Ranked by</t>
-  </si>
-  <si>
-    <t>Alpha (highest first)</t>
-  </si>
-  <si>
-    <t>Top N</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>Results</t>
-  </si>
-  <si>
-    <t>5 of 5 qualified</t>
-  </si>
-  <si>
-    <t>Dow Jones 30</t>
-  </si>
-  <si>
-    <t>&gt; $10</t>
-  </si>
-  <si>
-    <t>&gt; +5%</t>
-  </si>
-  <si>
-    <t>&lt; 35</t>
-  </si>
-  <si>
-    <t>All sectors</t>
-  </si>
-  <si>
-    <t>2 of 2 qualified</t>
-  </si>
-  <si>
-    <t>Nasdaq 100</t>
-  </si>
-  <si>
-    <t>&lt; 50</t>
-  </si>
-  <si>
-    <t>0.7 – 1.3</t>
-  </si>
-  <si>
-    <t>60</t>
+    <t>S&amp;P 500 (large-cap subset)</t>
+  </si>
+  <si>
+    <t>Large (approx. S&amp;P 100)</t>
+  </si>
+  <si>
+    <t>&gt; +8%</t>
+  </si>
+  <si>
+    <t>&lt; 40</t>
   </si>
   <si>
     <t>1 of 1 qualified</t>
-  </si>
-  <si>
-    <t>S&amp;P 500 (large-cap subset)</t>
-  </si>
-  <si>
-    <t>Large (approx. S&amp;P 100)</t>
-  </si>
-  <si>
-    <t>&gt; +8%</t>
-  </si>
-  <si>
-    <t>&lt; 40</t>
   </si>
   <si>
     <t>Component</t>
@@ -1394,10 +1409,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="C1" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -1408,7 +1423,7 @@
         <v>73.71951219512195</v>
       </c>
       <c r="C2" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1419,7 +1434,7 @@
         <v>69.39024390243902</v>
       </c>
       <c r="C3" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1430,7 +1445,7 @@
         <v>68.10975609756098</v>
       </c>
       <c r="C4" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1441,7 +1456,7 @@
         <v>67.07317073170731</v>
       </c>
       <c r="C5" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1452,7 +1467,7 @@
         <v>66.03658536585365</v>
       </c>
       <c r="C6" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1463,7 +1478,7 @@
         <v>64.08536585365853</v>
       </c>
       <c r="C7" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1474,7 +1489,7 @@
         <v>59.99999999999999</v>
       </c>
       <c r="C8" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -1485,7 +1500,7 @@
         <v>59.756097560975604</v>
       </c>
       <c r="C9" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -1496,7 +1511,7 @@
         <v>59.20731707317073</v>
       </c>
       <c r="C10" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -1507,7 +1522,7 @@
         <v>58.59756097560976</v>
       </c>
       <c r="C11" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -1518,7 +1533,7 @@
         <v>58.59756097560976</v>
       </c>
       <c r="C12" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -1529,7 +1544,7 @@
         <v>58.41463414634147</v>
       </c>
       <c r="C13" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -1540,7 +1555,7 @@
         <v>56.646341463414636</v>
       </c>
       <c r="C14" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -1551,7 +1566,7 @@
         <v>55.914634146341456</v>
       </c>
       <c r="C15" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -1562,7 +1577,7 @@
         <v>53.109756097560975</v>
       </c>
       <c r="C16" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -1573,7 +1588,7 @@
         <v>52.74390243902439</v>
       </c>
       <c r="C17" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -1584,7 +1599,7 @@
         <v>52.378048780487816</v>
       </c>
       <c r="C18" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -1595,7 +1610,7 @@
         <v>52.13414634146342</v>
       </c>
       <c r="C19" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -1606,7 +1621,7 @@
         <v>51.64634146341464</v>
       </c>
       <c r="C20" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -1617,7 +1632,7 @@
         <v>51.21951219512196</v>
       </c>
       <c r="C21" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -1628,7 +1643,7 @@
         <v>49.268292682926834</v>
       </c>
       <c r="C22" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -1639,7 +1654,7 @@
         <v>48.963414634146346</v>
       </c>
       <c r="C23" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -1650,7 +1665,7 @@
         <v>48.59756097560976</v>
       </c>
       <c r="C24" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -1661,7 +1676,7 @@
         <v>48.47560975609756</v>
       </c>
       <c r="C25" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -1672,7 +1687,7 @@
         <v>48.41463414634147</v>
       </c>
       <c r="C26" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -1683,7 +1698,7 @@
         <v>48.41463414634146</v>
       </c>
       <c r="C27" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -1694,7 +1709,7 @@
         <v>48.35365853658537</v>
       </c>
       <c r="C28" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -1705,7 +1720,7 @@
         <v>48.17073170731707</v>
       </c>
       <c r="C29" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -1716,7 +1731,7 @@
         <v>48.048780487804876</v>
       </c>
       <c r="C30" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -1727,7 +1742,7 @@
         <v>48.048780487804876</v>
       </c>
       <c r="C31" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -1738,7 +1753,7 @@
         <v>47.19512195121951</v>
       </c>
       <c r="C32" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -1749,7 +1764,7 @@
         <v>46.82926829268293</v>
       </c>
       <c r="C33" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -1760,7 +1775,7 @@
         <v>46.768292682926834</v>
       </c>
       <c r="C34" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -1771,7 +1786,7 @@
         <v>46.76829268292683</v>
       </c>
       <c r="C35" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -1782,7 +1797,7 @@
         <v>46.40243902439024</v>
       </c>
       <c r="C36" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -1793,7 +1808,7 @@
         <v>45.975609756097555</v>
       </c>
       <c r="C37" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -1804,7 +1819,7 @@
         <v>45.30487804878049</v>
       </c>
       <c r="C38" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -1815,7 +1830,7 @@
         <v>44.756097560975604</v>
       </c>
       <c r="C39" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -1826,7 +1841,7 @@
         <v>44.329268292682926</v>
       </c>
       <c r="C40" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -1837,7 +1852,7 @@
         <v>43.59756097560975</v>
       </c>
       <c r="C41" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -1848,7 +1863,7 @@
         <v>43.23170731707317</v>
       </c>
       <c r="C42" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -1859,7 +1874,7 @@
         <v>36.64634146341464</v>
       </c>
       <c r="C43" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -1870,7 +1885,7 @@
         <v>35.853658536585364</v>
       </c>
       <c r="C44" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -1881,7 +1896,7 @@
         <v>35.79268292682927</v>
       </c>
       <c r="C45" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
@@ -1892,7 +1907,7 @@
         <v>35.792682926829265</v>
       </c>
       <c r="C46" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -1903,7 +1918,7 @@
         <v>35.487804878048784</v>
       </c>
       <c r="C47" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -1914,7 +1929,7 @@
         <v>34.26829268292683</v>
       </c>
       <c r="C48" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -1925,7 +1940,7 @@
         <v>33.170731707317074</v>
       </c>
       <c r="C49" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -1936,7 +1951,7 @@
         <v>32.01219512195122</v>
       </c>
       <c r="C50" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -1947,7 +1962,7 @@
         <v>31.890243902439025</v>
       </c>
       <c r="C51" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
     </row>
   </sheetData>
@@ -7958,35 +7973,35 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>126</v>
+        <v>142</v>
       </c>
       <c r="C3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>127</v>
+        <v>145</v>
       </c>
       <c r="C4" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D4" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>128</v>
+        <v>148</v>
       </c>
       <c r="C5" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="D5" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -7994,82 +8009,82 @@
         <v>129</v>
       </c>
       <c r="C6" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D6" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="7" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="D7" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="D8" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="9" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="D9" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
     </row>
     <row r="10" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D10" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="11" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D11" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="12" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="D12" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="13" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="D13" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="14" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="D14" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
     </row>
     <row r="15" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D15" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -8096,7 +8111,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>130</v>
+        <v>49</v>
       </c>
       <c r="C2" t="s">
         <v>140</v>
@@ -8107,101 +8122,104 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>131</v>
       </c>
-      <c r="C3" t="s">
-        <v>142</v>
-      </c>
-      <c r="D3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="4" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="D4" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="5" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D5" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
     </row>
     <row r="6" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="D6" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="7" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="D7" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="D8" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D9" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D10" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="11" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="D11" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="12" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="D12" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="13" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="D13" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
     </row>
     <row r="14" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D14" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -8242,10 +8260,10 @@
         <v>133</v>
       </c>
       <c r="C3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D3" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -8253,90 +8271,90 @@
         <v>134</v>
       </c>
       <c r="C4" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="D4" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="5" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D5" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="6" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="D6" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="7" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="D7" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="D8" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D9" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
     </row>
     <row r="10" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D10" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="11" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="D11" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="12" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="D12" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="13" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="D13" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
     </row>
     <row r="14" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D14" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -8369,111 +8387,111 @@
         <v>140</v>
       </c>
       <c r="D2" t="s">
-        <v>141</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D3" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
     </row>
     <row r="4" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D4" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
     </row>
     <row r="5" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="D5" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="6" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D6" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
     </row>
     <row r="7" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="D7" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
     </row>
     <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="D8" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="9" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="D9" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
     </row>
     <row r="10" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D10" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="11" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D11" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="12" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="D12" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="13" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="D13" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="14" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="D14" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
     </row>
     <row r="15" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D15" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -8489,212 +8507,212 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="B1" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="C1" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="D1" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="B2" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="C2" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="D2" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="B3" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="C3" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="D3" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="B4" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="C4" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="D4" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="B5" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="C5" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="D5" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="B6" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="C6" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="D6" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="B7" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="C7" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="D7" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="B8" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="C8" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="D8" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="B9" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C9" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="D9" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="B10" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="C10" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="D10" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="B11" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="C11" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="D11" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>217</v>
+      </c>
+      <c r="B12" t="s">
+        <v>218</v>
+      </c>
+      <c r="C12" t="s">
         <v>212</v>
       </c>
-      <c r="B12" t="s">
-        <v>213</v>
-      </c>
-      <c r="C12" t="s">
-        <v>207</v>
-      </c>
       <c r="D12" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="B13" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="C13" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="D13" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="B14" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="C14" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="D14" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="B15" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="C15" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="D15" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>

</xml_diff>